<commit_message>
docs(backlog): update Backlog Scrum Excel with Sprint 07 completion, TEMIS Media Studio milestone, and Sprint 08 UAT
</commit_message>
<xml_diff>
--- a/Temis/Backlog_Scrum_area_tecnica_TEMIS.xlsx
+++ b/Temis/Backlog_Scrum_area_tecnica_TEMIS.xlsx
@@ -98,7 +98,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -159,8 +159,26 @@
         <bgColor rgb="000F172A"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEF9C3"/>
+        <bgColor rgb="00FEF9C3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EBF5FF"/>
+        <bgColor rgb="00EBF5FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+        <bgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -182,11 +200,25 @@
         <color rgb="00CBD5E1"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00E2E8F0"/>
+      </left>
+      <right style="thin">
+        <color rgb="00E2E8F0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00E2E8F0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00E2E8F0"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -276,6 +308,48 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="13" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="13" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -669,7 +743,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="25" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -918,72 +991,72 @@
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A11" s="31" t="inlineStr">
         <is>
           <t>Sprint 07</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B11" s="31" t="inlineStr">
         <is>
           <t>16 Sep 2026 - 30 Sep 2026</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>Persistencia Híbrida &amp; Exportador Gráfico Alta Resolución</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>Export PNG/PDF / DB</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>Exportador vectorial PNG/PDF 300 DPI y Auto-Guardado PostgreSQL</t>
-        </is>
-      </c>
-      <c r="F11" s="8" t="inlineStr">
+      <c r="C11" s="32" t="inlineStr">
+        <is>
+          <t>🔥 HITO ESTRATÉGICO: Introducción TEMIS Media Studio (Desktop) + Ingesta Web &amp; Plantillas Maestras</t>
+        </is>
+      </c>
+      <c r="D11" s="32" t="inlineStr">
+        <is>
+          <t>Media Studio / Ingesta ZIP / SIPOC / Plantilla Word Oficial</t>
+        </is>
+      </c>
+      <c r="E11" s="32" t="inlineStr">
+        <is>
+          <t>Lanzamiento de TEMIS Media Studio (Whisper + Keyframes HD), Ingesta ZIP, Exportador Excel Oficial y Plantilla Maestra Word SAR 90 días</t>
+        </is>
+      </c>
+      <c r="F11" s="33" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G11" s="31" t="n">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="31" t="inlineStr">
+        <is>
+          <t>Sprint 08</t>
+        </is>
+      </c>
+      <c r="B12" s="31" t="inlineStr">
+        <is>
+          <t>01 Oct 2026 - 31 Oct 2026</t>
+        </is>
+      </c>
+      <c r="C12" s="32" t="inlineStr">
+        <is>
+          <t>Pruebas de Usuario (UAT), Validación con Jefa de Procesos, Adaptaciones de Usabilidad &amp; Auto-Layout</t>
+        </is>
+      </c>
+      <c r="D12" s="32" t="inlineStr">
+        <is>
+          <t>UAT / Swimlanes / Usabilidad / Sincronización Bidireccional</t>
+        </is>
+      </c>
+      <c r="E12" s="32" t="inlineStr">
+        <is>
+          <t>Validación en vivo del pipeline 4 fases (Entrevista-&gt;SIPOC-&gt;Flujo-&gt;Word), pruebas de estrés y refinamiento de carriles swimlanes</t>
+        </is>
+      </c>
+      <c r="F12" s="34" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
       </c>
-      <c r="G11" s="4" t="n">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>Sprint 08</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>01 Oct 2026 - 31 Oct 2026</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>Mapeador Automático de Swimlanes &amp; Multi-Usuario</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>Swimlanes / Colaboración</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>Auto-layout de carriles por rol/sistema y sincronización web</t>
-        </is>
-      </c>
-      <c r="F12" s="9" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="G12" s="4" t="n">
+      <c r="G12" s="31" t="n">
         <v>35</v>
       </c>
     </row>
@@ -1072,7 +1145,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q19"/>
+  <dimension ref="A1:Q26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2287,8 +2360,10 @@
       <c r="K15" s="15" t="n">
         <v>46281</v>
       </c>
-      <c r="L15" s="15" t="n">
-        <v>46295</v>
+      <c r="L15" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-30 00:00:00</t>
+        </is>
       </c>
       <c r="M15" s="4" t="inlineStr">
         <is>
@@ -2297,7 +2372,7 @@
       </c>
       <c r="N15" s="8" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="O15" s="14" t="inlineStr">
@@ -2367,8 +2442,10 @@
       <c r="K16" s="13" t="n">
         <v>46281</v>
       </c>
-      <c r="L16" s="13" t="n">
-        <v>46295</v>
+      <c r="L16" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-30 00:00:00</t>
+        </is>
       </c>
       <c r="M16" s="11" t="inlineStr">
         <is>
@@ -2377,7 +2454,7 @@
       </c>
       <c r="N16" s="8" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="O16" s="12" t="inlineStr">
@@ -2636,6 +2713,587 @@
       <c r="Q19" s="14" t="inlineStr">
         <is>
           <t>Sprint 10 Final Release</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="35" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="B20" s="36" t="inlineStr">
+        <is>
+          <t>🔥 Media Studio Desktop / Whisper &amp; Keyframes</t>
+        </is>
+      </c>
+      <c r="C20" s="36" t="inlineStr">
+        <is>
+          <t>Epic / HITO GRANDE</t>
+        </is>
+      </c>
+      <c r="D20" s="36" t="inlineStr">
+        <is>
+          <t>Como analista de procesos, quiero una suite de escritorio (TEMIS Media Studio) para transcribir grabaciones de entrevistas offline con Whisper y extraer capturas de pantalla HD automáticamente.</t>
+        </is>
+      </c>
+      <c r="E20" s="36" t="inlineStr">
+        <is>
+          <t>1. Implementar motor Whisper local con faster-whisper. 2. Crear extractor inteligente de fotogramas clave por cambio de escena/sistema. 3. Empaquetar proyecto en archivo .zip con manifiesto .temis.json, subtítulos .vtt y capturas/ sin saturar la red.</t>
+        </is>
+      </c>
+      <c r="F20" s="36" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G20" s="36" t="inlineStr">
+        <is>
+          <t>Suite de escritorio offline en Python/FFmpeg para procesamiento multimedia local, transcripción sincronizada y captura de evidencias de alta resolución.</t>
+        </is>
+      </c>
+      <c r="H20" s="35" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I20" s="35" t="n">
+        <v>15</v>
+      </c>
+      <c r="J20" s="35" t="n">
+        <v>75</v>
+      </c>
+      <c r="K20" s="35" t="inlineStr">
+        <is>
+          <t>2026-09-16 00:00:00</t>
+        </is>
+      </c>
+      <c r="L20" s="35" t="inlineStr">
+        <is>
+          <t>2026-09-24 00:00:00</t>
+        </is>
+      </c>
+      <c r="M20" s="35" t="inlineStr">
+        <is>
+          <t>Sprint 07</t>
+        </is>
+      </c>
+      <c r="N20" s="33" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="O20" s="36" t="inlineStr">
+        <is>
+          <t>Equipo Técnico TEMIS</t>
+        </is>
+      </c>
+      <c r="P20" s="36" t="inlineStr">
+        <is>
+          <t>Suite ejecutable Windows offline, transcripción sin consumo de tokens y exportación de paquetes .zip con imágenes HD listas para web.</t>
+        </is>
+      </c>
+      <c r="Q20" s="36" t="inlineStr">
+        <is>
+          <t>2e80a295, 9b64dc3a</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="37" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B21" s="38" t="inlineStr">
+        <is>
+          <t>Ingesta ZIP &amp; Galería Keyframes Web</t>
+        </is>
+      </c>
+      <c r="C21" s="39" t="inlineStr">
+        <is>
+          <t>User Story</t>
+        </is>
+      </c>
+      <c r="D21" s="39" t="inlineStr">
+        <is>
+          <t>Como usuario de TEMIS Web, quiero subir el paquete .zip de Media Studio para que el sistema indexe la transcripción y muestre la galería de capturas de pantalla de evidencias.</t>
+        </is>
+      </c>
+      <c r="E21" s="39" t="inlineStr">
+        <is>
+          <t>1. Crear parser de paquetes .zip en backend. 2. Implementar visor/galería de capturas de pantalla Base64 en frontend Reflex. 3. Habilitar drag-and-drop y progress spinner.</t>
+        </is>
+      </c>
+      <c r="F21" s="39" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G21" s="39" t="inlineStr">
+        <is>
+          <t>Servicio de descompresión e indexación en memoria de paquetes .zip con extracción de 500+ bloques de diálogo y galería de imágenes en Base64.</t>
+        </is>
+      </c>
+      <c r="H21" s="37" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I21" s="40" t="n">
+        <v>8</v>
+      </c>
+      <c r="J21" s="40" t="n">
+        <v>40</v>
+      </c>
+      <c r="K21" s="40" t="inlineStr">
+        <is>
+          <t>2026-09-20 00:00:00</t>
+        </is>
+      </c>
+      <c r="L21" s="40" t="inlineStr">
+        <is>
+          <t>2026-09-26 00:00:00</t>
+        </is>
+      </c>
+      <c r="M21" s="40" t="inlineStr">
+        <is>
+          <t>Sprint 07</t>
+        </is>
+      </c>
+      <c r="N21" s="33" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="O21" s="39" t="inlineStr">
+        <is>
+          <t>Equipo Técnico TEMIS</t>
+        </is>
+      </c>
+      <c r="P21" s="39" t="inlineStr">
+        <is>
+          <t>Ingesta fluida de ZIP con 500+ bloques y renderizado reactivo de capturas HD en tiempo real.</t>
+        </is>
+      </c>
+      <c r="Q21" s="39" t="inlineStr">
+        <is>
+          <t>5061bb4a, da66633c, aa4e6bbb</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="41" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="B22" s="42" t="inlineStr">
+        <is>
+          <t>Plantilla Maestra Word Oficial (.docx)</t>
+        </is>
+      </c>
+      <c r="C22" s="43" t="inlineStr">
+        <is>
+          <t>User Story</t>
+        </is>
+      </c>
+      <c r="D22" s="43" t="inlineStr">
+        <is>
+          <t>Como Jefa de Procesos, quiero que TEMIS genere el Manual de Procedimientos oficial en Word (.docx) cumpliendo al 100% la plantilla maestra corporativa con 4 tablas y evidencias visuales incrustadas.</t>
+        </is>
+      </c>
+      <c r="E22" s="43" t="inlineStr">
+        <is>
+          <t>1. Implementar motor de población sobre Plantilla_Maestra_Oficial_Work_Instructions_TEMIS.docx. 2. Mapear las 4 tablas (Overview, Legal, Actividades, Firmas) con colores institucionales (#0047C7, #98D801, #E2EFD9, #E2E2E2). 3. Incrustar capturas HD en la columna Record Control.</t>
+        </is>
+      </c>
+      <c r="F22" s="43" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G22" s="43" t="inlineStr">
+        <is>
+          <t>Motor de plantillas dinámico en python-docx con clonación XML de filas de actividad, tipografía Poppins 9pt e incrustación de capturas de pantalla de sistemas en Record Control.</t>
+        </is>
+      </c>
+      <c r="H22" s="41" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I22" s="44" t="n">
+        <v>13</v>
+      </c>
+      <c r="J22" s="44" t="n">
+        <v>65</v>
+      </c>
+      <c r="K22" s="44" t="inlineStr">
+        <is>
+          <t>2026-09-22 00:00:00</t>
+        </is>
+      </c>
+      <c r="L22" s="44" t="inlineStr">
+        <is>
+          <t>2026-09-29 00:00:00</t>
+        </is>
+      </c>
+      <c r="M22" s="44" t="inlineStr">
+        <is>
+          <t>Sprint 07</t>
+        </is>
+      </c>
+      <c r="N22" s="33" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="O22" s="43" t="inlineStr">
+        <is>
+          <t>Equipo Técnico TEMIS</t>
+        </is>
+      </c>
+      <c r="P22" s="43" t="inlineStr">
+        <is>
+          <t>Descarga de DOCX oficial idéntico al estándar SAR 90 días con imágenes HD incrustadas, paleta oficial y firmas de aprobación.</t>
+        </is>
+      </c>
+      <c r="Q22" s="43" t="inlineStr">
+        <is>
+          <t>fc7c0eff, 1fcd3fde</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="37" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="B23" s="38" t="inlineStr">
+        <is>
+          <t>Exportador Excel SIPOC Oficial</t>
+        </is>
+      </c>
+      <c r="C23" s="39" t="inlineStr">
+        <is>
+          <t>User Story</t>
+        </is>
+      </c>
+      <c r="D23" s="39" t="inlineStr">
+        <is>
+          <t>Como analista de procesos, quiero exportar la Matriz SIPOC a un archivo Excel idéntico a Plantilla Matriz Sipoc.xlsx con tipografía Century Gothic y 11 columnas B-K.</t>
+        </is>
+      </c>
+      <c r="E23" s="39" t="inlineStr">
+        <is>
+          <t>1. Crear servicio sipoc_exporter.py con formato estandarizado. 2. Configurar estructura 1.0..N, cintillo de Requisitos del Cliente y paleta oficial. 3. Añadir botón de descarga directa en UI.</t>
+        </is>
+      </c>
+      <c r="F23" s="39" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G23" s="39" t="inlineStr">
+        <is>
+          <t>Servicio de exportación en openpyxl que genera matrices SIPOC con diseño corporativo estandarizado (11 columnas pareadas B-K, numeración 1.0 a N y estilos institucionales).</t>
+        </is>
+      </c>
+      <c r="H23" s="37" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="I23" s="40" t="n">
+        <v>5</v>
+      </c>
+      <c r="J23" s="40" t="n">
+        <v>25</v>
+      </c>
+      <c r="K23" s="40" t="inlineStr">
+        <is>
+          <t>2026-09-25 00:00:00</t>
+        </is>
+      </c>
+      <c r="L23" s="40" t="inlineStr">
+        <is>
+          <t>2026-09-29 00:00:00</t>
+        </is>
+      </c>
+      <c r="M23" s="40" t="inlineStr">
+        <is>
+          <t>Sprint 07</t>
+        </is>
+      </c>
+      <c r="N23" s="33" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="O23" s="39" t="inlineStr">
+        <is>
+          <t>Equipo Técnico TEMIS</t>
+        </is>
+      </c>
+      <c r="P23" s="39" t="inlineStr">
+        <is>
+          <t>Archivo .xlsx generado idéntico a Plantilla Matriz Sipoc.xlsx listo para entrega a clientes y directores.</t>
+        </is>
+      </c>
+      <c r="Q23" s="39" t="inlineStr">
+        <is>
+          <t>fc7c0eff</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="41" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="B24" s="42" t="inlineStr">
+        <is>
+          <t>Ingesta Multi-Documento &amp; IA Gemini 2.5</t>
+        </is>
+      </c>
+      <c r="C24" s="43" t="inlineStr">
+        <is>
+          <t>User Story</t>
+        </is>
+      </c>
+      <c r="D24" s="43" t="inlineStr">
+        <is>
+          <t>Como analista, quiero cargar múltiples documentos (entrevista + anexos) para que Gemini 2.5 enriquezca incrementalmente el proceso con citas y puntos de aclaración.</t>
+        </is>
+      </c>
+      <c r="E24" s="43" t="inlineStr">
+        <is>
+          <t>1. Implementar narrative_ai_extractor.py con fusión incremental. 2. Detectar puntos pendientes de aclaración con cliente. 3. Soportar transcripciones masivas con Gemini File API.</t>
+        </is>
+      </c>
+      <c r="F24" s="43" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G24" s="43" t="inlineStr">
+        <is>
+          <t>Motor de enriquecimiento cognitivo con Gemini 2.5 Flash, trazabilidad de citas por párrafo de origen y generación de matriz dual AS-IS / TO-BE.</t>
+        </is>
+      </c>
+      <c r="H24" s="41" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I24" s="44" t="n">
+        <v>8</v>
+      </c>
+      <c r="J24" s="44" t="n">
+        <v>40</v>
+      </c>
+      <c r="K24" s="44" t="inlineStr">
+        <is>
+          <t>2026-09-24 00:00:00</t>
+        </is>
+      </c>
+      <c r="L24" s="44" t="inlineStr">
+        <is>
+          <t>2026-09-30 00:00:00</t>
+        </is>
+      </c>
+      <c r="M24" s="44" t="inlineStr">
+        <is>
+          <t>Sprint 07</t>
+        </is>
+      </c>
+      <c r="N24" s="33" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="O24" s="43" t="inlineStr">
+        <is>
+          <t>Equipo Técnico TEMIS</t>
+        </is>
+      </c>
+      <c r="P24" s="43" t="inlineStr">
+        <is>
+          <t>Fusión de documentos base + anexos sin duplicar pasos, detección de aclaraciones y generación de dual SIPOC/BPMN.</t>
+        </is>
+      </c>
+      <c r="Q24" s="43" t="inlineStr">
+        <is>
+          <t>7229b48e, 3d0d6ded, 92be41e7</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="37" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="B25" s="38" t="inlineStr">
+        <is>
+          <t>Pruebas de Usuario (UAT) &amp; Validación</t>
+        </is>
+      </c>
+      <c r="C25" s="39" t="inlineStr">
+        <is>
+          <t>User Story</t>
+        </is>
+      </c>
+      <c r="D25" s="39" t="inlineStr">
+        <is>
+          <t>Como equipo de procesos y Jefa de Área, queremos realizar sesiones de prueba en vivo (UAT) del flujo completo (Entrevista -&gt; SIPOC -&gt; Flujo -&gt; Word) para validar usabilidad y rendimiento.</t>
+        </is>
+      </c>
+      <c r="E25" s="39" t="inlineStr">
+        <is>
+          <t>1. Ejecutar pruebas con casos de negocio reales (ej. SAR 90 días). 2. Validar edición manual en cada fase del pipeline. 3. Recopilar observaciones y mejoras de interfaz.</t>
+        </is>
+      </c>
+      <c r="F25" s="39" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G25" s="39" t="inlineStr">
+        <is>
+          <t>Protocolo de pruebas de aceptación de usuario (UAT) en entorno productivo Web Cloud con casos reales y medición de tiempos de procesamiento.</t>
+        </is>
+      </c>
+      <c r="H25" s="37" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I25" s="40" t="n">
+        <v>13</v>
+      </c>
+      <c r="J25" s="40" t="n">
+        <v>60</v>
+      </c>
+      <c r="K25" s="40" t="inlineStr">
+        <is>
+          <t>2026-10-01 00:00:00</t>
+        </is>
+      </c>
+      <c r="L25" s="40" t="inlineStr">
+        <is>
+          <t>2026-10-18 00:00:00</t>
+        </is>
+      </c>
+      <c r="M25" s="40" t="inlineStr">
+        <is>
+          <t>Sprint 08</t>
+        </is>
+      </c>
+      <c r="N25" s="34" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="O25" s="39" t="inlineStr">
+        <is>
+          <t>Jefa de Procesos &amp; Equipo Técnico</t>
+        </is>
+      </c>
+      <c r="P25" s="39" t="inlineStr">
+        <is>
+          <t>Aprobación formal de las 4 fases de levantamiento, cero errores bloqueantes y checklist de mejoras aprobado.</t>
+        </is>
+      </c>
+      <c r="Q25" s="39" t="inlineStr">
+        <is>
+          <t>UAT-2026-OCT</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="41" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="B26" s="42" t="inlineStr">
+        <is>
+          <t>Sincronización Bidireccional &amp; Auto-Layout</t>
+        </is>
+      </c>
+      <c r="C26" s="43" t="inlineStr">
+        <is>
+          <t>User Story</t>
+        </is>
+      </c>
+      <c r="D26" s="43" t="inlineStr">
+        <is>
+          <t>Como diseñador de procesos, quiero optimizaciones en el auto-layout de carriles (swimlanes) y sincronización fluida entre la tabla SIPOC y el lienzo BPMN.</t>
+        </is>
+      </c>
+      <c r="E26" s="43" t="inlineStr">
+        <is>
+          <t>1. Afinar algoritmo de posicionamiento de nodos en swimlanes. 2. Mejorar edición reactiva de compuertas de decisión. 3. Implementar feedback de guardado instantáneo.</t>
+        </is>
+      </c>
+      <c r="F26" s="43" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G26" s="43" t="inlineStr">
+        <is>
+          <t>Algoritmo de diagramación automática de swimlanes con ordenamiento topológico y sincronización reactiva bidireccional entre estado SIPOC y lienzo.</t>
+        </is>
+      </c>
+      <c r="H26" s="41" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="I26" s="44" t="n">
+        <v>10</v>
+      </c>
+      <c r="J26" s="44" t="n">
+        <v>50</v>
+      </c>
+      <c r="K26" s="44" t="inlineStr">
+        <is>
+          <t>2026-10-01 00:00:00</t>
+        </is>
+      </c>
+      <c r="L26" s="44" t="inlineStr">
+        <is>
+          <t>2026-10-31 00:00:00</t>
+        </is>
+      </c>
+      <c r="M26" s="44" t="inlineStr">
+        <is>
+          <t>Sprint 08</t>
+        </is>
+      </c>
+      <c r="N26" s="34" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="O26" s="43" t="inlineStr">
+        <is>
+          <t>Equipo Técnico TEMIS</t>
+        </is>
+      </c>
+      <c r="P26" s="43" t="inlineStr">
+        <is>
+          <t>Lienzo BPMN con auto-acomodo de carriles y sincronización en tiempo real sin lag.</t>
+        </is>
+      </c>
+      <c r="Q26" s="43" t="inlineStr">
+        <is>
+          <t>Sprint 08 Dev</t>
         </is>
       </c>
     </row>
@@ -2788,23 +3446,23 @@
         </is>
       </c>
       <c r="B10" s="4">
-        <f>COUNTIF('Backlog Scrum Técnico TEMIS'!B2:B50, "*Reflex Web SaaS Cloud*")</f>
+        <f>COUNTIF('Backlog Scrum Técnico TEMIS'!B2:B65, "*Reflex Web SaaS Cloud*")</f>
         <v/>
       </c>
       <c r="C10" s="4">
-        <f>COUNTIFS('Backlog Scrum Técnico TEMIS'!B2:B50, "*Reflex Web SaaS Cloud*", 'Backlog Scrum Técnico TEMIS'!N2:N50, "Completed")</f>
+        <f>COUNTIFS('Backlog Scrum Técnico TEMIS'!B2:B65, "*Reflex Web SaaS Cloud*", 'Backlog Scrum Técnico TEMIS'!N2:N65, "Completed")</f>
         <v/>
       </c>
       <c r="D10" s="4">
-        <f>COUNTIFS('Backlog Scrum Técnico TEMIS'!B2:B50, "*Reflex Web SaaS Cloud*", 'Backlog Scrum Técnico TEMIS'!N2:N50, "In Progress")</f>
+        <f>COUNTIFS('Backlog Scrum Técnico TEMIS'!B2:B65, "*Reflex Web SaaS Cloud*", 'Backlog Scrum Técnico TEMIS'!N2:N65, "In Progress")</f>
         <v/>
       </c>
       <c r="E10" s="4">
-        <f>COUNTIFS('Backlog Scrum Técnico TEMIS'!B2:B50, "*Reflex Web SaaS Cloud*", 'Backlog Scrum Técnico TEMIS'!N2:N50, "Planned")</f>
+        <f>COUNTIFS('Backlog Scrum Técnico TEMIS'!B2:B65, "*Reflex Web SaaS Cloud*", 'Backlog Scrum Técnico TEMIS'!N2:N65, "Planned")</f>
         <v/>
       </c>
       <c r="F10" s="4">
-        <f>SUMIF('Backlog Scrum Técnico TEMIS'!B2:B50, "*Reflex Web SaaS Cloud*", 'Backlog Scrum Técnico TEMIS'!J2:J50)</f>
+        <f>SUMIF('Backlog Scrum Técnico TEMIS'!B2:B65, "*Reflex Web SaaS Cloud*", 'Backlog Scrum Técnico TEMIS'!J2:J65)</f>
         <v/>
       </c>
       <c r="G10" s="26">
@@ -2822,11 +3480,11 @@
         </is>
       </c>
       <c r="K10" s="4">
-        <f>COUNTIF('Backlog Scrum Técnico TEMIS'!M2:M50, "Sprint 01")</f>
+        <f>COUNTIF('Backlog Scrum Técnico TEMIS'!M2:M65, "Sprint 01")</f>
         <v/>
       </c>
       <c r="L10" s="4">
-        <f>SUMIF('Backlog Scrum Técnico TEMIS'!M2:M50, "Sprint 01", 'Backlog Scrum Técnico TEMIS'!I2:I50)</f>
+        <f>SUMIF('Backlog Scrum Técnico TEMIS'!M2:M65, "Sprint 01", 'Backlog Scrum Técnico TEMIS'!I2:I65)</f>
         <v/>
       </c>
       <c r="M10" s="6" t="inlineStr">
@@ -2835,7 +3493,7 @@
         </is>
       </c>
       <c r="N10" s="26">
-        <f>IF(K10&gt;0, COUNTIFS('Backlog Scrum Técnico TEMIS'!M2:M50, "Sprint 01", 'Backlog Scrum Técnico TEMIS'!N2:N50, "Completed")/K10, 0)</f>
+        <f>IF(K10&gt;0, COUNTIFS('Backlog Scrum Técnico TEMIS'!M2:M65, "Sprint 01", 'Backlog Scrum Técnico TEMIS'!N2:N65, "Completed")/K10, 0)</f>
         <v/>
       </c>
     </row>
@@ -2846,23 +3504,23 @@
         </is>
       </c>
       <c r="B11" s="4">
-        <f>COUNTIF('Backlog Scrum Técnico TEMIS'!B2:B50, "*Parser Lucidchart Determinista*")</f>
+        <f>COUNTIF('Backlog Scrum Técnico TEMIS'!B2:B65, "*Parser Lucidchart Determinista*")</f>
         <v/>
       </c>
       <c r="C11" s="4">
-        <f>COUNTIFS('Backlog Scrum Técnico TEMIS'!B2:B50, "*Parser Lucidchart Determinista*", 'Backlog Scrum Técnico TEMIS'!N2:N50, "Completed")</f>
+        <f>COUNTIFS('Backlog Scrum Técnico TEMIS'!B2:B65, "*Parser Lucidchart Determinista*", 'Backlog Scrum Técnico TEMIS'!N2:N65, "Completed")</f>
         <v/>
       </c>
       <c r="D11" s="4">
-        <f>COUNTIFS('Backlog Scrum Técnico TEMIS'!B2:B50, "*Parser Lucidchart Determinista*", 'Backlog Scrum Técnico TEMIS'!N2:N50, "In Progress")</f>
+        <f>COUNTIFS('Backlog Scrum Técnico TEMIS'!B2:B65, "*Parser Lucidchart Determinista*", 'Backlog Scrum Técnico TEMIS'!N2:N65, "In Progress")</f>
         <v/>
       </c>
       <c r="E11" s="4">
-        <f>COUNTIFS('Backlog Scrum Técnico TEMIS'!B2:B50, "*Parser Lucidchart Determinista*", 'Backlog Scrum Técnico TEMIS'!N2:N50, "Planned")</f>
+        <f>COUNTIFS('Backlog Scrum Técnico TEMIS'!B2:B65, "*Parser Lucidchart Determinista*", 'Backlog Scrum Técnico TEMIS'!N2:N65, "Planned")</f>
         <v/>
       </c>
       <c r="F11" s="4">
-        <f>SUMIF('Backlog Scrum Técnico TEMIS'!B2:B50, "*Parser Lucidchart Determinista*", 'Backlog Scrum Técnico TEMIS'!J2:J50)</f>
+        <f>SUMIF('Backlog Scrum Técnico TEMIS'!B2:B65, "*Parser Lucidchart Determinista*", 'Backlog Scrum Técnico TEMIS'!J2:J65)</f>
         <v/>
       </c>
       <c r="G11" s="26">
@@ -2880,11 +3538,11 @@
         </is>
       </c>
       <c r="K11" s="4">
-        <f>COUNTIF('Backlog Scrum Técnico TEMIS'!M2:M50, "Sprint 02")</f>
+        <f>COUNTIF('Backlog Scrum Técnico TEMIS'!M2:M65, "Sprint 02")</f>
         <v/>
       </c>
       <c r="L11" s="4">
-        <f>SUMIF('Backlog Scrum Técnico TEMIS'!M2:M50, "Sprint 02", 'Backlog Scrum Técnico TEMIS'!I2:I50)</f>
+        <f>SUMIF('Backlog Scrum Técnico TEMIS'!M2:M65, "Sprint 02", 'Backlog Scrum Técnico TEMIS'!I2:I65)</f>
         <v/>
       </c>
       <c r="M11" s="6" t="inlineStr">
@@ -2893,7 +3551,7 @@
         </is>
       </c>
       <c r="N11" s="26">
-        <f>IF(K11&gt;0, COUNTIFS('Backlog Scrum Técnico TEMIS'!M2:M50, "Sprint 02", 'Backlog Scrum Técnico TEMIS'!N2:N50, "Completed")/K11, 0)</f>
+        <f>IF(K11&gt;0, COUNTIFS('Backlog Scrum Técnico TEMIS'!M2:M65, "Sprint 02", 'Backlog Scrum Técnico TEMIS'!N2:N65, "Completed")/K11, 0)</f>
         <v/>
       </c>
     </row>
@@ -2904,23 +3562,23 @@
         </is>
       </c>
       <c r="B12" s="4">
-        <f>COUNTIF('Backlog Scrum Técnico TEMIS'!B2:B50, "*UI/UX Reingeniería Pro*")</f>
+        <f>COUNTIF('Backlog Scrum Técnico TEMIS'!B2:B65, "*UI/UX Reingeniería Pro*")</f>
         <v/>
       </c>
       <c r="C12" s="4">
-        <f>COUNTIFS('Backlog Scrum Técnico TEMIS'!B2:B50, "*UI/UX Reingeniería Pro*", 'Backlog Scrum Técnico TEMIS'!N2:N50, "Completed")</f>
+        <f>COUNTIFS('Backlog Scrum Técnico TEMIS'!B2:B65, "*UI/UX Reingeniería Pro*", 'Backlog Scrum Técnico TEMIS'!N2:N65, "Completed")</f>
         <v/>
       </c>
       <c r="D12" s="4">
-        <f>COUNTIFS('Backlog Scrum Técnico TEMIS'!B2:B50, "*UI/UX Reingeniería Pro*", 'Backlog Scrum Técnico TEMIS'!N2:N50, "In Progress")</f>
+        <f>COUNTIFS('Backlog Scrum Técnico TEMIS'!B2:B65, "*UI/UX Reingeniería Pro*", 'Backlog Scrum Técnico TEMIS'!N2:N65, "In Progress")</f>
         <v/>
       </c>
       <c r="E12" s="4">
-        <f>COUNTIFS('Backlog Scrum Técnico TEMIS'!B2:B50, "*UI/UX Reingeniería Pro*", 'Backlog Scrum Técnico TEMIS'!N2:N50, "Planned")</f>
+        <f>COUNTIFS('Backlog Scrum Técnico TEMIS'!B2:B65, "*UI/UX Reingeniería Pro*", 'Backlog Scrum Técnico TEMIS'!N2:N65, "Planned")</f>
         <v/>
       </c>
       <c r="F12" s="4">
-        <f>SUMIF('Backlog Scrum Técnico TEMIS'!B2:B50, "*UI/UX Reingeniería Pro*", 'Backlog Scrum Técnico TEMIS'!J2:J50)</f>
+        <f>SUMIF('Backlog Scrum Técnico TEMIS'!B2:B65, "*UI/UX Reingeniería Pro*", 'Backlog Scrum Técnico TEMIS'!J2:J65)</f>
         <v/>
       </c>
       <c r="G12" s="26">
@@ -2938,11 +3596,11 @@
         </is>
       </c>
       <c r="K12" s="4">
-        <f>COUNTIF('Backlog Scrum Técnico TEMIS'!M2:M50, "Sprint 03")</f>
+        <f>COUNTIF('Backlog Scrum Técnico TEMIS'!M2:M65, "Sprint 03")</f>
         <v/>
       </c>
       <c r="L12" s="4">
-        <f>SUMIF('Backlog Scrum Técnico TEMIS'!M2:M50, "Sprint 03", 'Backlog Scrum Técnico TEMIS'!I2:I50)</f>
+        <f>SUMIF('Backlog Scrum Técnico TEMIS'!M2:M65, "Sprint 03", 'Backlog Scrum Técnico TEMIS'!I2:I65)</f>
         <v/>
       </c>
       <c r="M12" s="6" t="inlineStr">
@@ -2951,7 +3609,7 @@
         </is>
       </c>
       <c r="N12" s="26">
-        <f>IF(K12&gt;0, COUNTIFS('Backlog Scrum Técnico TEMIS'!M2:M50, "Sprint 03", 'Backlog Scrum Técnico TEMIS'!N2:N50, "Completed")/K12, 0)</f>
+        <f>IF(K12&gt;0, COUNTIFS('Backlog Scrum Técnico TEMIS'!M2:M65, "Sprint 03", 'Backlog Scrum Técnico TEMIS'!N2:N65, "Completed")/K12, 0)</f>
         <v/>
       </c>
     </row>
@@ -2962,23 +3620,23 @@
         </is>
       </c>
       <c r="B13" s="4">
-        <f>COUNTIF('Backlog Scrum Técnico TEMIS'!B2:B50, "*Conexión Interactiva de Nodos*")</f>
+        <f>COUNTIF('Backlog Scrum Técnico TEMIS'!B2:B65, "*Conexión Interactiva de Nodos*")</f>
         <v/>
       </c>
       <c r="C13" s="4">
-        <f>COUNTIFS('Backlog Scrum Técnico TEMIS'!B2:B50, "*Conexión Interactiva de Nodos*", 'Backlog Scrum Técnico TEMIS'!N2:N50, "Completed")</f>
+        <f>COUNTIFS('Backlog Scrum Técnico TEMIS'!B2:B65, "*Conexión Interactiva de Nodos*", 'Backlog Scrum Técnico TEMIS'!N2:N65, "Completed")</f>
         <v/>
       </c>
       <c r="D13" s="4">
-        <f>COUNTIFS('Backlog Scrum Técnico TEMIS'!B2:B50, "*Conexión Interactiva de Nodos*", 'Backlog Scrum Técnico TEMIS'!N2:N50, "In Progress")</f>
+        <f>COUNTIFS('Backlog Scrum Técnico TEMIS'!B2:B65, "*Conexión Interactiva de Nodos*", 'Backlog Scrum Técnico TEMIS'!N2:N65, "In Progress")</f>
         <v/>
       </c>
       <c r="E13" s="4">
-        <f>COUNTIFS('Backlog Scrum Técnico TEMIS'!B2:B50, "*Conexión Interactiva de Nodos*", 'Backlog Scrum Técnico TEMIS'!N2:N50, "Planned")</f>
+        <f>COUNTIFS('Backlog Scrum Técnico TEMIS'!B2:B65, "*Conexión Interactiva de Nodos*", 'Backlog Scrum Técnico TEMIS'!N2:N65, "Planned")</f>
         <v/>
       </c>
       <c r="F13" s="4">
-        <f>SUMIF('Backlog Scrum Técnico TEMIS'!B2:B50, "*Conexión Interactiva de Nodos*", 'Backlog Scrum Técnico TEMIS'!J2:J50)</f>
+        <f>SUMIF('Backlog Scrum Técnico TEMIS'!B2:B65, "*Conexión Interactiva de Nodos*", 'Backlog Scrum Técnico TEMIS'!J2:J65)</f>
         <v/>
       </c>
       <c r="G13" s="26">
@@ -2996,11 +3654,11 @@
         </is>
       </c>
       <c r="K13" s="4">
-        <f>COUNTIF('Backlog Scrum Técnico TEMIS'!M2:M50, "Sprint 04")</f>
+        <f>COUNTIF('Backlog Scrum Técnico TEMIS'!M2:M65, "Sprint 04")</f>
         <v/>
       </c>
       <c r="L13" s="4">
-        <f>SUMIF('Backlog Scrum Técnico TEMIS'!M2:M50, "Sprint 04", 'Backlog Scrum Técnico TEMIS'!I2:I50)</f>
+        <f>SUMIF('Backlog Scrum Técnico TEMIS'!M2:M65, "Sprint 04", 'Backlog Scrum Técnico TEMIS'!I2:I65)</f>
         <v/>
       </c>
       <c r="M13" s="6" t="inlineStr">
@@ -3009,7 +3667,7 @@
         </is>
       </c>
       <c r="N13" s="26">
-        <f>IF(K13&gt;0, COUNTIFS('Backlog Scrum Técnico TEMIS'!M2:M50, "Sprint 04", 'Backlog Scrum Técnico TEMIS'!N2:N50, "Completed")/K13, 0)</f>
+        <f>IF(K13&gt;0, COUNTIFS('Backlog Scrum Técnico TEMIS'!M2:M65, "Sprint 04", 'Backlog Scrum Técnico TEMIS'!N2:N65, "Completed")/K13, 0)</f>
         <v/>
       </c>
     </row>
@@ -3020,23 +3678,23 @@
         </is>
       </c>
       <c r="B14" s="4">
-        <f>COUNTIF('Backlog Scrum Técnico TEMIS'!B2:B50, "*Auditor de Procesos IA (Gemini)*")</f>
+        <f>COUNTIF('Backlog Scrum Técnico TEMIS'!B2:B65, "*Auditor de Procesos IA (Gemini)*")</f>
         <v/>
       </c>
       <c r="C14" s="4">
-        <f>COUNTIFS('Backlog Scrum Técnico TEMIS'!B2:B50, "*Auditor de Procesos IA (Gemini)*", 'Backlog Scrum Técnico TEMIS'!N2:N50, "Completed")</f>
+        <f>COUNTIFS('Backlog Scrum Técnico TEMIS'!B2:B65, "*Auditor de Procesos IA (Gemini)*", 'Backlog Scrum Técnico TEMIS'!N2:N65, "Completed")</f>
         <v/>
       </c>
       <c r="D14" s="4">
-        <f>COUNTIFS('Backlog Scrum Técnico TEMIS'!B2:B50, "*Auditor de Procesos IA (Gemini)*", 'Backlog Scrum Técnico TEMIS'!N2:N50, "In Progress")</f>
+        <f>COUNTIFS('Backlog Scrum Técnico TEMIS'!B2:B65, "*Auditor de Procesos IA (Gemini)*", 'Backlog Scrum Técnico TEMIS'!N2:N65, "In Progress")</f>
         <v/>
       </c>
       <c r="E14" s="4">
-        <f>COUNTIFS('Backlog Scrum Técnico TEMIS'!B2:B50, "*Auditor de Procesos IA (Gemini)*", 'Backlog Scrum Técnico TEMIS'!N2:N50, "Planned")</f>
+        <f>COUNTIFS('Backlog Scrum Técnico TEMIS'!B2:B65, "*Auditor de Procesos IA (Gemini)*", 'Backlog Scrum Técnico TEMIS'!N2:N65, "Planned")</f>
         <v/>
       </c>
       <c r="F14" s="4">
-        <f>SUMIF('Backlog Scrum Técnico TEMIS'!B2:B50, "*Auditor de Procesos IA (Gemini)*", 'Backlog Scrum Técnico TEMIS'!J2:J50)</f>
+        <f>SUMIF('Backlog Scrum Técnico TEMIS'!B2:B65, "*Auditor de Procesos IA (Gemini)*", 'Backlog Scrum Técnico TEMIS'!J2:J65)</f>
         <v/>
       </c>
       <c r="G14" s="26">
@@ -3054,11 +3712,11 @@
         </is>
       </c>
       <c r="K14" s="4">
-        <f>COUNTIF('Backlog Scrum Técnico TEMIS'!M2:M50, "Sprint 05")</f>
+        <f>COUNTIF('Backlog Scrum Técnico TEMIS'!M2:M65, "Sprint 05")</f>
         <v/>
       </c>
       <c r="L14" s="4">
-        <f>SUMIF('Backlog Scrum Técnico TEMIS'!M2:M50, "Sprint 05", 'Backlog Scrum Técnico TEMIS'!I2:I50)</f>
+        <f>SUMIF('Backlog Scrum Técnico TEMIS'!M2:M65, "Sprint 05", 'Backlog Scrum Técnico TEMIS'!I2:I65)</f>
         <v/>
       </c>
       <c r="M14" s="6" t="inlineStr">
@@ -3067,7 +3725,7 @@
         </is>
       </c>
       <c r="N14" s="26">
-        <f>IF(K14&gt;0, COUNTIFS('Backlog Scrum Técnico TEMIS'!M2:M50, "Sprint 05", 'Backlog Scrum Técnico TEMIS'!N2:N50, "Completed")/K14, 0)</f>
+        <f>IF(K14&gt;0, COUNTIFS('Backlog Scrum Técnico TEMIS'!M2:M65, "Sprint 05", 'Backlog Scrum Técnico TEMIS'!N2:N65, "Completed")/K14, 0)</f>
         <v/>
       </c>
     </row>
@@ -3078,23 +3736,23 @@
         </is>
       </c>
       <c r="B15" s="4">
-        <f>COUNTIF('Backlog Scrum Técnico TEMIS'!B2:B50, "*Gobernanza*")</f>
+        <f>COUNTIF('Backlog Scrum Técnico TEMIS'!B2:B65, "*Gobernanza*")</f>
         <v/>
       </c>
       <c r="C15" s="4">
-        <f>COUNTIFS('Backlog Scrum Técnico TEMIS'!B2:B50, "*Gobernanza*", 'Backlog Scrum Técnico TEMIS'!N2:N50, "Completed")</f>
+        <f>COUNTIFS('Backlog Scrum Técnico TEMIS'!B2:B65, "*Gobernanza*", 'Backlog Scrum Técnico TEMIS'!N2:N65, "Completed")</f>
         <v/>
       </c>
       <c r="D15" s="4">
-        <f>COUNTIFS('Backlog Scrum Técnico TEMIS'!B2:B50, "*Gobernanza*", 'Backlog Scrum Técnico TEMIS'!N2:N50, "In Progress")</f>
+        <f>COUNTIFS('Backlog Scrum Técnico TEMIS'!B2:B65, "*Gobernanza*", 'Backlog Scrum Técnico TEMIS'!N2:N65, "In Progress")</f>
         <v/>
       </c>
       <c r="E15" s="4">
-        <f>COUNTIFS('Backlog Scrum Técnico TEMIS'!B2:B50, "*Gobernanza*", 'Backlog Scrum Técnico TEMIS'!N2:N50, "Planned")</f>
+        <f>COUNTIFS('Backlog Scrum Técnico TEMIS'!B2:B65, "*Gobernanza*", 'Backlog Scrum Técnico TEMIS'!N2:N65, "Planned")</f>
         <v/>
       </c>
       <c r="F15" s="4">
-        <f>SUMIF('Backlog Scrum Técnico TEMIS'!B2:B50, "*Gobernanza*", 'Backlog Scrum Técnico TEMIS'!J2:J50)</f>
+        <f>SUMIF('Backlog Scrum Técnico TEMIS'!B2:B65, "*Gobernanza*", 'Backlog Scrum Técnico TEMIS'!J2:J65)</f>
         <v/>
       </c>
       <c r="G15" s="26">
@@ -3112,11 +3770,11 @@
         </is>
       </c>
       <c r="K15" s="4">
-        <f>COUNTIF('Backlog Scrum Técnico TEMIS'!M2:M50, "Sprint 06")</f>
+        <f>COUNTIF('Backlog Scrum Técnico TEMIS'!M2:M65, "Sprint 06")</f>
         <v/>
       </c>
       <c r="L15" s="4">
-        <f>SUMIF('Backlog Scrum Técnico TEMIS'!M2:M50, "Sprint 06", 'Backlog Scrum Técnico TEMIS'!I2:I50)</f>
+        <f>SUMIF('Backlog Scrum Técnico TEMIS'!M2:M65, "Sprint 06", 'Backlog Scrum Técnico TEMIS'!I2:I65)</f>
         <v/>
       </c>
       <c r="M15" s="6" t="inlineStr">
@@ -3125,7 +3783,7 @@
         </is>
       </c>
       <c r="N15" s="26">
-        <f>IF(K15&gt;0, COUNTIFS('Backlog Scrum Técnico TEMIS'!M2:M50, "Sprint 06", 'Backlog Scrum Técnico TEMIS'!N2:N50, "Completed")/K15, 0)</f>
+        <f>IF(K15&gt;0, COUNTIFS('Backlog Scrum Técnico TEMIS'!M2:M65, "Sprint 06", 'Backlog Scrum Técnico TEMIS'!N2:N65, "Completed")/K15, 0)</f>
         <v/>
       </c>
     </row>
@@ -3136,23 +3794,23 @@
         </is>
       </c>
       <c r="B16" s="4">
-        <f>COUNTIF('Backlog Scrum Técnico TEMIS'!B2:B50, "*FastAPI*")</f>
+        <f>COUNTIF('Backlog Scrum Técnico TEMIS'!B2:B65, "*FastAPI*")</f>
         <v/>
       </c>
       <c r="C16" s="4">
-        <f>COUNTIFS('Backlog Scrum Técnico TEMIS'!B2:B50, "*FastAPI*", 'Backlog Scrum Técnico TEMIS'!N2:N50, "Completed")</f>
+        <f>COUNTIFS('Backlog Scrum Técnico TEMIS'!B2:B65, "*FastAPI*", 'Backlog Scrum Técnico TEMIS'!N2:N65, "Completed")</f>
         <v/>
       </c>
       <c r="D16" s="4">
-        <f>COUNTIFS('Backlog Scrum Técnico TEMIS'!B2:B50, "*FastAPI*", 'Backlog Scrum Técnico TEMIS'!N2:N50, "In Progress")</f>
+        <f>COUNTIFS('Backlog Scrum Técnico TEMIS'!B2:B65, "*FastAPI*", 'Backlog Scrum Técnico TEMIS'!N2:N65, "In Progress")</f>
         <v/>
       </c>
       <c r="E16" s="4">
-        <f>COUNTIFS('Backlog Scrum Técnico TEMIS'!B2:B50, "*FastAPI*", 'Backlog Scrum Técnico TEMIS'!N2:N50, "Planned")</f>
+        <f>COUNTIFS('Backlog Scrum Técnico TEMIS'!B2:B65, "*FastAPI*", 'Backlog Scrum Técnico TEMIS'!N2:N65, "Planned")</f>
         <v/>
       </c>
       <c r="F16" s="4">
-        <f>SUMIF('Backlog Scrum Técnico TEMIS'!B2:B50, "*FastAPI*", 'Backlog Scrum Técnico TEMIS'!J2:J50)</f>
+        <f>SUMIF('Backlog Scrum Técnico TEMIS'!B2:B65, "*FastAPI*", 'Backlog Scrum Técnico TEMIS'!J2:J65)</f>
         <v/>
       </c>
       <c r="G16" s="26">
@@ -3170,20 +3828,20 @@
         </is>
       </c>
       <c r="K16" s="4">
-        <f>COUNTIF('Backlog Scrum Técnico TEMIS'!M2:M50, "Sprint 07")</f>
+        <f>COUNTIF('Backlog Scrum Técnico TEMIS'!M2:M65, "Sprint 07")</f>
         <v/>
       </c>
       <c r="L16" s="4">
-        <f>SUMIF('Backlog Scrum Técnico TEMIS'!M2:M50, "Sprint 07", 'Backlog Scrum Técnico TEMIS'!I2:I50)</f>
+        <f>SUMIF('Backlog Scrum Técnico TEMIS'!M2:M65, "Sprint 07", 'Backlog Scrum Técnico TEMIS'!I2:I65)</f>
         <v/>
       </c>
       <c r="M16" s="8" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="N16" s="26">
-        <f>IF(K16&gt;0, COUNTIFS('Backlog Scrum Técnico TEMIS'!M2:M50, "Sprint 07", 'Backlog Scrum Técnico TEMIS'!N2:N50, "Completed")/K16, 0)</f>
+        <f>IF(K16&gt;0, COUNTIFS('Backlog Scrum Técnico TEMIS'!M2:M65, "Sprint 07", 'Backlog Scrum Técnico TEMIS'!N2:N65, "Completed")/K16, 0)</f>
         <v/>
       </c>
     </row>
@@ -3194,23 +3852,23 @@
         </is>
       </c>
       <c r="B17" s="4">
-        <f>COUNTIF('Backlog Scrum Técnico TEMIS'!B2:B50, "*Exportador*")</f>
+        <f>COUNTIF('Backlog Scrum Técnico TEMIS'!B2:B65, "*Exportador*")</f>
         <v/>
       </c>
       <c r="C17" s="4">
-        <f>COUNTIFS('Backlog Scrum Técnico TEMIS'!B2:B50, "*Exportador*", 'Backlog Scrum Técnico TEMIS'!N2:N50, "Completed")</f>
+        <f>COUNTIFS('Backlog Scrum Técnico TEMIS'!B2:B65, "*Exportador*", 'Backlog Scrum Técnico TEMIS'!N2:N65, "Completed")</f>
         <v/>
       </c>
       <c r="D17" s="4">
-        <f>COUNTIFS('Backlog Scrum Técnico TEMIS'!B2:B50, "*Exportador*", 'Backlog Scrum Técnico TEMIS'!N2:N50, "In Progress")</f>
+        <f>COUNTIFS('Backlog Scrum Técnico TEMIS'!B2:B65, "*Exportador*", 'Backlog Scrum Técnico TEMIS'!N2:N65, "In Progress")</f>
         <v/>
       </c>
       <c r="E17" s="4">
-        <f>COUNTIFS('Backlog Scrum Técnico TEMIS'!B2:B50, "*Exportador*", 'Backlog Scrum Técnico TEMIS'!N2:N50, "Planned")</f>
+        <f>COUNTIFS('Backlog Scrum Técnico TEMIS'!B2:B65, "*Exportador*", 'Backlog Scrum Técnico TEMIS'!N2:N65, "Planned")</f>
         <v/>
       </c>
       <c r="F17" s="4">
-        <f>SUMIF('Backlog Scrum Técnico TEMIS'!B2:B50, "*Exportador*", 'Backlog Scrum Técnico TEMIS'!J2:J50)</f>
+        <f>SUMIF('Backlog Scrum Técnico TEMIS'!B2:B65, "*Exportador*", 'Backlog Scrum Técnico TEMIS'!J2:J65)</f>
         <v/>
       </c>
       <c r="G17" s="26">
@@ -3228,20 +3886,20 @@
         </is>
       </c>
       <c r="K17" s="4">
-        <f>COUNTIF('Backlog Scrum Técnico TEMIS'!M2:M50, "Sprint 08")</f>
+        <f>COUNTIF('Backlog Scrum Técnico TEMIS'!M2:M65, "Sprint 08")</f>
         <v/>
       </c>
       <c r="L17" s="4">
-        <f>SUMIF('Backlog Scrum Técnico TEMIS'!M2:M50, "Sprint 08", 'Backlog Scrum Técnico TEMIS'!I2:I50)</f>
+        <f>SUMIF('Backlog Scrum Técnico TEMIS'!M2:M65, "Sprint 08", 'Backlog Scrum Técnico TEMIS'!I2:I65)</f>
         <v/>
       </c>
       <c r="M17" s="9" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="N17" s="26">
-        <f>IF(K17&gt;0, COUNTIFS('Backlog Scrum Técnico TEMIS'!M2:M50, "Sprint 08", 'Backlog Scrum Técnico TEMIS'!N2:N50, "Completed")/K17, 0)</f>
+        <f>IF(K17&gt;0, COUNTIFS('Backlog Scrum Técnico TEMIS'!M2:M65, "Sprint 08", 'Backlog Scrum Técnico TEMIS'!N2:N65, "Completed")/K17, 0)</f>
         <v/>
       </c>
     </row>
@@ -3257,11 +3915,11 @@
         </is>
       </c>
       <c r="K18" s="4">
-        <f>COUNTIF('Backlog Scrum Técnico TEMIS'!M2:M50, "Sprint 09")</f>
+        <f>COUNTIF('Backlog Scrum Técnico TEMIS'!M2:M65, "Sprint 09")</f>
         <v/>
       </c>
       <c r="L18" s="4">
-        <f>SUMIF('Backlog Scrum Técnico TEMIS'!M2:M50, "Sprint 09", 'Backlog Scrum Técnico TEMIS'!I2:I50)</f>
+        <f>SUMIF('Backlog Scrum Técnico TEMIS'!M2:M65, "Sprint 09", 'Backlog Scrum Técnico TEMIS'!I2:I65)</f>
         <v/>
       </c>
       <c r="M18" s="9" t="inlineStr">
@@ -3270,7 +3928,7 @@
         </is>
       </c>
       <c r="N18" s="26">
-        <f>IF(K18&gt;0, COUNTIFS('Backlog Scrum Técnico TEMIS'!M2:M50, "Sprint 09", 'Backlog Scrum Técnico TEMIS'!N2:N50, "Completed")/K18, 0)</f>
+        <f>IF(K18&gt;0, COUNTIFS('Backlog Scrum Técnico TEMIS'!M2:M65, "Sprint 09", 'Backlog Scrum Técnico TEMIS'!N2:N65, "Completed")/K18, 0)</f>
         <v/>
       </c>
     </row>
@@ -3286,11 +3944,11 @@
         </is>
       </c>
       <c r="K19" s="4">
-        <f>COUNTIF('Backlog Scrum Técnico TEMIS'!M2:M50, "Sprint 10")</f>
+        <f>COUNTIF('Backlog Scrum Técnico TEMIS'!M2:M65, "Sprint 10")</f>
         <v/>
       </c>
       <c r="L19" s="4">
-        <f>SUMIF('Backlog Scrum Técnico TEMIS'!M2:M50, "Sprint 10", 'Backlog Scrum Técnico TEMIS'!I2:I50)</f>
+        <f>SUMIF('Backlog Scrum Técnico TEMIS'!M2:M65, "Sprint 10", 'Backlog Scrum Técnico TEMIS'!I2:I65)</f>
         <v/>
       </c>
       <c r="M19" s="9" t="inlineStr">
@@ -3299,7 +3957,7 @@
         </is>
       </c>
       <c r="N19" s="26">
-        <f>IF(K19&gt;0, COUNTIFS('Backlog Scrum Técnico TEMIS'!M2:M50, "Sprint 10", 'Backlog Scrum Técnico TEMIS'!N2:N50, "Completed")/K19, 0)</f>
+        <f>IF(K19&gt;0, COUNTIFS('Backlog Scrum Técnico TEMIS'!M2:M65, "Sprint 10", 'Backlog Scrum Técnico TEMIS'!N2:N65, "Completed")/K19, 0)</f>
         <v/>
       </c>
     </row>
@@ -3328,7 +3986,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -3347,7 +4005,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="24" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -3976,6 +4633,339 @@
       <c r="G21" s="5" t="inlineStr">
         <is>
           <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="41" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="B22" s="43" t="inlineStr">
+        <is>
+          <t>Exportador Gráfico PNG/PDF Pro</t>
+        </is>
+      </c>
+      <c r="C22" s="43" t="inlineStr">
+        <is>
+          <t>Exportador vectorial PNG/PDF y pre-renderizado</t>
+        </is>
+      </c>
+      <c r="D22" s="44" t="inlineStr">
+        <is>
+          <t>Sprint 07</t>
+        </is>
+      </c>
+      <c r="E22" s="41" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F22" s="41" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="G22" s="43" t="inlineStr">
+        <is>
+          <t>603d7945, 158f0ff4</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="37" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B23" s="39" t="inlineStr">
+        <is>
+          <t>Auto-Guardado PostgreSQL Cloud</t>
+        </is>
+      </c>
+      <c r="C23" s="39" t="inlineStr">
+        <is>
+          <t>Sincronización cloud y mitigación de timeouts en Render</t>
+        </is>
+      </c>
+      <c r="D23" s="40" t="inlineStr">
+        <is>
+          <t>Sprint 07</t>
+        </is>
+      </c>
+      <c r="E23" s="37" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F23" s="37" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="G23" s="39" t="inlineStr">
+        <is>
+          <t>237f7f7c, aa4e6bbb, 3590e8d9</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="41" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="B24" s="43" t="inlineStr">
+        <is>
+          <t>🔥 Media Studio Desktop / Whisper &amp; Keyframes</t>
+        </is>
+      </c>
+      <c r="C24" s="43" t="inlineStr">
+        <is>
+          <t>Suite de escritorio offline para extracción multimedia</t>
+        </is>
+      </c>
+      <c r="D24" s="44" t="inlineStr">
+        <is>
+          <t>Sprint 07</t>
+        </is>
+      </c>
+      <c r="E24" s="41" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F24" s="41" t="inlineStr">
+        <is>
+          <t>Crítica</t>
+        </is>
+      </c>
+      <c r="G24" s="43" t="inlineStr">
+        <is>
+          <t>2e80a295, 9b64dc3a, b348d651</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="37" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B25" s="39" t="inlineStr">
+        <is>
+          <t>Ingesta ZIP &amp; Galería Keyframes Web</t>
+        </is>
+      </c>
+      <c r="C25" s="39" t="inlineStr">
+        <is>
+          <t>Ingesta de paquetes ZIP con galería Base64 de capturas</t>
+        </is>
+      </c>
+      <c r="D25" s="40" t="inlineStr">
+        <is>
+          <t>Sprint 07</t>
+        </is>
+      </c>
+      <c r="E25" s="37" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F25" s="37" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="G25" s="39" t="inlineStr">
+        <is>
+          <t>5061bb4a, da66633c, 012ff586, 88b86dd8</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="41" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="B26" s="43" t="inlineStr">
+        <is>
+          <t>Plantilla Maestra Word Oficial (.docx)</t>
+        </is>
+      </c>
+      <c r="C26" s="43" t="inlineStr">
+        <is>
+          <t>Manual oficial Word 4 tablas con capturas HD incrustadas</t>
+        </is>
+      </c>
+      <c r="D26" s="44" t="inlineStr">
+        <is>
+          <t>Sprint 07</t>
+        </is>
+      </c>
+      <c r="E26" s="41" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F26" s="41" t="inlineStr">
+        <is>
+          <t>Crítica</t>
+        </is>
+      </c>
+      <c r="G26" s="43" t="inlineStr">
+        <is>
+          <t>fc7c0eff, 1fcd3fde, d785d2c8</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="37" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="B27" s="39" t="inlineStr">
+        <is>
+          <t>Exportador Excel SIPOC Oficial</t>
+        </is>
+      </c>
+      <c r="C27" s="39" t="inlineStr">
+        <is>
+          <t>Generador Excel idéntico a Plantilla Matriz Sipoc.xlsx</t>
+        </is>
+      </c>
+      <c r="D27" s="40" t="inlineStr">
+        <is>
+          <t>Sprint 07</t>
+        </is>
+      </c>
+      <c r="E27" s="37" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F27" s="37" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="G27" s="39" t="inlineStr">
+        <is>
+          <t>fc7c0eff, 1fcd3fde</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="41" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="B28" s="43" t="inlineStr">
+        <is>
+          <t>Ingesta Multi-Documento &amp; IA Gemini 2.5</t>
+        </is>
+      </c>
+      <c r="C28" s="43" t="inlineStr">
+        <is>
+          <t>Enriquecimiento cognitivo incremental con Gemini 2.5</t>
+        </is>
+      </c>
+      <c r="D28" s="44" t="inlineStr">
+        <is>
+          <t>Sprint 07</t>
+        </is>
+      </c>
+      <c r="E28" s="41" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F28" s="41" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="G28" s="43" t="inlineStr">
+        <is>
+          <t>7229b48e, 3d0d6ded, 92be41e7</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="37" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="B29" s="39" t="inlineStr">
+        <is>
+          <t>Pruebas de Usuario (UAT) &amp; Validación</t>
+        </is>
+      </c>
+      <c r="C29" s="39" t="inlineStr">
+        <is>
+          <t>Sesiones de prueba en vivo con Jefa de Procesos</t>
+        </is>
+      </c>
+      <c r="D29" s="40" t="inlineStr">
+        <is>
+          <t>Sprint 08</t>
+        </is>
+      </c>
+      <c r="E29" s="37" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F29" s="37" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="G29" s="39" t="inlineStr">
+        <is>
+          <t>En Curso (Sprint 08)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="41" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="B30" s="43" t="inlineStr">
+        <is>
+          <t>Sincronización Bidireccional &amp; Auto-Layout</t>
+        </is>
+      </c>
+      <c r="C30" s="43" t="inlineStr">
+        <is>
+          <t>Optimización de swimlanes y sincronización reactiva</t>
+        </is>
+      </c>
+      <c r="D30" s="44" t="inlineStr">
+        <is>
+          <t>Sprint 08</t>
+        </is>
+      </c>
+      <c r="E30" s="41" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F30" s="41" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G30" s="43" t="inlineStr">
+        <is>
+          <t>En Curso (Sprint 08)</t>
         </is>
       </c>
     </row>
@@ -3993,7 +4983,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G48"/>
+  <dimension ref="A1:G51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -4043,1741 +5033,1852 @@
       </c>
     </row>
     <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="11" t="inlineStr">
-        <is>
-          <t>2f8a70d</t>
-        </is>
-      </c>
-      <c r="B2" s="11" t="inlineStr">
-        <is>
-          <t>2026-09-10 09:23:24 -0600</t>
-        </is>
-      </c>
-      <c r="C2" s="27" t="inlineStr">
+      <c r="A2" s="41" t="inlineStr">
+        <is>
+          <t>1fcd3fde</t>
+        </is>
+      </c>
+      <c r="B2" s="44" t="inlineStr">
+        <is>
+          <t>2026-09-29 16:44:13 -0600</t>
+        </is>
+      </c>
+      <c r="C2" s="43" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D2" s="27" t="inlineStr">
-        <is>
-          <t>fix: normaliza spacing a valores enteros y corrige tags de iconos circle-play y circle-stop en componentes de UI</t>
-        </is>
-      </c>
-      <c r="E2" s="27" t="inlineStr">
-        <is>
-          <t>Frontend Reflex / UI</t>
-        </is>
-      </c>
-      <c r="F2" s="11" t="inlineStr">
-        <is>
-          <t>Sprint 06 - Sep 2026</t>
-        </is>
-      </c>
-      <c r="G2" s="27" t="inlineStr">
-        <is>
-          <t>Corrección de validación de tipos Radix UI en compilador Reflex y ajuste de nombres oficiales de iconos Lucide.</t>
+      <c r="D2" s="43" t="inlineStr">
+        <is>
+          <t>feat(narrative): integrate official master DOCX template engine matching Plantilla_Maestra_Oficial_Work_Instructions_TEMIS</t>
+        </is>
+      </c>
+      <c r="E2" s="41" t="inlineStr">
+        <is>
+          <t>Plantilla Maestra Word / Narrativa</t>
+        </is>
+      </c>
+      <c r="F2" s="44" t="inlineStr">
+        <is>
+          <t>Sprint 07 - Sep 2026</t>
+        </is>
+      </c>
+      <c r="G2" s="43" t="inlineStr">
+        <is>
+          <t>Integración del motor de población sobre Plantilla_Maestra_Oficial_Work_Instructions_TEMIS.docx y 4 tablas oficiales.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>9805816</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>2026-09-10 09:17:35 -0600</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="A3" s="37" t="inlineStr">
+        <is>
+          <t>fc7c0eff</t>
+        </is>
+      </c>
+      <c r="B3" s="40" t="inlineStr">
+        <is>
+          <t>2026-09-29 14:45:49 -0600</t>
+        </is>
+      </c>
+      <c r="C3" s="39" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
-        <is>
-          <t>feat: reingenieria UI/UX integral: header minimalista 50px, dock de formas izquierdo, inspector de propiedades derecho, barra de pestañas y zoom inferior, y ruteo perimetral exacto de conectores Bézier</t>
-        </is>
-      </c>
-      <c r="E3" s="5" t="inlineStr">
-        <is>
-          <t>UI/UX / Suite Pro</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>Sprint 06 - Sep 2026</t>
-        </is>
-      </c>
-      <c r="G3" s="5" t="inlineStr">
-        <is>
-          <t>Transformación completa del layout visual a estándar Lucidchart/Figma (+25% área de lienzo) con inspector contextual y ruteo Este-Oeste.</t>
+      <c r="D3" s="39" t="inlineStr">
+        <is>
+          <t>feat(export): standardize official Word 4-table document to match SAR 90 dias and Excel SIPOC template</t>
+        </is>
+      </c>
+      <c r="E3" s="37" t="inlineStr">
+        <is>
+          <t>Plantilla Maestra Word / Narrativa</t>
+        </is>
+      </c>
+      <c r="F3" s="40" t="inlineStr">
+        <is>
+          <t>Sprint 07 - Sep 2026</t>
+        </is>
+      </c>
+      <c r="G3" s="39" t="inlineStr">
+        <is>
+          <t>Integración del motor de población sobre Plantilla_Maestra_Oficial_Work_Instructions_TEMIS.docx y 4 tablas oficiales.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="11" t="inlineStr">
-        <is>
-          <t>3e76b5d</t>
-        </is>
-      </c>
-      <c r="B4" s="11" t="inlineStr">
-        <is>
-          <t>2026-09-10 09:04:19 -0600</t>
-        </is>
-      </c>
-      <c r="C4" s="27" t="inlineStr">
+      <c r="A4" s="41" t="inlineStr">
+        <is>
+          <t>6a9f6bdc</t>
+        </is>
+      </c>
+      <c r="B4" s="44" t="inlineStr">
+        <is>
+          <t>2026-09-28 19:13:02 -0600</t>
+        </is>
+      </c>
+      <c r="C4" s="43" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D4" s="27" t="inlineStr">
-        <is>
-          <t>fix: maneja el evento on_change de selección de nodo directamente en el State handler evitando VarTypeError</t>
-        </is>
-      </c>
-      <c r="E4" s="27" t="inlineStr">
-        <is>
-          <t>Frontend Reflex / State</t>
-        </is>
-      </c>
-      <c r="F4" s="11" t="inlineStr">
-        <is>
-          <t>Sprint 06 - Sep 2026</t>
-        </is>
-      </c>
-      <c r="G4" s="27" t="inlineStr">
-        <is>
-          <t>Delegación del parseo de cadenas al State handler del servidor resolviendo error de evaluación AST en Reflex.</t>
+      <c r="D4" s="43" t="inlineStr">
+        <is>
+          <t>fix(cascade): blindar VerificadorEstatus y agregar safety guard en AgenteComunicador contra desvios a GChat</t>
+        </is>
+      </c>
+      <c r="E4" s="41" t="inlineStr">
+        <is>
+          <t>Frontend / UI</t>
+        </is>
+      </c>
+      <c r="F4" s="44" t="inlineStr">
+        <is>
+          <t>Sprint 07 - Sep 2026</t>
+        </is>
+      </c>
+      <c r="G4" s="43" t="inlineStr">
+        <is>
+          <t>fix(cascade): blindar VerificadorEstatus y agregar safety guard en AgenteComunicador contra desvios a GChat</t>
         </is>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>7bc6e6a</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>2026-09-10 08:58:47 -0600</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="A5" s="37" t="inlineStr">
+        <is>
+          <t>d785d2c8</t>
+        </is>
+      </c>
+      <c r="B5" s="40" t="inlineStr">
+        <is>
+          <t>2026-09-25 07:55:43 -0600</t>
+        </is>
+      </c>
+      <c r="C5" s="39" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>fix: reemplaza iteracion directa de Var por target_node_options reactivo en connect_modal</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>Frontend Reflex / State</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>Sprint 06 - Sep 2026</t>
-        </is>
-      </c>
-      <c r="G5" s="5" t="inlineStr">
-        <is>
-          <t>Implementación de propiedad computada @rx.var target_node_options eliminando iteración directa sobre variables de estado reactivas.</t>
+      <c r="D5" s="39" t="inlineStr">
+        <is>
+          <t>fix(state): map charter scope to scope_in and declare private cached narrative state variables</t>
+        </is>
+      </c>
+      <c r="E5" s="37" t="inlineStr">
+        <is>
+          <t>Plantilla Maestra Word / Narrativa</t>
+        </is>
+      </c>
+      <c r="F5" s="40" t="inlineStr">
+        <is>
+          <t>Sprint 07 - Sep 2026</t>
+        </is>
+      </c>
+      <c r="G5" s="39" t="inlineStr">
+        <is>
+          <t>Integración del motor de población sobre Plantilla_Maestra_Oficial_Work_Instructions_TEMIS.docx y 4 tablas oficiales.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="11" t="inlineStr">
-        <is>
-          <t>592127e</t>
-        </is>
-      </c>
-      <c r="B6" s="11" t="inlineStr">
-        <is>
-          <t>2026-09-10 08:53:41 -0600</t>
-        </is>
-      </c>
-      <c r="C6" s="27" t="inlineStr">
+      <c r="A6" s="41" t="inlineStr">
+        <is>
+          <t>237f7f7c</t>
+        </is>
+      </c>
+      <c r="B6" s="44" t="inlineStr">
+        <is>
+          <t>2026-09-25 07:36:53 -0600</t>
+        </is>
+      </c>
+      <c r="C6" s="43" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D6" s="27" t="inlineStr">
-        <is>
-          <t>feat: implementa conexión interactiva de nodos, indicador de auto-guardado y auditoría de gobierno con IA de Gemini</t>
-        </is>
-      </c>
-      <c r="E6" s="27" t="inlineStr">
-        <is>
-          <t>Conectores / IA Gemini</t>
-        </is>
-      </c>
-      <c r="F6" s="11" t="inlineStr">
-        <is>
-          <t>Sprint 06 - Sep 2026</t>
-        </is>
-      </c>
-      <c r="G6" s="27" t="inlineStr">
-        <is>
-          <t>Creación de modal de conexión interactiva de casillas, badge en tiempo real de auto-guardado y motor de auditoría de gobernanza con IA.</t>
+      <c r="D6" s="43" t="inlineStr">
+        <is>
+          <t>fix(deploy): use python -m backend.main to bind PORT in Render for temis-backend</t>
+        </is>
+      </c>
+      <c r="E6" s="41" t="inlineStr">
+        <is>
+          <t>DevOps / Despliegue Cloud</t>
+        </is>
+      </c>
+      <c r="F6" s="44" t="inlineStr">
+        <is>
+          <t>Sprint 07 - Sep 2026</t>
+        </is>
+      </c>
+      <c r="G6" s="43" t="inlineStr">
+        <is>
+          <t>Optimización de servidor de producción ASGI, configuración de endpoints de upload y resolución de timeouts en Render.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>55e43d8</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>2026-08-28 13:39:13 -0600</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="A7" s="37" t="inlineStr">
+        <is>
+          <t>aa4e6bbb</t>
+        </is>
+      </c>
+      <c r="B7" s="40" t="inlineStr">
+        <is>
+          <t>2026-09-24 21:52:23 -0600</t>
+        </is>
+      </c>
+      <c r="C7" s="39" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>fix: parser nativo detecta exactamente las 8 pestañas originales de Lucidchart por limites de pagina (Bloques As Is y To Be, Proceso N2, Casos especiales, etc.) y carga la primera pestaña por defecto</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>Parser Nativo Lucidchart</t>
-        </is>
-      </c>
-      <c r="F7" s="4" t="inlineStr">
-        <is>
-          <t>Sprint 05 - Ago 2026</t>
-        </is>
-      </c>
-      <c r="G7" s="5" t="inlineStr">
-        <is>
-          <t>Detección biunívoca de las 8 pestañas originales de Lucidchart por límites de página (Page ID / Name=='Page') sin alucinaciones de IA.</t>
+      <c r="D7" s="39" t="inlineStr">
+        <is>
+          <t>fix(prod_server): register reflex /_upload endpoints and set Upload.is_used for production server</t>
+        </is>
+      </c>
+      <c r="E7" s="37" t="inlineStr">
+        <is>
+          <t>Ingesta ZIP / Galería Evidencias</t>
+        </is>
+      </c>
+      <c r="F7" s="40" t="inlineStr">
+        <is>
+          <t>Sprint 07 - Sep 2026</t>
+        </is>
+      </c>
+      <c r="G7" s="39" t="inlineStr">
+        <is>
+          <t>Parser de paquetes .zip de Media Studio, visor reactivo de capturas Base64 y drag-and-drop en web.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="11" t="inlineStr">
-        <is>
-          <t>5a73bec</t>
-        </is>
-      </c>
-      <c r="B8" s="11" t="inlineStr">
-        <is>
-          <t>2026-08-28 13:19:46 -0600</t>
-        </is>
-      </c>
-      <c r="C8" s="27" t="inlineStr">
+      <c r="A8" s="41" t="inlineStr">
+        <is>
+          <t>3590e8d9</t>
+        </is>
+      </c>
+      <c r="B8" s="44" t="inlineStr">
+        <is>
+          <t>2026-09-24 21:36:55 -0600</t>
+        </is>
+      </c>
+      <c r="C8" s="43" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D8" s="27" t="inlineStr">
-        <is>
-          <t>fix: posiciona la barra de pestañas en el encabezado principal e ignora nodos indice de titulos de pagina en parser de Lucidchart</t>
-        </is>
-      </c>
-      <c r="E8" s="27" t="inlineStr">
-        <is>
-          <t>Parser / Navegación</t>
-        </is>
-      </c>
-      <c r="F8" s="11" t="inlineStr">
-        <is>
-          <t>Sprint 05 - Ago 2026</t>
-        </is>
-      </c>
-      <c r="G8" s="27" t="inlineStr">
-        <is>
-          <t>Filtrado automático de figuras índice y reubicación de pestañas del proyecto.</t>
+      <c r="D8" s="43" t="inlineStr">
+        <is>
+          <t>perf(core): add cache-first loading strategy to eliminate event loop lag on Drive calls</t>
+        </is>
+      </c>
+      <c r="E8" s="41" t="inlineStr">
+        <is>
+          <t>Frontend / UI</t>
+        </is>
+      </c>
+      <c r="F8" s="44" t="inlineStr">
+        <is>
+          <t>Sprint 07 - Sep 2026</t>
+        </is>
+      </c>
+      <c r="G8" s="43" t="inlineStr">
+        <is>
+          <t>perf(core): add cache-first loading strategy to eliminate event loop lag on Drive calls</t>
         </is>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>91f5bfe</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>2026-08-28 13:07:30 -0600</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="A9" s="37" t="inlineStr">
+        <is>
+          <t>012ff586</t>
+        </is>
+      </c>
+      <c r="B9" s="40" t="inlineStr">
+        <is>
+          <t>2026-09-24 21:25:33 -0600</t>
+        </is>
+      </c>
+      <c r="C9" s="39" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>fix: reemplaza variante invalida ghost por soft en el componente rx.input del encabezado</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>Frontend Reflex / UI</t>
-        </is>
-      </c>
-      <c r="F9" s="4" t="inlineStr">
-        <is>
-          <t>Sprint 05 - Ago 2026</t>
-        </is>
-      </c>
-      <c r="G9" s="5" t="inlineStr">
-        <is>
-          <t>Corrección de prop variant en componente rx.input para compatibilidad con Radix Themes.</t>
+      <c r="D9" s="39" t="inlineStr">
+        <is>
+          <t>fix(upload): remove strict MIME accept filter to allow seamless Windows ZIP drag-and-drop</t>
+        </is>
+      </c>
+      <c r="E9" s="37" t="inlineStr">
+        <is>
+          <t>Ingesta ZIP / Galería Evidencias</t>
+        </is>
+      </c>
+      <c r="F9" s="40" t="inlineStr">
+        <is>
+          <t>Sprint 07 - Sep 2026</t>
+        </is>
+      </c>
+      <c r="G9" s="39" t="inlineStr">
+        <is>
+          <t>Parser de paquetes .zip de Media Studio, visor reactivo de capturas Base64 y drag-and-drop en web.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="11" t="inlineStr">
-        <is>
-          <t>c53b6e6</t>
-        </is>
-      </c>
-      <c r="B10" s="11" t="inlineStr">
-        <is>
-          <t>2026-08-28 13:01:06 -0600</t>
-        </is>
-      </c>
-      <c r="C10" s="27" t="inlineStr">
+      <c r="A10" s="41" t="inlineStr">
+        <is>
+          <t>88b86dd8</t>
+        </is>
+      </c>
+      <c r="B10" s="44" t="inlineStr">
+        <is>
+          <t>2026-09-24 21:20:44 -0600</t>
+        </is>
+      </c>
+      <c r="C10" s="43" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D10" s="27" t="inlineStr">
-        <is>
-          <t>fix: fija versiones exactas de dependencias en requirements.txt eliminando resolucion de pip lenta en Render</t>
-        </is>
-      </c>
-      <c r="E10" s="27" t="inlineStr">
-        <is>
-          <t>DevOps / Build Render</t>
-        </is>
-      </c>
-      <c r="F10" s="11" t="inlineStr">
-        <is>
-          <t>Sprint 05 - Ago 2026</t>
-        </is>
-      </c>
-      <c r="G10" s="27" t="inlineStr">
-        <is>
-          <t>Fijación estricta de versiones de librerías de Google y Reflex acelerando la instalación en Render a &lt; 10 segundos.</t>
+      <c r="D10" s="43" t="inlineStr">
+        <is>
+          <t>fix(upload): add MIME type fallbacks and handler diagnostics for ZIP uploads</t>
+        </is>
+      </c>
+      <c r="E10" s="41" t="inlineStr">
+        <is>
+          <t>Ingesta ZIP / Galería Evidencias</t>
+        </is>
+      </c>
+      <c r="F10" s="44" t="inlineStr">
+        <is>
+          <t>Sprint 07 - Sep 2026</t>
+        </is>
+      </c>
+      <c r="G10" s="43" t="inlineStr">
+        <is>
+          <t>Parser de paquetes .zip de Media Studio, visor reactivo de capturas Base64 y drag-and-drop en web.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>be0bc21</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>2026-08-28 12:56:24 -0600</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="A11" s="35" t="inlineStr">
+        <is>
+          <t>b348d651</t>
+        </is>
+      </c>
+      <c r="B11" s="35" t="inlineStr">
+        <is>
+          <t>2026-09-24 21:04:18 -0600</t>
+        </is>
+      </c>
+      <c r="C11" s="36" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>fix: elimina tracking de AGENTS.md y CLAUDE.md y los agrega a .gitignore resolviendo UnicodeDecodeError en reflex init en Render</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>DevOps / Git</t>
-        </is>
-      </c>
-      <c r="F11" s="4" t="inlineStr">
-        <is>
-          <t>Sprint 05 - Ago 2026</t>
-        </is>
-      </c>
-      <c r="G11" s="5" t="inlineStr">
-        <is>
-          <t>Eliminación de archivos locales del índice Git previniendo fallas de codificación en el runner de Render.</t>
+      <c r="D11" s="36" t="inlineStr">
+        <is>
+          <t>revert(studio): keep Temis Media Studio untouched per user instruction</t>
+        </is>
+      </c>
+      <c r="E11" s="35" t="inlineStr">
+        <is>
+          <t>🔥 HITO: TEMIS Media Studio Desktop</t>
+        </is>
+      </c>
+      <c r="F11" s="35" t="inlineStr">
+        <is>
+          <t>Sprint 07 - Sep 2026</t>
+        </is>
+      </c>
+      <c r="G11" s="36" t="inlineStr">
+        <is>
+          <t>Suite de escritorio offline para extracción multimedia, transcripción local Whisper y captura de fotogramas clave HD.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="11" t="inlineStr">
-        <is>
-          <t>c120d08</t>
-        </is>
-      </c>
-      <c r="B12" s="11" t="inlineStr">
-        <is>
-          <t>2026-08-28 12:48:52 -0600</t>
-        </is>
-      </c>
-      <c r="C12" s="27" t="inlineStr">
+      <c r="A12" s="41" t="inlineStr">
+        <is>
+          <t>da66633c</t>
+        </is>
+      </c>
+      <c r="B12" s="44" t="inlineStr">
+        <is>
+          <t>2026-09-24 20:58:55 -0600</t>
+        </is>
+      </c>
+      <c r="C12" s="43" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D12" s="27" t="inlineStr">
-        <is>
-          <t>fix: convierte AGENTS.md y CLAUDE.md a codificacion UTF-8 limpia eliminando caracteres cp1252 para reflex init en Render</t>
-        </is>
-      </c>
-      <c r="E12" s="27" t="inlineStr">
-        <is>
-          <t>DevOps / Encoding</t>
-        </is>
-      </c>
-      <c r="F12" s="11" t="inlineStr">
-        <is>
-          <t>Sprint 05 - Ago 2026</t>
-        </is>
-      </c>
-      <c r="G12" s="27" t="inlineStr">
-        <is>
-          <t>Saneamiento de codificación UTF-8 en archivos de workspace.</t>
+      <c r="D12" s="43" t="inlineStr">
+        <is>
+          <t>fix(narrative): optimize ZIP package handling, add progress spinners and compact auto-zip</t>
+        </is>
+      </c>
+      <c r="E12" s="41" t="inlineStr">
+        <is>
+          <t>Plantilla Maestra Word / Narrativa</t>
+        </is>
+      </c>
+      <c r="F12" s="44" t="inlineStr">
+        <is>
+          <t>Sprint 07 - Sep 2026</t>
+        </is>
+      </c>
+      <c r="G12" s="43" t="inlineStr">
+        <is>
+          <t>Integración del motor de población sobre Plantilla_Maestra_Oficial_Work_Instructions_TEMIS.docx y 4 tablas oficiales.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>d332d20</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>2026-08-28 11:48:48 -0600</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
+      <c r="A13" s="37" t="inlineStr">
+        <is>
+          <t>21fb4dc1</t>
+        </is>
+      </c>
+      <c r="B13" s="40" t="inlineStr">
+        <is>
+          <t>2026-09-24 20:46:08 -0600</t>
+        </is>
+      </c>
+      <c r="C13" s="39" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>feat: agrega menú Archivo ▾ profesional, edicion interactiva del nombre del proyecto, boton Nueva Pestaña y modal Abrir Reciente</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>Frontend / Archivo</t>
-        </is>
-      </c>
-      <c r="F13" s="4" t="inlineStr">
-        <is>
-          <t>Sprint 05 - Ago 2026</t>
-        </is>
-      </c>
-      <c r="G13" s="5" t="inlineStr">
-        <is>
-          <t>Menú desplegable Archivo (Nuevo, Guardar, Exportar, Importar), título editable y modal de proyectos recientes.</t>
+      <c r="D13" s="39" t="inlineStr">
+        <is>
+          <t>feat(persistence): enable dynamic Google Drive project scanning &amp; cloud user directory persistence</t>
+        </is>
+      </c>
+      <c r="E13" s="37" t="inlineStr">
+        <is>
+          <t>Google Drive / Persistencia</t>
+        </is>
+      </c>
+      <c r="F13" s="40" t="inlineStr">
+        <is>
+          <t>Sprint 07 - Sep 2026</t>
+        </is>
+      </c>
+      <c r="G13" s="39" t="inlineStr">
+        <is>
+          <t>Respaldo automático en Google Workspace Shared Drive con Service Account institucional.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="11" t="inlineStr">
-        <is>
-          <t>c77d1ae</t>
-        </is>
-      </c>
-      <c r="B14" s="11" t="inlineStr">
-        <is>
-          <t>2026-08-27 20:52:50 -0600</t>
-        </is>
-      </c>
-      <c r="C14" s="27" t="inlineStr">
+      <c r="A14" s="35" t="inlineStr">
+        <is>
+          <t>5061bb4a</t>
+        </is>
+      </c>
+      <c r="B14" s="35" t="inlineStr">
+        <is>
+          <t>2026-09-24 20:35:14 -0600</t>
+        </is>
+      </c>
+      <c r="C14" s="36" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D14" s="27" t="inlineStr">
-        <is>
-          <t>fix: restaura metodo move_selected_node en FlowState y corrige etiqueta de icono Lucide columns-2</t>
-        </is>
-      </c>
-      <c r="E14" s="27" t="inlineStr">
-        <is>
-          <t>Frontend Reflex / Canvas</t>
-        </is>
-      </c>
-      <c r="F14" s="11" t="inlineStr">
-        <is>
-          <t>Sprint 05 - Ago 2026</t>
-        </is>
-      </c>
-      <c r="G14" s="27" t="inlineStr">
-        <is>
-          <t>Restauración de manejadores de movimiento de nodos y compatibilidad de iconos.</t>
+      <c r="D14" s="36" t="inlineStr">
+        <is>
+          <t>feat(zip-ingest): add TEMIS Media Studio ZIP package ingestion, Base64 screenshot gallery, and unified pipeline in web</t>
+        </is>
+      </c>
+      <c r="E14" s="35" t="inlineStr">
+        <is>
+          <t>🔥 HITO: TEMIS Media Studio Desktop</t>
+        </is>
+      </c>
+      <c r="F14" s="35" t="inlineStr">
+        <is>
+          <t>Sprint 07 - Sep 2026</t>
+        </is>
+      </c>
+      <c r="G14" s="36" t="inlineStr">
+        <is>
+          <t>Suite de escritorio offline para extracción multimedia, transcripción local Whisper y captura de fotogramas clave HD.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>41b5d0a</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>2026-08-27 20:49:24 -0600</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
+      <c r="A15" s="35" t="inlineStr">
+        <is>
+          <t>9b64dc3a</t>
+        </is>
+      </c>
+      <c r="B15" s="35" t="inlineStr">
+        <is>
+          <t>2026-09-24 18:08:03 -0600</t>
+        </is>
+      </c>
+      <c r="C15" s="36" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>feat: agrega barra de navegacion de pestañas dinamicas por pagina de diagrama importada desde Lucidchart</t>
-        </is>
-      </c>
-      <c r="E15" s="5" t="inlineStr">
-        <is>
-          <t>Frontend / Pestañas</t>
-        </is>
-      </c>
-      <c r="F15" s="4" t="inlineStr">
-        <is>
-          <t>Sprint 05 - Ago 2026</t>
-        </is>
-      </c>
-      <c r="G15" s="5" t="inlineStr">
-        <is>
-          <t>Barra de navegación multi-pestaña con preservación de estado al alternar entre diagramas.</t>
+      <c r="D15" s="36" t="inlineStr">
+        <is>
+          <t>feat(studio): switch TEMIS Media Studio to 100% local faster-whisper engine and zero-token local process builder</t>
+        </is>
+      </c>
+      <c r="E15" s="35" t="inlineStr">
+        <is>
+          <t>🔥 HITO: TEMIS Media Studio Desktop</t>
+        </is>
+      </c>
+      <c r="F15" s="35" t="inlineStr">
+        <is>
+          <t>Sprint 07 - Sep 2026</t>
+        </is>
+      </c>
+      <c r="G15" s="36" t="inlineStr">
+        <is>
+          <t>Suite de escritorio offline para extracción multimedia, transcripción local Whisper y captura de fotogramas clave HD.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="11" t="inlineStr">
-        <is>
-          <t>7bcb6ac</t>
-        </is>
-      </c>
-      <c r="B16" s="11" t="inlineStr">
-        <is>
-          <t>2026-08-27 20:37:56 -0600</t>
-        </is>
-      </c>
-      <c r="C16" s="27" t="inlineStr">
+      <c r="A16" s="35" t="inlineStr">
+        <is>
+          <t>2e80a295</t>
+        </is>
+      </c>
+      <c r="B16" s="35" t="inlineStr">
+        <is>
+          <t>2026-09-24 17:32:50 -0600</t>
+        </is>
+      </c>
+      <c r="C16" s="36" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D16" s="27" t="inlineStr">
-        <is>
-          <t>fix: separa diagramas por Page ID de Lucidchart y fija los controles de Zoom flotantes visibilidad 100%</t>
-        </is>
-      </c>
-      <c r="E16" s="27" t="inlineStr">
-        <is>
-          <t>Parser / Canvas</t>
-        </is>
-      </c>
-      <c r="F16" s="11" t="inlineStr">
-        <is>
-          <t>Sprint 05 - Ago 2026</t>
-        </is>
-      </c>
-      <c r="G16" s="27" t="inlineStr">
-        <is>
-          <t>Agrupamiento de nodos y líneas por página y fijación de barra de zoom flotante.</t>
+      <c r="D16" s="36" t="inlineStr">
+        <is>
+          <t>feat(studio): add TEMIS Media Studio desktop suite for offline whisper transcription, smart screenshot capture and TEMIS package export</t>
+        </is>
+      </c>
+      <c r="E16" s="35" t="inlineStr">
+        <is>
+          <t>🔥 HITO: TEMIS Media Studio Desktop</t>
+        </is>
+      </c>
+      <c r="F16" s="35" t="inlineStr">
+        <is>
+          <t>Sprint 07 - Sep 2026</t>
+        </is>
+      </c>
+      <c r="G16" s="36" t="inlineStr">
+        <is>
+          <t>Suite de escritorio offline para extracción multimedia, transcripción local Whisper y captura de fotogramas clave HD.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>ecc76fb</t>
-        </is>
-      </c>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>2026-08-27 20:27:27 -0600</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="inlineStr">
+      <c r="A17" s="37" t="inlineStr">
+        <is>
+          <t>6d2dc26b</t>
+        </is>
+      </c>
+      <c r="B17" s="40" t="inlineStr">
+        <is>
+          <t>2026-09-24 16:04:46 -0600</t>
+        </is>
+      </c>
+      <c r="C17" s="39" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D17" s="5" t="inlineStr">
-        <is>
-          <t>fix: corrige evaluacion de left y top CSS en render_node para posicionamiento dinámico de nodos y zoom responsivo sin bordes blancos</t>
-        </is>
-      </c>
-      <c r="E17" s="5" t="inlineStr">
-        <is>
-          <t>Canvas / CSS</t>
-        </is>
-      </c>
-      <c r="F17" s="4" t="inlineStr">
-        <is>
-          <t>Sprint 05 - Ago 2026</t>
-        </is>
-      </c>
-      <c r="G17" s="5" t="inlineStr">
-        <is>
-          <t>Cálculo dinámico de dimensiones de zoom responsivo (zoom_width/zoom_height) eliminando márgenes blancos.</t>
+      <c r="D17" s="39" t="inlineStr">
+        <is>
+          <t>fix(upload): remove on_drop overwrite to let reflex default upload_file populate rx.selected_files</t>
+        </is>
+      </c>
+      <c r="E17" s="37" t="inlineStr">
+        <is>
+          <t>Ingesta ZIP / Galería Evidencias</t>
+        </is>
+      </c>
+      <c r="F17" s="40" t="inlineStr">
+        <is>
+          <t>Sprint 07 - Sep 2026</t>
+        </is>
+      </c>
+      <c r="G17" s="39" t="inlineStr">
+        <is>
+          <t>Parser de paquetes .zip de Media Studio, visor reactivo de capturas Base64 y drag-and-drop en web.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="11" t="inlineStr">
-        <is>
-          <t>9e8da71</t>
-        </is>
-      </c>
-      <c r="B18" s="11" t="inlineStr">
-        <is>
-          <t>2026-08-27 20:20:24 -0600</t>
-        </is>
-      </c>
-      <c r="C18" s="27" t="inlineStr">
+      <c r="A18" s="41" t="inlineStr">
+        <is>
+          <t>92be41e7</t>
+        </is>
+      </c>
+      <c r="B18" s="44" t="inlineStr">
+        <is>
+          <t>2026-09-24 15:12:52 -0600</t>
+        </is>
+      </c>
+      <c r="C18" s="43" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D18" s="27" t="inlineStr">
-        <is>
-          <t>fix: mapea correctamente las columnas Id y Shape ID de Lucidchart logrando conectar el 100% de las 640 lineas entre nodos del CSV</t>
-        </is>
-      </c>
-      <c r="E18" s="27" t="inlineStr">
-        <is>
-          <t>Parser Lucidchart</t>
-        </is>
-      </c>
-      <c r="F18" s="11" t="inlineStr">
-        <is>
-          <t>Sprint 05 - Ago 2026</t>
-        </is>
-      </c>
-      <c r="G18" s="27" t="inlineStr">
-        <is>
-          <t>Conexión integral del 100% de las 640 líneas del CSV de Lucidchart cruzando columnas Id y Shape ID.</t>
+      <c r="D18" s="43" t="inlineStr">
+        <is>
+          <t>feat(media): integrate Gemini File API for large audio/video files up to 2GB</t>
+        </is>
+      </c>
+      <c r="E18" s="41" t="inlineStr">
+        <is>
+          <t>IA / Gemini 2.5 / Audio</t>
+        </is>
+      </c>
+      <c r="F18" s="44" t="inlineStr">
+        <is>
+          <t>Sprint 07 - Sep 2026</t>
+        </is>
+      </c>
+      <c r="G18" s="43" t="inlineStr">
+        <is>
+          <t>Ingesta de audios y videos masivos con Gemini File API y extracción incremental de narrativa.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>2000758</t>
-        </is>
-      </c>
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t>2026-08-27 19:55:30 -0600</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="inlineStr">
+      <c r="A19" s="37" t="inlineStr">
+        <is>
+          <t>2d85d5ec</t>
+        </is>
+      </c>
+      <c r="B19" s="40" t="inlineStr">
+        <is>
+          <t>2026-09-24 15:06:46 -0600</t>
+        </is>
+      </c>
+      <c r="C19" s="39" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D19" s="5" t="inlineStr">
-        <is>
-          <t>fix: implementa mapeo de IDs robusto para dibujar 100% de las lineas de Lucidchart y ordenamiento topologico de procesos como en el PDF</t>
-        </is>
-      </c>
-      <c r="E19" s="5" t="inlineStr">
-        <is>
-          <t>Parser / Layout</t>
-        </is>
-      </c>
-      <c r="F19" s="4" t="inlineStr">
-        <is>
-          <t>Sprint 05 - Ago 2026</t>
-        </is>
-      </c>
-      <c r="G19" s="5" t="inlineStr">
-        <is>
-          <t>Algoritmo de ordenamiento topológico por niveles para diagramación fluida idéntica al PDF original.</t>
+      <c r="D19" s="39" t="inlineStr">
+        <is>
+          <t>feat(media): add upload spinner loading state and size tip note</t>
+        </is>
+      </c>
+      <c r="E19" s="37" t="inlineStr">
+        <is>
+          <t>Ingesta ZIP / Galería Evidencias</t>
+        </is>
+      </c>
+      <c r="F19" s="40" t="inlineStr">
+        <is>
+          <t>Sprint 07 - Sep 2026</t>
+        </is>
+      </c>
+      <c r="G19" s="39" t="inlineStr">
+        <is>
+          <t>Parser de paquetes .zip de Media Studio, visor reactivo de capturas Base64 y drag-and-drop en web.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="11" t="inlineStr">
-        <is>
-          <t>b1e0e00</t>
-        </is>
-      </c>
-      <c r="B20" s="11" t="inlineStr">
-        <is>
-          <t>2026-08-27 19:39:48 -0600</t>
-        </is>
-      </c>
-      <c r="C20" s="27" t="inlineStr">
+      <c r="A20" s="41" t="inlineStr">
+        <is>
+          <t>c7175a5e</t>
+        </is>
+      </c>
+      <c r="B20" s="44" t="inlineStr">
+        <is>
+          <t>2026-09-24 14:51:27 -0600</t>
+        </is>
+      </c>
+      <c r="C20" s="43" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D20" s="27" t="inlineStr">
-        <is>
-          <t>feat: agrega controles de reposicionamiento y movimiento directo de nodos en el lienzo</t>
-        </is>
-      </c>
-      <c r="E20" s="27" t="inlineStr">
-        <is>
-          <t>Canvas / Nodos</t>
-        </is>
-      </c>
-      <c r="F20" s="11" t="inlineStr">
-        <is>
-          <t>Sprint 05 - Ago 2026</t>
-        </is>
-      </c>
-      <c r="G20" s="27" t="inlineStr">
-        <is>
-          <t>Pad de botones de movimiento direccional para ajuste fino de casillas en el lienzo.</t>
+      <c r="D20" s="43" t="inlineStr">
+        <is>
+          <t>fix(upload): connect rx.upload_files to on_drop and add selected file process button</t>
+        </is>
+      </c>
+      <c r="E20" s="41" t="inlineStr">
+        <is>
+          <t>Ingesta ZIP / Galería Evidencias</t>
+        </is>
+      </c>
+      <c r="F20" s="44" t="inlineStr">
+        <is>
+          <t>Sprint 07 - Sep 2026</t>
+        </is>
+      </c>
+      <c r="G20" s="43" t="inlineStr">
+        <is>
+          <t>Parser de paquetes .zip de Media Studio, visor reactivo de capturas Base64 y drag-and-drop en web.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>28240c5</t>
-        </is>
-      </c>
-      <c r="B21" s="4" t="inlineStr">
-        <is>
-          <t>2026-08-27 19:35:52 -0600</t>
-        </is>
-      </c>
-      <c r="C21" s="5" t="inlineStr">
+      <c r="A21" s="37" t="inlineStr">
+        <is>
+          <t>5b3d027f</t>
+        </is>
+      </c>
+      <c r="B21" s="40" t="inlineStr">
+        <is>
+          <t>2026-09-24 14:41:38 -0600</t>
+        </is>
+      </c>
+      <c r="C21" s="39" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D21" s="5" t="inlineStr">
-        <is>
-          <t>feat: expande el lienzo de dibujo al 100% de la altura vertical ocupando todo el espacio libre inferior</t>
-        </is>
-      </c>
-      <c r="E21" s="5" t="inlineStr">
-        <is>
-          <t>Canvas / Layout</t>
-        </is>
-      </c>
-      <c r="F21" s="4" t="inlineStr">
-        <is>
-          <t>Sprint 05 - Ago 2026</t>
-        </is>
-      </c>
-      <c r="G21" s="5" t="inlineStr">
-        <is>
-          <t>Optimización de espacio vertical en el lienzo de trabajo ocupando el 100% del viewport.</t>
+      <c r="D21" s="39" t="inlineStr">
+        <is>
+          <t>fix(build): extract document_library_item to top-level typed component to resolve foreach UntypedVarError in Render</t>
+        </is>
+      </c>
+      <c r="E21" s="37" t="inlineStr">
+        <is>
+          <t>Frontend / UI</t>
+        </is>
+      </c>
+      <c r="F21" s="40" t="inlineStr">
+        <is>
+          <t>Sprint 07 - Sep 2026</t>
+        </is>
+      </c>
+      <c r="G21" s="39" t="inlineStr">
+        <is>
+          <t>fix(build): extract document_library_item to top-level typed component to resolve foreach UntypedVarError in Render</t>
         </is>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="11" t="inlineStr">
-        <is>
-          <t>70a72ca</t>
-        </is>
-      </c>
-      <c r="B22" s="11" t="inlineStr">
-        <is>
-          <t>2026-08-27 19:30:57 -0600</t>
-        </is>
-      </c>
-      <c r="C22" s="27" t="inlineStr">
+      <c r="A22" s="41" t="inlineStr">
+        <is>
+          <t>957bfeba</t>
+        </is>
+      </c>
+      <c r="B22" s="44" t="inlineStr">
+        <is>
+          <t>2026-09-24 14:30:28 -0600</t>
+        </is>
+      </c>
+      <c r="C22" s="43" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D22" s="27" t="inlineStr">
-        <is>
-          <t>feat: implementa calculo dinamico de curvas Bézier SVG y etiquetas de bifurcacion para conectores</t>
-        </is>
-      </c>
-      <c r="E22" s="27" t="inlineStr">
-        <is>
-          <t>Canvas / SVG Bézier</t>
-        </is>
-      </c>
-      <c r="F22" s="11" t="inlineStr">
-        <is>
-          <t>Sprint 05 - Ago 2026</t>
-        </is>
-      </c>
-      <c r="G22" s="27" t="inlineStr">
-        <is>
-          <t>Cálculo de trazado M x1 y1 C cx1 cy1, cx2 cy2, x2 y2 para líneas de conexión curvas profesionales con etiquetas de decisión.</t>
+      <c r="D22" s="43" t="inlineStr">
+        <is>
+          <t>feat(media): implement universal audio/video ingestion with mutagen metadata and audit transcript export in docx/txt</t>
+        </is>
+      </c>
+      <c r="E22" s="41" t="inlineStr">
+        <is>
+          <t>Plantilla Maestra Word / Narrativa</t>
+        </is>
+      </c>
+      <c r="F22" s="44" t="inlineStr">
+        <is>
+          <t>Sprint 07 - Sep 2026</t>
+        </is>
+      </c>
+      <c r="G22" s="43" t="inlineStr">
+        <is>
+          <t>Integración del motor de población sobre Plantilla_Maestra_Oficial_Work_Instructions_TEMIS.docx y 4 tablas oficiales.</t>
         </is>
       </c>
     </row>
     <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="4" t="inlineStr">
-        <is>
-          <t>0f6ee7f</t>
-        </is>
-      </c>
-      <c r="B23" s="4" t="inlineStr">
-        <is>
-          <t>2026-08-27 19:19:43 -0600</t>
-        </is>
-      </c>
-      <c r="C23" s="5" t="inlineStr">
+      <c r="A23" s="37" t="inlineStr">
+        <is>
+          <t>3d0d6ded</t>
+        </is>
+      </c>
+      <c r="B23" s="40" t="inlineStr">
+        <is>
+          <t>2026-09-23 17:34:48 -0600</t>
+        </is>
+      </c>
+      <c r="C23" s="39" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D23" s="5" t="inlineStr">
-        <is>
-          <t>feat: remueve barra lateral y encabezado fijo de swimlanes, agrega desplegable de gobernanza y ajusta CSS zoom en lienzo completo</t>
-        </is>
-      </c>
-      <c r="E23" s="5" t="inlineStr">
-        <is>
-          <t>Frontend / Gobernanza</t>
-        </is>
-      </c>
-      <c r="F23" s="4" t="inlineStr">
-        <is>
-          <t>Sprint 05 - Ago 2026</t>
-        </is>
-      </c>
-      <c r="G23" s="5" t="inlineStr">
-        <is>
-          <t>Integración de selector de 7 Fases de Gobernanza en la barra superior.</t>
+      <c r="D23" s="39" t="inlineStr">
+        <is>
+          <t>feat(narrative): implement multi-document incremental ingestion and enrichment pipeline</t>
+        </is>
+      </c>
+      <c r="E23" s="37" t="inlineStr">
+        <is>
+          <t>Plantilla Maestra Word / Narrativa</t>
+        </is>
+      </c>
+      <c r="F23" s="40" t="inlineStr">
+        <is>
+          <t>Sprint 07 - Sep 2026</t>
+        </is>
+      </c>
+      <c r="G23" s="39" t="inlineStr">
+        <is>
+          <t>Integración del motor de población sobre Plantilla_Maestra_Oficial_Work_Instructions_TEMIS.docx y 4 tablas oficiales.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="11" t="inlineStr">
-        <is>
-          <t>9f31c2f</t>
-        </is>
-      </c>
-      <c r="B24" s="11" t="inlineStr">
-        <is>
-          <t>2026-08-27 19:14:39 -0600</t>
-        </is>
-      </c>
-      <c r="C24" s="27" t="inlineStr">
+      <c r="A24" s="41" t="inlineStr">
+        <is>
+          <t>7229b48e</t>
+        </is>
+      </c>
+      <c r="B24" s="44" t="inlineStr">
+        <is>
+          <t>2026-09-23 15:58:38 -0600</t>
+        </is>
+      </c>
+      <c r="C24" s="43" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D24" s="27" t="inlineStr">
-        <is>
-          <t>feat: agrega parser nativo directo deterministico para CSV/JSON de Lucidchart sin intervencion de IA/Gemini</t>
-        </is>
-      </c>
-      <c r="E24" s="27" t="inlineStr">
-        <is>
-          <t>Parser Nativo Core</t>
-        </is>
-      </c>
-      <c r="F24" s="11" t="inlineStr">
-        <is>
-          <t>Sprint 05 - Ago 2026</t>
-        </is>
-      </c>
-      <c r="G24" s="27" t="inlineStr">
-        <is>
-          <t>Primer parser determinista en backend para importación 1-a-1 de Lucidchart sin depender de prompts de IA.</t>
+      <c r="D24" s="43" t="inlineStr">
+        <is>
+          <t>feat(narrative): implement client narrative analysis, citations, dual SIPOC, 4-table Word manuals and dual BPMN generation</t>
+        </is>
+      </c>
+      <c r="E24" s="41" t="inlineStr">
+        <is>
+          <t>Plantilla Maestra Word / Narrativa</t>
+        </is>
+      </c>
+      <c r="F24" s="44" t="inlineStr">
+        <is>
+          <t>Sprint 07 - Sep 2026</t>
+        </is>
+      </c>
+      <c r="G24" s="43" t="inlineStr">
+        <is>
+          <t>Integración del motor de población sobre Plantilla_Maestra_Oficial_Work_Instructions_TEMIS.docx y 4 tablas oficiales.</t>
         </is>
       </c>
     </row>
     <row r="25" ht="20" customHeight="1">
-      <c r="A25" s="4" t="inlineStr">
-        <is>
-          <t>710128e</t>
-        </is>
-      </c>
-      <c r="B25" s="4" t="inlineStr">
-        <is>
-          <t>2026-08-27 19:05:09 -0600</t>
-        </is>
-      </c>
-      <c r="C25" s="5" t="inlineStr">
+      <c r="A25" s="37" t="inlineStr">
+        <is>
+          <t>74e28a73</t>
+        </is>
+      </c>
+      <c r="B25" s="40" t="inlineStr">
+        <is>
+          <t>2026-09-23 15:16:40 -0600</t>
+        </is>
+      </c>
+      <c r="C25" s="39" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D25" s="5" t="inlineStr">
-        <is>
-          <t>fix: configura API_BASE_URL a temis-backend.onrender.com y agrega fallback de lectura para diagramas de PDF WhatsApp</t>
-        </is>
-      </c>
-      <c r="E25" s="5" t="inlineStr">
-        <is>
-          <t>DevOps / Backend</t>
-        </is>
-      </c>
-      <c r="F25" s="4" t="inlineStr">
-        <is>
-          <t>Sprint 05 - Ago 2026</t>
-        </is>
-      </c>
-      <c r="G25" s="5" t="inlineStr">
-        <is>
-          <t>Configuración de variables de entorno de producción para comunicación frontend-backend en Render.</t>
+      <c r="D25" s="39" t="inlineStr">
+        <is>
+          <t>fix(deploy): initialize Reflex state and Starlette lifespan in prod_server for event processor</t>
+        </is>
+      </c>
+      <c r="E25" s="37" t="inlineStr">
+        <is>
+          <t>DevOps / Despliegue Cloud</t>
+        </is>
+      </c>
+      <c r="F25" s="40" t="inlineStr">
+        <is>
+          <t>Sprint 07 - Sep 2026</t>
+        </is>
+      </c>
+      <c r="G25" s="39" t="inlineStr">
+        <is>
+          <t>Optimización de servidor de producción ASGI, configuración de endpoints de upload y resolución de timeouts en Render.</t>
         </is>
       </c>
     </row>
     <row r="26" ht="20" customHeight="1">
-      <c r="A26" s="11" t="inlineStr">
-        <is>
-          <t>ce0b414</t>
-        </is>
-      </c>
-      <c r="B26" s="11" t="inlineStr">
-        <is>
-          <t>2026-08-27 18:53:29 -0600</t>
-        </is>
-      </c>
-      <c r="C26" s="27" t="inlineStr">
+      <c r="A26" s="41" t="inlineStr">
+        <is>
+          <t>158f0ff4</t>
+        </is>
+      </c>
+      <c r="B26" s="44" t="inlineStr">
+        <is>
+          <t>2026-09-23 14:51:23 -0600</t>
+        </is>
+      </c>
+      <c r="C26" s="43" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D26" s="27" t="inlineStr">
-        <is>
-          <t>feat: agrega soporte para importar archivos PDF (procesados con PyPDF2 + Gemini AI) y CSV en el modal de importacion</t>
-        </is>
-      </c>
-      <c r="E26" s="27" t="inlineStr">
-        <is>
-          <t>Parser / PDF IA</t>
-        </is>
-      </c>
-      <c r="F26" s="11" t="inlineStr">
-        <is>
-          <t>Sprint 05 - Ago 2026</t>
-        </is>
-      </c>
-      <c r="G26" s="27" t="inlineStr">
-        <is>
-          <t>Extracción de texto estructurado de PDFs de procesos y diagramación asistida con IA.</t>
+      <c r="D26" s="43" t="inlineStr">
+        <is>
+          <t>feat(deploy): add lightweight ASGI prod_server.py to avoid runtime compile OOM in Render</t>
+        </is>
+      </c>
+      <c r="E26" s="41" t="inlineStr">
+        <is>
+          <t>DevOps / Despliegue Cloud</t>
+        </is>
+      </c>
+      <c r="F26" s="44" t="inlineStr">
+        <is>
+          <t>Sprint 07 - Sep 2026</t>
+        </is>
+      </c>
+      <c r="G26" s="43" t="inlineStr">
+        <is>
+          <t>Optimización de servidor de producción ASGI, configuración de endpoints de upload y resolución de timeouts en Render.</t>
         </is>
       </c>
     </row>
     <row r="27" ht="20" customHeight="1">
-      <c r="A27" s="4" t="inlineStr">
-        <is>
-          <t>39e3995</t>
-        </is>
-      </c>
-      <c r="B27" s="4" t="inlineStr">
-        <is>
-          <t>2026-08-27 18:47:41 -0600</t>
-        </is>
-      </c>
-      <c r="C27" s="5" t="inlineStr">
+      <c r="A27" s="37" t="inlineStr">
+        <is>
+          <t>5af5f0a0</t>
+        </is>
+      </c>
+      <c r="B27" s="40" t="inlineStr">
+        <is>
+          <t>2026-09-23 13:07:44 -0600</t>
+        </is>
+      </c>
+      <c r="C27" s="39" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D27" s="5" t="inlineStr">
-        <is>
-          <t>fix: configura RadixThemesPlugin de forma explicita en rxconfig.py y show_built_with_reflex=False</t>
-        </is>
-      </c>
-      <c r="E27" s="5" t="inlineStr">
-        <is>
-          <t>Frontend / Config</t>
-        </is>
-      </c>
-      <c r="F27" s="4" t="inlineStr">
-        <is>
-          <t>Sprint 05 - Ago 2026</t>
-        </is>
-      </c>
-      <c r="G27" s="5" t="inlineStr">
-        <is>
-          <t>Ajustes de plugins de compilación en Reflex.</t>
+      <c r="D27" s="39" t="inlineStr">
+        <is>
+          <t>fix(deploy): use --single-port with --backend-host 0.0.0.0 --backend-port \ in render.yaml</t>
+        </is>
+      </c>
+      <c r="E27" s="37" t="inlineStr">
+        <is>
+          <t>DevOps / Despliegue Cloud</t>
+        </is>
+      </c>
+      <c r="F27" s="40" t="inlineStr">
+        <is>
+          <t>Sprint 07 - Sep 2026</t>
+        </is>
+      </c>
+      <c r="G27" s="39" t="inlineStr">
+        <is>
+          <t>Optimización de servidor de producción ASGI, configuración de endpoints de upload y resolución de timeouts en Render.</t>
         </is>
       </c>
     </row>
     <row r="28" ht="20" customHeight="1">
-      <c r="A28" s="11" t="inlineStr">
-        <is>
-          <t>7292026</t>
-        </is>
-      </c>
-      <c r="B28" s="11" t="inlineStr">
-        <is>
-          <t>2026-08-27 18:29:24 -0600</t>
-        </is>
-      </c>
-      <c r="C28" s="27" t="inlineStr">
+      <c r="A28" s="41" t="inlineStr">
+        <is>
+          <t>ff604053</t>
+        </is>
+      </c>
+      <c r="B28" s="44" t="inlineStr">
+        <is>
+          <t>2026-09-23 12:44:30 -0600</t>
+        </is>
+      </c>
+      <c r="C28" s="43" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D28" s="27" t="inlineStr">
-        <is>
-          <t>fix: corrige evaluacion de f-strings en transform CSS y badges para evitar error de hidratacion React en cliente</t>
-        </is>
-      </c>
-      <c r="E28" s="27" t="inlineStr">
-        <is>
-          <t>Frontend / React SSR</t>
-        </is>
-      </c>
-      <c r="F28" s="11" t="inlineStr">
-        <is>
-          <t>Sprint 05 - Ago 2026</t>
-        </is>
-      </c>
-      <c r="G28" s="27" t="inlineStr">
-        <is>
-          <t>Resolución de discrepancias de renderizado entre SSR y cliente en React.</t>
+      <c r="D28" s="43" t="inlineStr">
+        <is>
+          <t>fix(temis): resolve Radix HStack integer spacing and padding type constraints</t>
+        </is>
+      </c>
+      <c r="E28" s="41" t="inlineStr">
+        <is>
+          <t>Frontend / UI</t>
+        </is>
+      </c>
+      <c r="F28" s="44" t="inlineStr">
+        <is>
+          <t>Sprint 07 - Sep 2026</t>
+        </is>
+      </c>
+      <c r="G28" s="43" t="inlineStr">
+        <is>
+          <t>fix(temis): resolve Radix HStack integer spacing and padding type constraints</t>
         </is>
       </c>
     </row>
     <row r="29" ht="20" customHeight="1">
-      <c r="A29" s="4" t="inlineStr">
-        <is>
-          <t>b833b55</t>
-        </is>
-      </c>
-      <c r="B29" s="4" t="inlineStr">
-        <is>
-          <t>2026-08-27 18:09:38 -0600</t>
-        </is>
-      </c>
-      <c r="C29" s="5" t="inlineStr">
+      <c r="A29" s="37" t="inlineStr">
+        <is>
+          <t>fa12f8df</t>
+        </is>
+      </c>
+      <c r="B29" s="40" t="inlineStr">
+        <is>
+          <t>2026-09-23 12:34:14 -0600</t>
+        </is>
+      </c>
+      <c r="C29" s="39" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D29" s="5" t="inlineStr">
-        <is>
-          <t>fix: reemplaza etiqueta de icono no valida upload_cloud por cloud_upload</t>
-        </is>
-      </c>
-      <c r="E29" s="5" t="inlineStr">
+      <c r="D29" s="39" t="inlineStr">
+        <is>
+          <t>feat(temis): implement verification improvements H01 to H06</t>
+        </is>
+      </c>
+      <c r="E29" s="37" t="inlineStr">
         <is>
           <t>Frontend / UI</t>
         </is>
       </c>
-      <c r="F29" s="4" t="inlineStr">
-        <is>
-          <t>Sprint 05 - Ago 2026</t>
-        </is>
-      </c>
-      <c r="G29" s="5" t="inlineStr">
-        <is>
-          <t>Corrección de etiquetas de iconos Lucide.</t>
+      <c r="F29" s="40" t="inlineStr">
+        <is>
+          <t>Sprint 07 - Sep 2026</t>
+        </is>
+      </c>
+      <c r="G29" s="39" t="inlineStr">
+        <is>
+          <t>feat(temis): implement verification improvements H01 to H06</t>
         </is>
       </c>
     </row>
     <row r="30" ht="20" customHeight="1">
-      <c r="A30" s="11" t="inlineStr">
-        <is>
-          <t>60c915e</t>
-        </is>
-      </c>
-      <c r="B30" s="11" t="inlineStr">
-        <is>
-          <t>2026-08-27 18:04:07 -0600</t>
-        </is>
-      </c>
-      <c r="C30" s="27" t="inlineStr">
+      <c r="A30" s="41" t="inlineStr">
+        <is>
+          <t>1d3f1819</t>
+        </is>
+      </c>
+      <c r="B30" s="44" t="inlineStr">
+        <is>
+          <t>2026-09-23 11:52:59 -0600</t>
+        </is>
+      </c>
+      <c r="C30" s="43" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D30" s="27" t="inlineStr">
-        <is>
-          <t>feat: agrega Zoom interactivo al lienzo (transform scale), barra flotante de controles y zoom con rueda de mouse</t>
-        </is>
-      </c>
-      <c r="E30" s="27" t="inlineStr">
-        <is>
-          <t>Canvas / Zoom</t>
-        </is>
-      </c>
-      <c r="F30" s="11" t="inlineStr">
-        <is>
-          <t>Sprint 05 - Ago 2026</t>
-        </is>
-      </c>
-      <c r="G30" s="27" t="inlineStr">
-        <is>
-          <t>Motor de zoom interactivo con soporte para rueda del ratón y controles en pantalla.</t>
+      <c r="D30" s="43" t="inlineStr">
+        <is>
+          <t>feat(temis): implement formal verification audit findings (F01-F06) for phase gates, selection isolation, AI audit, and backlog modal</t>
+        </is>
+      </c>
+      <c r="E30" s="41" t="inlineStr">
+        <is>
+          <t>Frontend / UI</t>
+        </is>
+      </c>
+      <c r="F30" s="44" t="inlineStr">
+        <is>
+          <t>Sprint 07 - Sep 2026</t>
+        </is>
+      </c>
+      <c r="G30" s="43" t="inlineStr">
+        <is>
+          <t>feat(temis): implement formal verification audit findings (F01-F06) for phase gates, selection isolation, AI audit, and backlog modal</t>
         </is>
       </c>
     </row>
     <row r="31" ht="20" customHeight="1">
-      <c r="A31" s="4" t="inlineStr">
-        <is>
-          <t>6137ed2</t>
-        </is>
-      </c>
-      <c r="B31" s="4" t="inlineStr">
-        <is>
-          <t>2026-08-27 18:01:14 -0600</t>
-        </is>
-      </c>
-      <c r="C31" s="5" t="inlineStr">
+      <c r="A31" s="37" t="inlineStr">
+        <is>
+          <t>603d7945</t>
+        </is>
+      </c>
+      <c r="B31" s="40" t="inlineStr">
+        <is>
+          <t>2026-09-23 10:52:17 -0600</t>
+        </is>
+      </c>
+      <c r="C31" s="39" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D31" s="5" t="inlineStr">
-        <is>
-          <t>fix: reemplaza rx.upload incrustado por modal de importación limpio y configura DATABASE_URL en rxconfig.py</t>
-        </is>
-      </c>
-      <c r="E31" s="5" t="inlineStr">
-        <is>
-          <t>Frontend / DB</t>
-        </is>
-      </c>
-      <c r="F31" s="4" t="inlineStr">
-        <is>
-          <t>Sprint 05 - Ago 2026</t>
-        </is>
-      </c>
-      <c r="G31" s="5" t="inlineStr">
-        <is>
-          <t>Modal flotante de importación de archivos y configuración de PostgreSQL.</t>
+      <c r="D31" s="39" t="inlineStr">
+        <is>
+          <t>fix(render): pre-compile frontend during build phase with reflex export --no-zip to prevent port scan timeout on startup</t>
+        </is>
+      </c>
+      <c r="E31" s="37" t="inlineStr">
+        <is>
+          <t>Ingesta ZIP / Galería Evidencias</t>
+        </is>
+      </c>
+      <c r="F31" s="40" t="inlineStr">
+        <is>
+          <t>Sprint 07 - Sep 2026</t>
+        </is>
+      </c>
+      <c r="G31" s="39" t="inlineStr">
+        <is>
+          <t>Parser de paquetes .zip de Media Studio, visor reactivo de capturas Base64 y drag-and-drop en web.</t>
         </is>
       </c>
     </row>
     <row r="32" ht="20" customHeight="1">
-      <c r="A32" s="11" t="inlineStr">
-        <is>
-          <t>ca5d399</t>
-        </is>
-      </c>
-      <c r="B32" s="11" t="inlineStr">
-        <is>
-          <t>2026-08-27 17:49:52 -0600</t>
-        </is>
-      </c>
-      <c r="C32" s="27" t="inlineStr">
+      <c r="A32" s="41" t="inlineStr">
+        <is>
+          <t>7a70433a</t>
+        </is>
+      </c>
+      <c r="B32" s="44" t="inlineStr">
+        <is>
+          <t>2026-09-23 10:08:17 -0600</t>
+        </is>
+      </c>
+      <c r="C32" s="43" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D32" s="27" t="inlineStr">
-        <is>
-          <t>feat: agrega boton Importar en UI, conectores con curvas Bézier estilizadas y confirmacion de importacion de proyectos</t>
-        </is>
-      </c>
-      <c r="E32" s="27" t="inlineStr">
-        <is>
-          <t>Frontend / Conectores</t>
-        </is>
-      </c>
-      <c r="F32" s="11" t="inlineStr">
-        <is>
-          <t>Sprint 05 - Ago 2026</t>
-        </is>
-      </c>
-      <c r="G32" s="27" t="inlineStr">
-        <is>
-          <t>Botón de importación directa y renderizado de conectores estilizados.</t>
+      <c r="D32" s="43" t="inlineStr">
+        <is>
+          <t>fix(temis): resolve BPMN multi-page selection desync P0, non-destructive SIPOC flow generation P0, accessible 44px nudge controls P1, AI proposal review modal P1, and Excel MIME export P2</t>
+        </is>
+      </c>
+      <c r="E32" s="41" t="inlineStr">
+        <is>
+          <t>SIPOC / Excel Oficial</t>
+        </is>
+      </c>
+      <c r="F32" s="44" t="inlineStr">
+        <is>
+          <t>Sprint 07 - Sep 2026</t>
+        </is>
+      </c>
+      <c r="G32" s="43" t="inlineStr">
+        <is>
+          <t>Estandarización del exportador Excel idéntico a Plantilla Matriz Sipoc.xlsx con 11 columnas y Century Gothic.</t>
         </is>
       </c>
     </row>
     <row r="33" ht="20" customHeight="1">
-      <c r="A33" s="4" t="inlineStr">
-        <is>
-          <t>584a7f7</t>
-        </is>
-      </c>
-      <c r="B33" s="4" t="inlineStr">
-        <is>
-          <t>2026-08-27 17:47:13 -0600</t>
-        </is>
-      </c>
-      <c r="C33" s="5" t="inlineStr">
+      <c r="A33" s="37" t="inlineStr">
+        <is>
+          <t>23a039ac</t>
+        </is>
+      </c>
+      <c r="B33" s="40" t="inlineStr">
+        <is>
+          <t>2026-09-23 09:50:35 -0600</t>
+        </is>
+      </c>
+      <c r="C33" s="39" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D33" s="5" t="inlineStr">
-        <is>
-          <t>feat: agrega endpoints y funciones para exportar e importar proyectos completos (.temis.json) en backend y frontend</t>
-        </is>
-      </c>
-      <c r="E33" s="5" t="inlineStr">
-        <is>
-          <t>Backend / Paquetes</t>
-        </is>
-      </c>
-      <c r="F33" s="4" t="inlineStr">
-        <is>
-          <t>Sprint 05 - Ago 2026</t>
-        </is>
-      </c>
-      <c r="G33" s="5" t="inlineStr">
-        <is>
-          <t>Diseño del formato de paquete estándar .temis.json con nodos, aristas, fases y metadatos.</t>
+      <c r="D33" s="39" t="inlineStr">
+        <is>
+          <t>feat(temis): resolve audit findings - P0 user recovery, canonical SP consistency, Executive Light Slate theme (WCAG 2.2 AA), and BPMN/SIPOC usability</t>
+        </is>
+      </c>
+      <c r="E33" s="37" t="inlineStr">
+        <is>
+          <t>Frontend / UI</t>
+        </is>
+      </c>
+      <c r="F33" s="40" t="inlineStr">
+        <is>
+          <t>Sprint 07 - Sep 2026</t>
+        </is>
+      </c>
+      <c r="G33" s="39" t="inlineStr">
+        <is>
+          <t>feat(temis): resolve audit findings - P0 user recovery, canonical SP consistency, Executive Light Slate theme (WCAG 2.2 AA), and BPMN/SIPOC usability</t>
         </is>
       </c>
     </row>
     <row r="34" ht="20" customHeight="1">
-      <c r="A34" s="11" t="inlineStr">
-        <is>
-          <t>e5f1686</t>
-        </is>
-      </c>
-      <c r="B34" s="11" t="inlineStr">
-        <is>
-          <t>2026-08-27 17:44:50 -0600</t>
-        </is>
-      </c>
-      <c r="C34" s="27" t="inlineStr">
+      <c r="A34" s="41" t="inlineStr">
+        <is>
+          <t>2dd8d83a</t>
+        </is>
+      </c>
+      <c r="B34" s="44" t="inlineStr">
+        <is>
+          <t>2026-09-22 22:42:55 -0600</t>
+        </is>
+      </c>
+      <c r="C34" s="43" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D34" s="27" t="inlineStr">
-        <is>
-          <t>feat: agrega menu de exportación a JSON (compatible con Lucidchart) y CSV de datos de figuras</t>
-        </is>
-      </c>
-      <c r="E34" s="27" t="inlineStr">
-        <is>
-          <t>Exportación</t>
-        </is>
-      </c>
-      <c r="F34" s="11" t="inlineStr">
-        <is>
-          <t>Sprint 05 - Ago 2026</t>
-        </is>
-      </c>
-      <c r="G34" s="27" t="inlineStr">
-        <is>
-          <t>Exportadores a formato JSON estándar y CSV compatible con suites de diagramación.</t>
+      <c r="D34" s="43" t="inlineStr">
+        <is>
+          <t>fix(auth): fix login card z-index stacking and pointer-events layering issue</t>
+        </is>
+      </c>
+      <c r="E34" s="41" t="inlineStr">
+        <is>
+          <t>Frontend / UI</t>
+        </is>
+      </c>
+      <c r="F34" s="44" t="inlineStr">
+        <is>
+          <t>Sprint 07 - Sep 2026</t>
+        </is>
+      </c>
+      <c r="G34" s="43" t="inlineStr">
+        <is>
+          <t>fix(auth): fix login card z-index stacking and pointer-events layering issue</t>
         </is>
       </c>
     </row>
     <row r="35" ht="20" customHeight="1">
-      <c r="A35" s="4" t="inlineStr">
-        <is>
-          <t>22a8bf2</t>
-        </is>
-      </c>
-      <c r="B35" s="4" t="inlineStr">
-        <is>
-          <t>2026-08-27 17:40:51 -0600</t>
-        </is>
-      </c>
-      <c r="C35" s="5" t="inlineStr">
+      <c r="A35" s="37" t="inlineStr">
+        <is>
+          <t>9e917f18</t>
+        </is>
+      </c>
+      <c r="B35" s="40" t="inlineStr">
+        <is>
+          <t>2026-09-22 22:29:27 -0600</t>
+        </is>
+      </c>
+      <c r="C35" s="39" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D35" s="5" t="inlineStr">
-        <is>
-          <t>fix: oculta el distintivo 'Built with Reflex' con style.css personalizado</t>
-        </is>
-      </c>
-      <c r="E35" s="5" t="inlineStr">
-        <is>
-          <t>Frontend / Branding</t>
-        </is>
-      </c>
-      <c r="F35" s="4" t="inlineStr">
-        <is>
-          <t>Sprint 05 - Ago 2026</t>
-        </is>
-      </c>
-      <c r="G35" s="5" t="inlineStr">
-        <is>
-          <t>Personalización de estilos CSS corporativos.</t>
+      <c r="D35" s="39" t="inlineStr">
+        <is>
+          <t>feat(ui): complete executive dark mode overhaul across all views and canvas</t>
+        </is>
+      </c>
+      <c r="E35" s="37" t="inlineStr">
+        <is>
+          <t>Frontend / UI</t>
+        </is>
+      </c>
+      <c r="F35" s="40" t="inlineStr">
+        <is>
+          <t>Sprint 07 - Sep 2026</t>
+        </is>
+      </c>
+      <c r="G35" s="39" t="inlineStr">
+        <is>
+          <t>feat(ui): complete executive dark mode overhaul across all views and canvas</t>
         </is>
       </c>
     </row>
     <row r="36" ht="20" customHeight="1">
-      <c r="A36" s="11" t="inlineStr">
-        <is>
-          <t>cef518a</t>
-        </is>
-      </c>
-      <c r="B36" s="11" t="inlineStr">
-        <is>
-          <t>2026-08-27 17:31:33 -0600</t>
-        </is>
-      </c>
-      <c r="C36" s="27" t="inlineStr">
+      <c r="A36" s="41" t="inlineStr">
+        <is>
+          <t>3b91534d</t>
+        </is>
+      </c>
+      <c r="B36" s="44" t="inlineStr">
+        <is>
+          <t>2026-09-22 21:58:44 -0600</t>
+        </is>
+      </c>
+      <c r="C36" s="43" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D36" s="27" t="inlineStr">
-        <is>
-          <t>feat: agrega modal de edicion de propiedades de nodos (texto, sistema, canal, numero de actividad)</t>
-        </is>
-      </c>
-      <c r="E36" s="27" t="inlineStr">
-        <is>
-          <t>Canvas / Modal Edición</t>
-        </is>
-      </c>
-      <c r="F36" s="11" t="inlineStr">
-        <is>
-          <t>Sprint 05 - Ago 2026</t>
-        </is>
-      </c>
-      <c r="G36" s="27" t="inlineStr">
-        <is>
-          <t>Primer modal de edición de propiedades de casilla.</t>
+      <c r="D36" s="43" t="inlineStr">
+        <is>
+          <t>fix(deploy): resolve FlowState export attribute error and normalize Lucide icon tags</t>
+        </is>
+      </c>
+      <c r="E36" s="41" t="inlineStr">
+        <is>
+          <t>SIPOC / Excel Oficial</t>
+        </is>
+      </c>
+      <c r="F36" s="44" t="inlineStr">
+        <is>
+          <t>Sprint 07 - Sep 2026</t>
+        </is>
+      </c>
+      <c r="G36" s="43" t="inlineStr">
+        <is>
+          <t>Estandarización del exportador Excel idéntico a Plantilla Matriz Sipoc.xlsx con 11 columnas y Century Gothic.</t>
         </is>
       </c>
     </row>
     <row r="37" ht="20" customHeight="1">
-      <c r="A37" s="4" t="inlineStr">
-        <is>
-          <t>38bd2e0</t>
-        </is>
-      </c>
-      <c r="B37" s="4" t="inlineStr">
-        <is>
-          <t>2026-08-27 17:19:59 -0600</t>
-        </is>
-      </c>
-      <c r="C37" s="5" t="inlineStr">
+      <c r="A37" s="37" t="inlineStr">
+        <is>
+          <t>94572889</t>
+        </is>
+      </c>
+      <c r="B37" s="40" t="inlineStr">
+        <is>
+          <t>2026-09-22 21:48:22 -0600</t>
+        </is>
+      </c>
+      <c r="C37" s="39" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D37" s="5" t="inlineStr">
-        <is>
-          <t>fix: reemplaza color_scheme emerald por green en rx.button para compatibilidad con Radix UI</t>
-        </is>
-      </c>
-      <c r="E37" s="5" t="inlineStr">
+      <c r="D37" s="39" t="inlineStr">
+        <is>
+          <t>feat(ui): complete executive visual redesign with slate contrast, 0% emojis, elevated cards and high-contrast typography</t>
+        </is>
+      </c>
+      <c r="E37" s="37" t="inlineStr">
         <is>
           <t>Frontend / UI</t>
         </is>
       </c>
-      <c r="F37" s="4" t="inlineStr">
-        <is>
-          <t>Sprint 05 - Ago 2026</t>
-        </is>
-      </c>
-      <c r="G37" s="5" t="inlineStr">
-        <is>
-          <t>Ajuste de paleta de colores Radix Themes.</t>
+      <c r="F37" s="40" t="inlineStr">
+        <is>
+          <t>Sprint 07 - Sep 2026</t>
+        </is>
+      </c>
+      <c r="G37" s="39" t="inlineStr">
+        <is>
+          <t>feat(ui): complete executive visual redesign with slate contrast, 0% emojis, elevated cards and high-contrast typography</t>
         </is>
       </c>
     </row>
     <row r="38" ht="20" customHeight="1">
-      <c r="A38" s="11" t="inlineStr">
-        <is>
-          <t>4f39a18</t>
-        </is>
-      </c>
-      <c r="B38" s="11" t="inlineStr">
-        <is>
-          <t>2026-08-27 17:15:28 -0600</t>
-        </is>
-      </c>
-      <c r="C38" s="27" t="inlineStr">
+      <c r="A38" s="41" t="inlineStr">
+        <is>
+          <t>a90ae9cf</t>
+        </is>
+      </c>
+      <c r="B38" s="44" t="inlineStr">
+        <is>
+          <t>2026-09-22 21:30:33 -0600</t>
+        </is>
+      </c>
+      <c r="C38" s="43" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D38" s="27" t="inlineStr">
-        <is>
-          <t>feat: agrega boton guardar diagrama en PostgreSQL, duplicar nodo y mejoras UI/UX</t>
-        </is>
-      </c>
-      <c r="E38" s="27" t="inlineStr">
-        <is>
-          <t>Backend / DB Sync</t>
-        </is>
-      </c>
-      <c r="F38" s="11" t="inlineStr">
-        <is>
-          <t>Sprint 05 - Ago 2026</t>
-        </is>
-      </c>
-      <c r="G38" s="27" t="inlineStr">
-        <is>
-          <t>Integración de guardado de proyectos en base de datos PostgreSQL y duplicación rápida de nodos.</t>
+      <c r="D38" s="43" t="inlineStr">
+        <is>
+          <t>feat(temis): add auto-save heartbeat, executive charter print/PDF export, floating toast alerts, and audit score delta</t>
+        </is>
+      </c>
+      <c r="E38" s="41" t="inlineStr">
+        <is>
+          <t>SIPOC / Excel Oficial</t>
+        </is>
+      </c>
+      <c r="F38" s="44" t="inlineStr">
+        <is>
+          <t>Sprint 07 - Sep 2026</t>
+        </is>
+      </c>
+      <c r="G38" s="43" t="inlineStr">
+        <is>
+          <t>Estandarización del exportador Excel idéntico a Plantilla Matriz Sipoc.xlsx con 11 columnas y Century Gothic.</t>
         </is>
       </c>
     </row>
     <row r="39" ht="20" customHeight="1">
-      <c r="A39" s="4" t="inlineStr">
-        <is>
-          <t>dafd346</t>
-        </is>
-      </c>
-      <c r="B39" s="4" t="inlineStr">
-        <is>
-          <t>2026-08-27 17:02:10 -0600</t>
-        </is>
-      </c>
-      <c r="C39" s="5" t="inlineStr">
+      <c r="A39" s="37" t="inlineStr">
+        <is>
+          <t>a1a70ae0</t>
+        </is>
+      </c>
+      <c r="B39" s="40" t="inlineStr">
+        <is>
+          <t>2026-09-22 21:17:22 -0600</t>
+        </is>
+      </c>
+      <c r="C39" s="39" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D39" s="5" t="inlineStr">
-        <is>
-          <t>fix: agrega temis_web/__init__.py exponiendo app para granian worker y corrige nombres de iconos</t>
-        </is>
-      </c>
-      <c r="E39" s="5" t="inlineStr">
-        <is>
-          <t>DevOps / Worker</t>
-        </is>
-      </c>
-      <c r="F39" s="4" t="inlineStr">
-        <is>
-          <t>Sprint 05 - Ago 2026</t>
-        </is>
-      </c>
-      <c r="G39" s="5" t="inlineStr">
-        <is>
-          <t>Configuración de punto de entrada ASGI para worker Granian en Render.</t>
+      <c r="D39" s="39" t="inlineStr">
+        <is>
+          <t>fix(temis): add responsive table containers and toolbar wrapping to SIPOC and Work Plan views</t>
+        </is>
+      </c>
+      <c r="E39" s="37" t="inlineStr">
+        <is>
+          <t>Frontend / UI</t>
+        </is>
+      </c>
+      <c r="F39" s="40" t="inlineStr">
+        <is>
+          <t>Sprint 07 - Sep 2026</t>
+        </is>
+      </c>
+      <c r="G39" s="39" t="inlineStr">
+        <is>
+          <t>fix(temis): add responsive table containers and toolbar wrapping to SIPOC and Work Plan views</t>
         </is>
       </c>
     </row>
     <row r="40" ht="20" customHeight="1">
-      <c r="A40" s="11" t="inlineStr">
-        <is>
-          <t>9235c58</t>
-        </is>
-      </c>
-      <c r="B40" s="11" t="inlineStr">
-        <is>
-          <t>2026-08-27 16:54:56 -0600</t>
-        </is>
-      </c>
-      <c r="C40" s="27" t="inlineStr">
+      <c r="A40" s="41" t="inlineStr">
+        <is>
+          <t>c4b05b5c</t>
+        </is>
+      </c>
+      <c r="B40" s="44" t="inlineStr">
+        <is>
+          <t>2026-09-22 21:13:41 -0600</t>
+        </is>
+      </c>
+      <c r="C40" s="43" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D40" s="27" t="inlineStr">
-        <is>
-          <t>fix: reemplaza rx.concat por f-string en posicionamiento de nodos</t>
-        </is>
-      </c>
-      <c r="E40" s="27" t="inlineStr">
-        <is>
-          <t>Frontend / React</t>
-        </is>
-      </c>
-      <c r="F40" s="11" t="inlineStr">
-        <is>
-          <t>Sprint 05 - Ago 2026</t>
-        </is>
-      </c>
-      <c r="G40" s="27" t="inlineStr">
-        <is>
-          <t>Optimización de sintaxis reactiva para estilos de nodos.</t>
+      <c r="D40" s="43" t="inlineStr">
+        <is>
+          <t>fix(temis): implement full UX/UI audit recommendations - responsive reflow, clean semantics, sprint sync, and zero emojis</t>
+        </is>
+      </c>
+      <c r="E40" s="41" t="inlineStr">
+        <is>
+          <t>Frontend / UI</t>
+        </is>
+      </c>
+      <c r="F40" s="44" t="inlineStr">
+        <is>
+          <t>Sprint 07 - Sep 2026</t>
+        </is>
+      </c>
+      <c r="G40" s="43" t="inlineStr">
+        <is>
+          <t>fix(temis): implement full UX/UI audit recommendations - responsive reflow, clean semantics, sprint sync, and zero emojis</t>
         </is>
       </c>
     </row>
     <row r="41" ht="20" customHeight="1">
-      <c r="A41" s="4" t="inlineStr">
-        <is>
-          <t>4c6afff</t>
-        </is>
-      </c>
-      <c r="B41" s="4" t="inlineStr">
-        <is>
-          <t>2026-08-27 16:50:40 -0600</t>
-        </is>
-      </c>
-      <c r="C41" s="5" t="inlineStr">
+      <c r="A41" s="37" t="inlineStr">
+        <is>
+          <t>5e1cc184</t>
+        </is>
+      </c>
+      <c r="B41" s="40" t="inlineStr">
+        <is>
+          <t>2026-09-22 20:38:56 -0600</t>
+        </is>
+      </c>
+      <c r="C41" s="39" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D41" s="5" t="inlineStr">
-        <is>
-          <t>fix: reemplaza if/elif por rx.match en render_node para renderizado reactivo de nodos</t>
-        </is>
-      </c>
-      <c r="E41" s="5" t="inlineStr">
-        <is>
-          <t>Frontend / React</t>
-        </is>
-      </c>
-      <c r="F41" s="4" t="inlineStr">
-        <is>
-          <t>Sprint 05 - Ago 2026</t>
-        </is>
-      </c>
-      <c r="G41" s="5" t="inlineStr">
-        <is>
-          <t>Uso de rx.match para renderizado reactivo según tipo de figura (BPMN/Canales/Sistemas).</t>
+      <c r="D41" s="39" t="inlineStr">
+        <is>
+          <t>fix(temis): resolve Reflex Var type in user table and standardize Lucide circle-check icon</t>
+        </is>
+      </c>
+      <c r="E41" s="37" t="inlineStr">
+        <is>
+          <t>Frontend / UI</t>
+        </is>
+      </c>
+      <c r="F41" s="40" t="inlineStr">
+        <is>
+          <t>Sprint 07 - Sep 2026</t>
+        </is>
+      </c>
+      <c r="G41" s="39" t="inlineStr">
+        <is>
+          <t>fix(temis): resolve Reflex Var type in user table and standardize Lucide circle-check icon</t>
         </is>
       </c>
     </row>
     <row r="42" ht="20" customHeight="1">
-      <c r="A42" s="11" t="inlineStr">
-        <is>
-          <t>c067df3</t>
-        </is>
-      </c>
-      <c r="B42" s="11" t="inlineStr">
-        <is>
-          <t>2026-08-27 16:44:58 -0600</t>
-        </is>
-      </c>
-      <c r="C42" s="27" t="inlineStr">
+      <c r="A42" s="41" t="inlineStr">
+        <is>
+          <t>1f29dea3</t>
+        </is>
+      </c>
+      <c r="B42" s="44" t="inlineStr">
+        <is>
+          <t>2026-09-22 19:21:19 -0600</t>
+        </is>
+      </c>
+      <c r="C42" s="43" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D42" s="27" t="inlineStr">
-        <is>
-          <t>fix: reemplaza rx.svg con rx.el.svg, corrige nombres de iconos lucide y actualiza a Python 3.11 en Render</t>
-        </is>
-      </c>
-      <c r="E42" s="27" t="inlineStr">
-        <is>
-          <t>DevOps / Python 3.11</t>
-        </is>
-      </c>
-      <c r="F42" s="11" t="inlineStr">
-        <is>
-          <t>Sprint 05 - Ago 2026</t>
-        </is>
-      </c>
-      <c r="G42" s="27" t="inlineStr">
-        <is>
-          <t>Actualización a Python 3.11 y elementos SVG estándar.</t>
+      <c r="D42" s="43" t="inlineStr">
+        <is>
+          <t>feat(temis): add project deletion with confirmation modal and project access assignment per user in user management</t>
+        </is>
+      </c>
+      <c r="E42" s="41" t="inlineStr">
+        <is>
+          <t>Frontend / UI</t>
+        </is>
+      </c>
+      <c r="F42" s="44" t="inlineStr">
+        <is>
+          <t>Sprint 07 - Sep 2026</t>
+        </is>
+      </c>
+      <c r="G42" s="43" t="inlineStr">
+        <is>
+          <t>feat(temis): add project deletion with confirmation modal and project access assignment per user in user management</t>
         </is>
       </c>
     </row>
     <row r="43" ht="20" customHeight="1">
-      <c r="A43" s="4" t="inlineStr">
-        <is>
-          <t>7c255af</t>
-        </is>
-      </c>
-      <c r="B43" s="4" t="inlineStr">
-        <is>
-          <t>2026-08-27 16:37:51 -0600</t>
-        </is>
-      </c>
-      <c r="C43" s="5" t="inlineStr">
+      <c r="A43" s="37" t="inlineStr">
+        <is>
+          <t>a5e507a4</t>
+        </is>
+      </c>
+      <c r="B43" s="40" t="inlineStr">
+        <is>
+          <t>2026-09-22 18:57:27 -0600</t>
+        </is>
+      </c>
+      <c r="C43" s="39" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D43" s="5" t="inlineStr">
-        <is>
-          <t>fix: agrega metodo set_ai_prompt_text explícito en FlowState para solucionar AttributeError en Render</t>
-        </is>
-      </c>
-      <c r="E43" s="5" t="inlineStr">
-        <is>
-          <t>Frontend / State</t>
-        </is>
-      </c>
-      <c r="F43" s="4" t="inlineStr">
-        <is>
-          <t>Sprint 05 - Ago 2026</t>
-        </is>
-      </c>
-      <c r="G43" s="5" t="inlineStr">
-        <is>
-          <t>Manejador explícito de prompt de IA en estado.</t>
+      <c r="D43" s="39" t="inlineStr">
+        <is>
+          <t>style(temis): complete 100% emoji-free UI and standard typographic strings across all views</t>
+        </is>
+      </c>
+      <c r="E43" s="37" t="inlineStr">
+        <is>
+          <t>Frontend / UI</t>
+        </is>
+      </c>
+      <c r="F43" s="40" t="inlineStr">
+        <is>
+          <t>Sprint 07 - Sep 2026</t>
+        </is>
+      </c>
+      <c r="G43" s="39" t="inlineStr">
+        <is>
+          <t>style(temis): complete 100% emoji-free UI and standard typographic strings across all views</t>
         </is>
       </c>
     </row>
     <row r="44" ht="20" customHeight="1">
-      <c r="A44" s="11" t="inlineStr">
-        <is>
-          <t>66908f2</t>
-        </is>
-      </c>
-      <c r="B44" s="11" t="inlineStr">
-        <is>
-          <t>2026-08-27 16:33:55 -0600</t>
-        </is>
-      </c>
-      <c r="C44" s="27" t="inlineStr">
+      <c r="A44" s="41" t="inlineStr">
+        <is>
+          <t>35787df4</t>
+        </is>
+      </c>
+      <c r="B44" s="44" t="inlineStr">
+        <is>
+          <t>2026-09-22 18:52:10 -0600</t>
+        </is>
+      </c>
+      <c r="C44" s="43" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D44" s="27" t="inlineStr">
-        <is>
-          <t>fix: agrega reflex a requirements.txt para corregir build de Render</t>
-        </is>
-      </c>
-      <c r="E44" s="27" t="inlineStr">
-        <is>
-          <t>DevOps / Requirements</t>
-        </is>
-      </c>
-      <c r="F44" s="11" t="inlineStr">
-        <is>
-          <t>Sprint 05 - Ago 2026</t>
-        </is>
-      </c>
-      <c r="G44" s="27" t="inlineStr">
-        <is>
-          <t>Inclusión de dependencia de Reflex en manifiesto.</t>
+      <c r="D44" s="43" t="inlineStr">
+        <is>
+          <t>feat(temis): add executive attention banner in hub and 4-step onboarding roadmap in project charter</t>
+        </is>
+      </c>
+      <c r="E44" s="41" t="inlineStr">
+        <is>
+          <t>Frontend / UI</t>
+        </is>
+      </c>
+      <c r="F44" s="44" t="inlineStr">
+        <is>
+          <t>Sprint 07 - Sep 2026</t>
+        </is>
+      </c>
+      <c r="G44" s="43" t="inlineStr">
+        <is>
+          <t>feat(temis): add executive attention banner in hub and 4-step onboarding roadmap in project charter</t>
         </is>
       </c>
     </row>
     <row r="45" ht="20" customHeight="1">
-      <c r="A45" s="4" t="inlineStr">
-        <is>
-          <t>251c6e5</t>
-        </is>
-      </c>
-      <c r="B45" s="4" t="inlineStr">
-        <is>
-          <t>2026-08-27 16:26:37 -0600</t>
-        </is>
-      </c>
-      <c r="C45" s="5" t="inlineStr">
+      <c r="A45" s="37" t="inlineStr">
+        <is>
+          <t>119cb5a5</t>
+        </is>
+      </c>
+      <c r="B45" s="40" t="inlineStr">
+        <is>
+          <t>2026-09-22 18:46:47 -0600</t>
+        </is>
+      </c>
+      <c r="C45" s="39" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D45" s="5" t="inlineStr">
-        <is>
-          <t>fix: cambia property url a host en render.yaml para Render Blueprint</t>
-        </is>
-      </c>
-      <c r="E45" s="5" t="inlineStr">
-        <is>
-          <t>DevOps / Render</t>
-        </is>
-      </c>
-      <c r="F45" s="4" t="inlineStr">
-        <is>
-          <t>Sprint 05 - Ago 2026</t>
-        </is>
-      </c>
-      <c r="G45" s="5" t="inlineStr">
-        <is>
-          <t>Configuración de base de datos PostgreSQL administrada en render.yaml.</t>
+      <c r="D45" s="39" t="inlineStr">
+        <is>
+          <t>feat(temis): implement enterprise visual design system, 3-step project wizard, workspace lateral sidebar, and remove all emojis in favor of Lucide vector icons</t>
+        </is>
+      </c>
+      <c r="E45" s="37" t="inlineStr">
+        <is>
+          <t>Frontend / UI</t>
+        </is>
+      </c>
+      <c r="F45" s="40" t="inlineStr">
+        <is>
+          <t>Sprint 07 - Sep 2026</t>
+        </is>
+      </c>
+      <c r="G45" s="39" t="inlineStr">
+        <is>
+          <t>feat(temis): implement enterprise visual design system, 3-step project wizard, workspace lateral sidebar, and remove all emojis in favor of Lucide vector icons</t>
         </is>
       </c>
     </row>
     <row r="46" ht="20" customHeight="1">
-      <c r="A46" s="11" t="inlineStr">
-        <is>
-          <t>4481522</t>
-        </is>
-      </c>
-      <c r="B46" s="11" t="inlineStr">
-        <is>
-          <t>2026-08-27 16:24:37 -0600</t>
-        </is>
-      </c>
-      <c r="C46" s="27" t="inlineStr">
+      <c r="A46" s="41" t="inlineStr">
+        <is>
+          <t>14d7dac8</t>
+        </is>
+      </c>
+      <c r="B46" s="44" t="inlineStr">
+        <is>
+          <t>2026-09-22 18:31:41 -0600</t>
+        </is>
+      </c>
+      <c r="C46" s="43" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D46" s="27" t="inlineStr">
-        <is>
-          <t>fix: agrega rootDir: Temis a render.yaml</t>
-        </is>
-      </c>
-      <c r="E46" s="27" t="inlineStr">
-        <is>
-          <t>DevOps / Render</t>
-        </is>
-      </c>
-      <c r="F46" s="11" t="inlineStr">
-        <is>
-          <t>Sprint 05 - Ago 2026</t>
-        </is>
-      </c>
-      <c r="G46" s="27" t="inlineStr">
-        <is>
-          <t>Ajuste de directorio raíz de compilación en Render Blueprint.</t>
+      <c r="D46" s="43" t="inlineStr">
+        <is>
+          <t>feat(temis): complete T15 and T16 audit tickets (onboarding tab routing, save states, and operational governance gates)</t>
+        </is>
+      </c>
+      <c r="E46" s="41" t="inlineStr">
+        <is>
+          <t>Frontend / UI</t>
+        </is>
+      </c>
+      <c r="F46" s="44" t="inlineStr">
+        <is>
+          <t>Sprint 07 - Sep 2026</t>
+        </is>
+      </c>
+      <c r="G46" s="43" t="inlineStr">
+        <is>
+          <t>feat(temis): complete T15 and T16 audit tickets (onboarding tab routing, save states, and operational governance gates)</t>
         </is>
       </c>
     </row>
     <row r="47" ht="20" customHeight="1">
-      <c r="A47" s="16" t="inlineStr">
-        <is>
-          <t>fe136da</t>
-        </is>
-      </c>
-      <c r="B47" s="19" t="inlineStr">
-        <is>
-          <t>2026-08-27 16:16:55 -0600</t>
-        </is>
-      </c>
-      <c r="C47" s="29" t="inlineStr">
+      <c r="A47" s="37" t="inlineStr">
+        <is>
+          <t>35b6a849</t>
+        </is>
+      </c>
+      <c r="B47" s="40" t="inlineStr">
+        <is>
+          <t>2026-09-22 18:26:30 -0600</t>
+        </is>
+      </c>
+      <c r="C47" s="39" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D47" s="28" t="inlineStr">
-        <is>
-          <t>feat: evoluciona TEMIS a Web Flow con Reflex, simbologia oficial PDF y despliegue Render</t>
-        </is>
-      </c>
-      <c r="E47" s="28" t="inlineStr">
-        <is>
-          <t>🔥 HITO ARQUITECTURA</t>
-        </is>
-      </c>
-      <c r="F47" s="19" t="inlineStr">
-        <is>
-          <t>Sprint 05 - Ago 2026</t>
-        </is>
-      </c>
-      <c r="G47" s="29" t="inlineStr">
-        <is>
-          <t>🔥 HITO DE REESTRUCTURACIÓN: Migración fundacional de TEMIS desde aplicación de escritorio Windows a Web SaaS Full-Stack con Reflex, FastAPI, PostgreSQL y Render.</t>
+      <c r="D47" s="39" t="inlineStr">
+        <is>
+          <t>fix(temis): resolve QA audit findings T01-T14 (security, data isolation, dates, idempotency, UX improvements)</t>
+        </is>
+      </c>
+      <c r="E47" s="37" t="inlineStr">
+        <is>
+          <t>Frontend / UI</t>
+        </is>
+      </c>
+      <c r="F47" s="40" t="inlineStr">
+        <is>
+          <t>Sprint 07 - Sep 2026</t>
+        </is>
+      </c>
+      <c r="G47" s="39" t="inlineStr">
+        <is>
+          <t>fix(temis): resolve QA audit findings T01-T14 (security, data isolation, dates, idempotency, UX improvements)</t>
         </is>
       </c>
     </row>
     <row r="48" ht="20" customHeight="1">
-      <c r="A48" s="16" t="inlineStr">
-        <is>
-          <t>4c0e337</t>
-        </is>
-      </c>
-      <c r="B48" s="19" t="inlineStr">
-        <is>
-          <t>2026-01-16 16:40:11 -0600</t>
-        </is>
-      </c>
-      <c r="C48" s="29" t="inlineStr">
+      <c r="A48" s="41" t="inlineStr">
+        <is>
+          <t>19f3e4e6</t>
+        </is>
+      </c>
+      <c r="B48" s="44" t="inlineStr">
+        <is>
+          <t>2026-09-22 13:38:38 -0600</t>
+        </is>
+      </c>
+      <c r="C48" s="43" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D48" s="28" t="inlineStr">
-        <is>
-          <t>feat: Implementado sistema de base de datos compartida con Google Drive - Auto-sync cada 5 minutos - Backups automáticos - UI de configuración en Settings - Colaboración entre múltiples usuarios</t>
-        </is>
-      </c>
-      <c r="E48" s="28" t="inlineStr">
-        <is>
-          <t>Base de Datos / Inicio</t>
-        </is>
-      </c>
-      <c r="F48" s="19" t="inlineStr">
-        <is>
-          <t>Sprint 01 - Ene 2026</t>
-        </is>
-      </c>
-      <c r="G48" s="29" t="inlineStr">
-        <is>
-          <t>PRIMER COMMIT OFICIAL DE TEMIS: Arquitectura de base de datos compartida SQLite y sincronización inicial.</t>
+      <c r="D48" s="43" t="inlineStr">
+        <is>
+          <t>feat(backend): robustecer schemas con aliases, unificar reply_text en CSAT y homologar cierre de AgenteComunicador</t>
+        </is>
+      </c>
+      <c r="E48" s="41" t="inlineStr">
+        <is>
+          <t>Frontend / UI</t>
+        </is>
+      </c>
+      <c r="F48" s="44" t="inlineStr">
+        <is>
+          <t>Sprint 07 - Sep 2026</t>
+        </is>
+      </c>
+      <c r="G48" s="43" t="inlineStr">
+        <is>
+          <t>feat(backend): robustecer schemas con aliases, unificar reply_text en CSAT y homologar cierre de AgenteComunicador</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="37" t="inlineStr">
+        <is>
+          <t>8b2a6e55</t>
+        </is>
+      </c>
+      <c r="B49" s="40" t="inlineStr">
+        <is>
+          <t>2026-09-22 13:26:06 -0600</t>
+        </is>
+      </c>
+      <c r="C49" s="39" t="inlineStr">
+        <is>
+          <t>Jose Antonio Hurtado Palestina</t>
+        </is>
+      </c>
+      <c r="D49" s="39" t="inlineStr">
+        <is>
+          <t>docs(cascada): homologar prompts de los 15 agentes, estandarizar payloads HTTP y orden de cierre</t>
+        </is>
+      </c>
+      <c r="E49" s="37" t="inlineStr">
+        <is>
+          <t>Frontend / UI</t>
+        </is>
+      </c>
+      <c r="F49" s="40" t="inlineStr">
+        <is>
+          <t>Sprint 07 - Sep 2026</t>
+        </is>
+      </c>
+      <c r="G49" s="39" t="inlineStr">
+        <is>
+          <t>docs(cascada): homologar prompts de los 15 agentes, estandarizar payloads HTTP y orden de cierre</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="41" t="inlineStr">
+        <is>
+          <t>23ba5a70</t>
+        </is>
+      </c>
+      <c r="B50" s="44" t="inlineStr">
+        <is>
+          <t>2026-09-22 13:13:46 -0600</t>
+        </is>
+      </c>
+      <c r="C50" s="43" t="inlineStr">
+        <is>
+          <t>Jose Antonio Hurtado Palestina</t>
+        </is>
+      </c>
+      <c r="D50" s="43" t="inlineStr">
+        <is>
+          <t>fix(bsa-fraudes): implementar persistencia de estado post-cierre y emision de SC.037</t>
+        </is>
+      </c>
+      <c r="E50" s="41" t="inlineStr">
+        <is>
+          <t>Frontend / UI</t>
+        </is>
+      </c>
+      <c r="F50" s="44" t="inlineStr">
+        <is>
+          <t>Sprint 07 - Sep 2026</t>
+        </is>
+      </c>
+      <c r="G50" s="43" t="inlineStr">
+        <is>
+          <t>fix(bsa-fraudes): implementar persistencia de estado post-cierre y emision de SC.037</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="37" t="inlineStr">
+        <is>
+          <t>8a76d8ef</t>
+        </is>
+      </c>
+      <c r="B51" s="40" t="inlineStr">
+        <is>
+          <t>2026-09-22 12:44:54 -0600</t>
+        </is>
+      </c>
+      <c r="C51" s="39" t="inlineStr">
+        <is>
+          <t>Jose Antonio Hurtado Palestina</t>
+        </is>
+      </c>
+      <c r="D51" s="39" t="inlineStr">
+        <is>
+          <t>fix(db): ignore deleted postgres host and fallback safely to SQLite for Google Drive persistence</t>
+        </is>
+      </c>
+      <c r="E51" s="37" t="inlineStr">
+        <is>
+          <t>Google Drive / Persistencia</t>
+        </is>
+      </c>
+      <c r="F51" s="40" t="inlineStr">
+        <is>
+          <t>Sprint 07 - Sep 2026</t>
+        </is>
+      </c>
+      <c r="G51" s="39" t="inlineStr">
+        <is>
+          <t>Respaldo automático en Google Workspace Shared Drive con Service Account institucional.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(architecture): decouple corporate governance to AppSheet and re-scope TEMIS as Process Documentation Engine
</commit_message>
<xml_diff>
--- a/Temis/Backlog_Scrum_area_tecnica_TEMIS.xlsx
+++ b/Temis/Backlog_Scrum_area_tecnica_TEMIS.xlsx
@@ -718,7 +718,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
@@ -1038,17 +1038,17 @@
       </c>
       <c r="C12" s="32" t="inlineStr">
         <is>
-          <t>Pruebas de Usuario (UAT), Validación con Jefa de Procesos, Adaptaciones de Usabilidad &amp; Auto-Layout</t>
+          <t>🔥 HITO DE ARQUITECTURA: Desacoplamiento de Gobernanza a AppSheet &amp; Enfoque Motor Documental TEMIS</t>
         </is>
       </c>
       <c r="D12" s="32" t="inlineStr">
         <is>
-          <t>UAT / Swimlanes / Usabilidad / Sincronización Bidireccional</t>
+          <t>AppSheet Link / Ficha Técnica / SIPOC / BPMN / DOCX / Auditor IA</t>
         </is>
       </c>
       <c r="E12" s="32" t="inlineStr">
         <is>
-          <t>Validación en vivo del pipeline 4 fases (Entrevista-&gt;SIPOC-&gt;Flujo-&gt;Word), pruebas de estrés y refinamiento de carriles swimlanes</t>
+          <t>Desacoplamiento a AppSheet, Reenfoque a 4 Vistas Técnicas, Auditor IA 0-100 pts técnico, UAT en vivo y auto-layout</t>
         </is>
       </c>
       <c r="F12" s="34" t="inlineStr">
@@ -1057,7 +1057,7 @@
         </is>
       </c>
       <c r="G12" s="31" t="n">
-        <v>35</v>
+        <v>44</v>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
@@ -1145,8 +1145,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q26"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <dimension ref="A1:Q28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
@@ -3297,6 +3297,176 @@
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" s="41" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="B27" s="42" t="inlineStr">
+        <is>
+          <t>🔥 Desacoplamiento Gobernanza ➔ AppSheet</t>
+        </is>
+      </c>
+      <c r="C27" s="43" t="inlineStr">
+        <is>
+          <t>Epic / HITO ARQUITECTURA</t>
+        </is>
+      </c>
+      <c r="D27" s="43" t="inlineStr">
+        <is>
+          <t>Como Director de Tecnología y PMO, quiero desacoplar el flujo de gobernanza corporativa (7 fases, diarios, aprobaciones) hacia Google AppSheet, para que TEMIS opere exclusivamente como Motor Especializado de Automatización Documental de Procesos.</t>
+        </is>
+      </c>
+      <c r="E27" s="43" t="inlineStr">
+        <is>
+          <t>1. Delegar intake, estatus y aprobaciones a AppSheet. 2. Integrar ID de Iniciativa AppSheet (external_governance_id) en Ficha Técnica. 3. Limpiar navegación y sidebar en Reflex hacia 4 módulos técnicos (Ficha, SIPOC, BPMN, Work Instructions).</t>
+        </is>
+      </c>
+      <c r="F27" s="43" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G27" s="43" t="inlineStr">
+        <is>
+          <t>Separación de responsabilidades arquitecturales: AppSheet como capa de gobernanza institucional y TEMIS Web como motor de modelado BPMN, SIPOC y generación DOCX oficial.</t>
+        </is>
+      </c>
+      <c r="H27" s="41" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I27" s="44" t="n">
+        <v>13</v>
+      </c>
+      <c r="J27" s="44" t="n">
+        <v>55</v>
+      </c>
+      <c r="K27" s="44" t="inlineStr">
+        <is>
+          <t>2026-10-01 00:00:00</t>
+        </is>
+      </c>
+      <c r="L27" s="44" t="inlineStr">
+        <is>
+          <t>2026-10-15 00:00:00</t>
+        </is>
+      </c>
+      <c r="M27" s="44" t="inlineStr">
+        <is>
+          <t>Sprint 08</t>
+        </is>
+      </c>
+      <c r="N27" s="34" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="O27" s="43" t="inlineStr">
+        <is>
+          <t>Equipo Técnico TEMIS</t>
+        </is>
+      </c>
+      <c r="P27" s="43" t="inlineStr">
+        <is>
+          <t>• Navegación simplificada a 4 vistas técnicas (Ficha, SIPOC, BPMN, Work Instructions).
+• ID de Gobernanza AppSheet persistido en proyectos.
+• Cero dependencias circulares con tablas de gobernanza.</t>
+        </is>
+      </c>
+      <c r="Q27" s="43" t="inlineStr">
+        <is>
+          <t>Plan Técnico Desacoplamiento v1.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="41" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="B28" s="42" t="inlineStr">
+        <is>
+          <t>Reorientación Auditor IA Calidad Técnica (0-100)</t>
+        </is>
+      </c>
+      <c r="C28" s="43" t="inlineStr">
+        <is>
+          <t>User Story</t>
+        </is>
+      </c>
+      <c r="D28" s="43" t="inlineStr">
+        <is>
+          <t>Como analista y Jefa de Procesos, quiero que el Auditor IA evalúe la completitud y consistencia técnica de la documentación (nodos BPMN, sistemas/canales, consistencia SIPOC y capturas HD) sin penalizaciones por gobernanza externa.</t>
+        </is>
+      </c>
+      <c r="E28" s="43" t="inlineStr">
+        <is>
+          <t>1. Rediseñar rúbrica 0-100 pts con 4 pilares técnicos. 2. Ajustar prompt de auditoría en backend. 3. Actualizar interfaz modal en Reflex con feedback positivo y métricas de calidad documental.</t>
+        </is>
+      </c>
+      <c r="F28" s="43" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G28" s="43" t="inlineStr">
+        <is>
+          <t>Motor de auditoría técnica con IA enfocado en consistencia SIPOC-BPMN, conectividad de flujos, asignación de sistemas y completitud de evidencias visuales.</t>
+        </is>
+      </c>
+      <c r="H28" s="41" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I28" s="44" t="n">
+        <v>8</v>
+      </c>
+      <c r="J28" s="44" t="n">
+        <v>35</v>
+      </c>
+      <c r="K28" s="44" t="inlineStr">
+        <is>
+          <t>2026-10-02 00:00:00</t>
+        </is>
+      </c>
+      <c r="L28" s="44" t="inlineStr">
+        <is>
+          <t>2026-10-10 00:00:00</t>
+        </is>
+      </c>
+      <c r="M28" s="44" t="inlineStr">
+        <is>
+          <t>Sprint 08</t>
+        </is>
+      </c>
+      <c r="N28" s="34" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="O28" s="43" t="inlineStr">
+        <is>
+          <t>Equipo Técnico TEMIS</t>
+        </is>
+      </c>
+      <c r="P28" s="43" t="inlineStr">
+        <is>
+          <t>• Auditoría técnica 0-100 pts con desglose por pilar.
+• Sin penalizaciones por roles o fases de gobernanza.
+• Diagnóstico accionable en tiempo real.</t>
+        </is>
+      </c>
+      <c r="Q28" s="43" t="inlineStr">
+        <is>
+          <t>audit_modal.py, state.py</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3309,7 +3479,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N19"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
@@ -3341,7 +3511,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="21" t="inlineStr">
         <is>
@@ -3382,7 +3551,6 @@
         <v/>
       </c>
     </row>
-    <row r="6"/>
     <row r="7" ht="24" customHeight="1">
       <c r="A7" s="24" t="inlineStr">
         <is>
@@ -3395,7 +3563,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
@@ -3986,8 +4153,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G30"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <dimension ref="A1:G32"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
@@ -4966,6 +5133,76 @@
       <c r="G30" s="43" t="inlineStr">
         <is>
           <t>En Curso (Sprint 08)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="41" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="B31" s="43" t="inlineStr">
+        <is>
+          <t>Desacoplamiento Gobernanza / AppSheet</t>
+        </is>
+      </c>
+      <c r="C31" s="43" t="inlineStr">
+        <is>
+          <t>Desacoplamiento de gobernanza corporativa hacia AppSheet e integración external_governance_id</t>
+        </is>
+      </c>
+      <c r="D31" s="44" t="inlineStr">
+        <is>
+          <t>Sprint 08</t>
+        </is>
+      </c>
+      <c r="E31" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="F31" s="41" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="G31" s="43" t="inlineStr">
+        <is>
+          <t>feat(architecture)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="41" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="B32" s="43" t="inlineStr">
+        <is>
+          <t>Auditor IA Calidad Técnica</t>
+        </is>
+      </c>
+      <c r="C32" s="43" t="inlineStr">
+        <is>
+          <t>Reorientación de rúbrica 0-100 pts a consistencia técnica BPMN/SIPOC/Evidencias</t>
+        </is>
+      </c>
+      <c r="D32" s="44" t="inlineStr">
+        <is>
+          <t>Sprint 08</t>
+        </is>
+      </c>
+      <c r="E32" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="F32" s="41" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="G32" s="43" t="inlineStr">
+        <is>
+          <t>feat(audit)</t>
         </is>
       </c>
     </row>
@@ -4983,8 +5220,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G51"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <dimension ref="A1:G52"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
@@ -5035,493 +5272,493 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="41" t="inlineStr">
         <is>
+          <t>7b49a12c</t>
+        </is>
+      </c>
+      <c r="B2" s="44" t="inlineStr">
+        <is>
+          <t>2026-10-02 14:30:00 -0600</t>
+        </is>
+      </c>
+      <c r="C2" s="43" t="inlineStr">
+        <is>
+          <t>Jose Antonio Hurtado Palestina</t>
+        </is>
+      </c>
+      <c r="D2" s="43" t="inlineStr">
+        <is>
+          <t>feat(architecture): decouple corporate governance to AppSheet and re-scope TEMIS as Process Documentation Engine</t>
+        </is>
+      </c>
+      <c r="E2" s="41" t="inlineStr">
+        <is>
+          <t>Arquitectura / Gobernanza AppSheet</t>
+        </is>
+      </c>
+      <c r="F2" s="44" t="inlineStr">
+        <is>
+          <t>Sprint 08 - Oct 2026</t>
+        </is>
+      </c>
+      <c r="G2" s="43" t="inlineStr">
+        <is>
+          <t>Desacoplamiento de gobernanza corporativa hacia AppSheet, reorientación a 4 vistas técnicas (Ficha, SIPOC, BPMN, Work Instructions) y actualización del Auditor IA a calidad técnica (0-100 pts).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="41" t="inlineStr">
+        <is>
           <t>1fcd3fde</t>
         </is>
       </c>
-      <c r="B2" s="44" t="inlineStr">
+      <c r="B3" s="44" t="inlineStr">
         <is>
           <t>2026-09-29 16:44:13 -0600</t>
         </is>
       </c>
-      <c r="C2" s="43" t="inlineStr">
+      <c r="C3" s="43" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D2" s="43" t="inlineStr">
+      <c r="D3" s="43" t="inlineStr">
         <is>
           <t>feat(narrative): integrate official master DOCX template engine matching Plantilla_Maestra_Oficial_Work_Instructions_TEMIS</t>
         </is>
       </c>
-      <c r="E2" s="41" t="inlineStr">
+      <c r="E3" s="41" t="inlineStr">
         <is>
           <t>Plantilla Maestra Word / Narrativa</t>
         </is>
       </c>
-      <c r="F2" s="44" t="inlineStr">
+      <c r="F3" s="44" t="inlineStr">
         <is>
           <t>Sprint 07 - Sep 2026</t>
         </is>
       </c>
-      <c r="G2" s="43" t="inlineStr">
+      <c r="G3" s="43" t="inlineStr">
         <is>
           <t>Integración del motor de población sobre Plantilla_Maestra_Oficial_Work_Instructions_TEMIS.docx y 4 tablas oficiales.</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="37" t="inlineStr">
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="37" t="inlineStr">
         <is>
           <t>fc7c0eff</t>
         </is>
       </c>
-      <c r="B3" s="40" t="inlineStr">
+      <c r="B4" s="40" t="inlineStr">
         <is>
           <t>2026-09-29 14:45:49 -0600</t>
         </is>
       </c>
-      <c r="C3" s="39" t="inlineStr">
+      <c r="C4" s="39" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D3" s="39" t="inlineStr">
+      <c r="D4" s="39" t="inlineStr">
         <is>
           <t>feat(export): standardize official Word 4-table document to match SAR 90 dias and Excel SIPOC template</t>
         </is>
       </c>
-      <c r="E3" s="37" t="inlineStr">
+      <c r="E4" s="37" t="inlineStr">
         <is>
           <t>Plantilla Maestra Word / Narrativa</t>
         </is>
       </c>
-      <c r="F3" s="40" t="inlineStr">
+      <c r="F4" s="40" t="inlineStr">
         <is>
           <t>Sprint 07 - Sep 2026</t>
         </is>
       </c>
-      <c r="G3" s="39" t="inlineStr">
+      <c r="G4" s="39" t="inlineStr">
         <is>
           <t>Integración del motor de población sobre Plantilla_Maestra_Oficial_Work_Instructions_TEMIS.docx y 4 tablas oficiales.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="41" t="inlineStr">
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="41" t="inlineStr">
         <is>
           <t>6a9f6bdc</t>
         </is>
       </c>
-      <c r="B4" s="44" t="inlineStr">
+      <c r="B5" s="44" t="inlineStr">
         <is>
           <t>2026-09-28 19:13:02 -0600</t>
         </is>
       </c>
-      <c r="C4" s="43" t="inlineStr">
+      <c r="C5" s="43" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D4" s="43" t="inlineStr">
+      <c r="D5" s="43" t="inlineStr">
         <is>
           <t>fix(cascade): blindar VerificadorEstatus y agregar safety guard en AgenteComunicador contra desvios a GChat</t>
         </is>
       </c>
-      <c r="E4" s="41" t="inlineStr">
+      <c r="E5" s="41" t="inlineStr">
         <is>
           <t>Frontend / UI</t>
         </is>
       </c>
-      <c r="F4" s="44" t="inlineStr">
+      <c r="F5" s="44" t="inlineStr">
         <is>
           <t>Sprint 07 - Sep 2026</t>
         </is>
       </c>
-      <c r="G4" s="43" t="inlineStr">
+      <c r="G5" s="43" t="inlineStr">
         <is>
           <t>fix(cascade): blindar VerificadorEstatus y agregar safety guard en AgenteComunicador contra desvios a GChat</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="37" t="inlineStr">
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="37" t="inlineStr">
         <is>
           <t>d785d2c8</t>
         </is>
       </c>
-      <c r="B5" s="40" t="inlineStr">
+      <c r="B6" s="40" t="inlineStr">
         <is>
           <t>2026-09-25 07:55:43 -0600</t>
         </is>
       </c>
-      <c r="C5" s="39" t="inlineStr">
+      <c r="C6" s="39" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D5" s="39" t="inlineStr">
+      <c r="D6" s="39" t="inlineStr">
         <is>
           <t>fix(state): map charter scope to scope_in and declare private cached narrative state variables</t>
         </is>
       </c>
-      <c r="E5" s="37" t="inlineStr">
+      <c r="E6" s="37" t="inlineStr">
         <is>
           <t>Plantilla Maestra Word / Narrativa</t>
         </is>
       </c>
-      <c r="F5" s="40" t="inlineStr">
+      <c r="F6" s="40" t="inlineStr">
         <is>
           <t>Sprint 07 - Sep 2026</t>
         </is>
       </c>
-      <c r="G5" s="39" t="inlineStr">
+      <c r="G6" s="39" t="inlineStr">
         <is>
           <t>Integración del motor de población sobre Plantilla_Maestra_Oficial_Work_Instructions_TEMIS.docx y 4 tablas oficiales.</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="41" t="inlineStr">
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="41" t="inlineStr">
         <is>
           <t>237f7f7c</t>
         </is>
       </c>
-      <c r="B6" s="44" t="inlineStr">
+      <c r="B7" s="44" t="inlineStr">
         <is>
           <t>2026-09-25 07:36:53 -0600</t>
         </is>
       </c>
-      <c r="C6" s="43" t="inlineStr">
+      <c r="C7" s="43" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D6" s="43" t="inlineStr">
+      <c r="D7" s="43" t="inlineStr">
         <is>
           <t>fix(deploy): use python -m backend.main to bind PORT in Render for temis-backend</t>
         </is>
       </c>
-      <c r="E6" s="41" t="inlineStr">
+      <c r="E7" s="41" t="inlineStr">
         <is>
           <t>DevOps / Despliegue Cloud</t>
         </is>
       </c>
-      <c r="F6" s="44" t="inlineStr">
+      <c r="F7" s="44" t="inlineStr">
         <is>
           <t>Sprint 07 - Sep 2026</t>
         </is>
       </c>
-      <c r="G6" s="43" t="inlineStr">
+      <c r="G7" s="43" t="inlineStr">
         <is>
           <t>Optimización de servidor de producción ASGI, configuración de endpoints de upload y resolución de timeouts en Render.</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="37" t="inlineStr">
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="37" t="inlineStr">
         <is>
           <t>aa4e6bbb</t>
         </is>
       </c>
-      <c r="B7" s="40" t="inlineStr">
+      <c r="B8" s="40" t="inlineStr">
         <is>
           <t>2026-09-24 21:52:23 -0600</t>
         </is>
       </c>
-      <c r="C7" s="39" t="inlineStr">
+      <c r="C8" s="39" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D7" s="39" t="inlineStr">
+      <c r="D8" s="39" t="inlineStr">
         <is>
           <t>fix(prod_server): register reflex /_upload endpoints and set Upload.is_used for production server</t>
         </is>
       </c>
-      <c r="E7" s="37" t="inlineStr">
+      <c r="E8" s="37" t="inlineStr">
         <is>
           <t>Ingesta ZIP / Galería Evidencias</t>
         </is>
       </c>
-      <c r="F7" s="40" t="inlineStr">
+      <c r="F8" s="40" t="inlineStr">
         <is>
           <t>Sprint 07 - Sep 2026</t>
         </is>
       </c>
-      <c r="G7" s="39" t="inlineStr">
+      <c r="G8" s="39" t="inlineStr">
         <is>
           <t>Parser de paquetes .zip de Media Studio, visor reactivo de capturas Base64 y drag-and-drop en web.</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="41" t="inlineStr">
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="41" t="inlineStr">
         <is>
           <t>3590e8d9</t>
         </is>
       </c>
-      <c r="B8" s="44" t="inlineStr">
+      <c r="B9" s="44" t="inlineStr">
         <is>
           <t>2026-09-24 21:36:55 -0600</t>
         </is>
       </c>
-      <c r="C8" s="43" t="inlineStr">
+      <c r="C9" s="43" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D8" s="43" t="inlineStr">
+      <c r="D9" s="43" t="inlineStr">
         <is>
           <t>perf(core): add cache-first loading strategy to eliminate event loop lag on Drive calls</t>
         </is>
       </c>
-      <c r="E8" s="41" t="inlineStr">
+      <c r="E9" s="41" t="inlineStr">
         <is>
           <t>Frontend / UI</t>
         </is>
       </c>
-      <c r="F8" s="44" t="inlineStr">
+      <c r="F9" s="44" t="inlineStr">
         <is>
           <t>Sprint 07 - Sep 2026</t>
         </is>
       </c>
-      <c r="G8" s="43" t="inlineStr">
+      <c r="G9" s="43" t="inlineStr">
         <is>
           <t>perf(core): add cache-first loading strategy to eliminate event loop lag on Drive calls</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="37" t="inlineStr">
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="37" t="inlineStr">
         <is>
           <t>012ff586</t>
         </is>
       </c>
-      <c r="B9" s="40" t="inlineStr">
+      <c r="B10" s="40" t="inlineStr">
         <is>
           <t>2026-09-24 21:25:33 -0600</t>
         </is>
       </c>
-      <c r="C9" s="39" t="inlineStr">
+      <c r="C10" s="39" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D9" s="39" t="inlineStr">
+      <c r="D10" s="39" t="inlineStr">
         <is>
           <t>fix(upload): remove strict MIME accept filter to allow seamless Windows ZIP drag-and-drop</t>
         </is>
       </c>
-      <c r="E9" s="37" t="inlineStr">
+      <c r="E10" s="37" t="inlineStr">
         <is>
           <t>Ingesta ZIP / Galería Evidencias</t>
         </is>
       </c>
-      <c r="F9" s="40" t="inlineStr">
+      <c r="F10" s="40" t="inlineStr">
         <is>
           <t>Sprint 07 - Sep 2026</t>
         </is>
       </c>
-      <c r="G9" s="39" t="inlineStr">
+      <c r="G10" s="39" t="inlineStr">
         <is>
           <t>Parser de paquetes .zip de Media Studio, visor reactivo de capturas Base64 y drag-and-drop en web.</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="41" t="inlineStr">
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="41" t="inlineStr">
         <is>
           <t>88b86dd8</t>
         </is>
       </c>
-      <c r="B10" s="44" t="inlineStr">
+      <c r="B11" s="44" t="inlineStr">
         <is>
           <t>2026-09-24 21:20:44 -0600</t>
         </is>
       </c>
-      <c r="C10" s="43" t="inlineStr">
+      <c r="C11" s="43" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D10" s="43" t="inlineStr">
+      <c r="D11" s="43" t="inlineStr">
         <is>
           <t>fix(upload): add MIME type fallbacks and handler diagnostics for ZIP uploads</t>
         </is>
       </c>
-      <c r="E10" s="41" t="inlineStr">
+      <c r="E11" s="41" t="inlineStr">
         <is>
           <t>Ingesta ZIP / Galería Evidencias</t>
         </is>
       </c>
-      <c r="F10" s="44" t="inlineStr">
+      <c r="F11" s="44" t="inlineStr">
         <is>
           <t>Sprint 07 - Sep 2026</t>
         </is>
       </c>
-      <c r="G10" s="43" t="inlineStr">
+      <c r="G11" s="43" t="inlineStr">
         <is>
           <t>Parser de paquetes .zip de Media Studio, visor reactivo de capturas Base64 y drag-and-drop en web.</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="35" t="inlineStr">
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="35" t="inlineStr">
         <is>
           <t>b348d651</t>
         </is>
       </c>
-      <c r="B11" s="35" t="inlineStr">
+      <c r="B12" s="35" t="inlineStr">
         <is>
           <t>2026-09-24 21:04:18 -0600</t>
         </is>
       </c>
-      <c r="C11" s="36" t="inlineStr">
+      <c r="C12" s="36" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D11" s="36" t="inlineStr">
+      <c r="D12" s="36" t="inlineStr">
         <is>
           <t>revert(studio): keep Temis Media Studio untouched per user instruction</t>
         </is>
       </c>
-      <c r="E11" s="35" t="inlineStr">
+      <c r="E12" s="35" t="inlineStr">
         <is>
           <t>🔥 HITO: TEMIS Media Studio Desktop</t>
         </is>
       </c>
-      <c r="F11" s="35" t="inlineStr">
+      <c r="F12" s="35" t="inlineStr">
         <is>
           <t>Sprint 07 - Sep 2026</t>
         </is>
       </c>
-      <c r="G11" s="36" t="inlineStr">
+      <c r="G12" s="36" t="inlineStr">
         <is>
           <t>Suite de escritorio offline para extracción multimedia, transcripción local Whisper y captura de fotogramas clave HD.</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="41" t="inlineStr">
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="41" t="inlineStr">
         <is>
           <t>da66633c</t>
         </is>
       </c>
-      <c r="B12" s="44" t="inlineStr">
+      <c r="B13" s="44" t="inlineStr">
         <is>
           <t>2026-09-24 20:58:55 -0600</t>
         </is>
       </c>
-      <c r="C12" s="43" t="inlineStr">
+      <c r="C13" s="43" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D12" s="43" t="inlineStr">
+      <c r="D13" s="43" t="inlineStr">
         <is>
           <t>fix(narrative): optimize ZIP package handling, add progress spinners and compact auto-zip</t>
         </is>
       </c>
-      <c r="E12" s="41" t="inlineStr">
+      <c r="E13" s="41" t="inlineStr">
         <is>
           <t>Plantilla Maestra Word / Narrativa</t>
         </is>
       </c>
-      <c r="F12" s="44" t="inlineStr">
+      <c r="F13" s="44" t="inlineStr">
         <is>
           <t>Sprint 07 - Sep 2026</t>
         </is>
       </c>
-      <c r="G12" s="43" t="inlineStr">
+      <c r="G13" s="43" t="inlineStr">
         <is>
           <t>Integración del motor de población sobre Plantilla_Maestra_Oficial_Work_Instructions_TEMIS.docx y 4 tablas oficiales.</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="37" t="inlineStr">
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="37" t="inlineStr">
         <is>
           <t>21fb4dc1</t>
         </is>
       </c>
-      <c r="B13" s="40" t="inlineStr">
+      <c r="B14" s="40" t="inlineStr">
         <is>
           <t>2026-09-24 20:46:08 -0600</t>
         </is>
       </c>
-      <c r="C13" s="39" t="inlineStr">
+      <c r="C14" s="39" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D13" s="39" t="inlineStr">
+      <c r="D14" s="39" t="inlineStr">
         <is>
           <t>feat(persistence): enable dynamic Google Drive project scanning &amp; cloud user directory persistence</t>
         </is>
       </c>
-      <c r="E13" s="37" t="inlineStr">
+      <c r="E14" s="37" t="inlineStr">
         <is>
           <t>Google Drive / Persistencia</t>
         </is>
       </c>
-      <c r="F13" s="40" t="inlineStr">
+      <c r="F14" s="40" t="inlineStr">
         <is>
           <t>Sprint 07 - Sep 2026</t>
         </is>
       </c>
-      <c r="G13" s="39" t="inlineStr">
+      <c r="G14" s="39" t="inlineStr">
         <is>
           <t>Respaldo automático en Google Workspace Shared Drive con Service Account institucional.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="35" t="inlineStr">
-        <is>
-          <t>5061bb4a</t>
-        </is>
-      </c>
-      <c r="B14" s="35" t="inlineStr">
-        <is>
-          <t>2026-09-24 20:35:14 -0600</t>
-        </is>
-      </c>
-      <c r="C14" s="36" t="inlineStr">
-        <is>
-          <t>Jose Antonio Hurtado Palestina</t>
-        </is>
-      </c>
-      <c r="D14" s="36" t="inlineStr">
-        <is>
-          <t>feat(zip-ingest): add TEMIS Media Studio ZIP package ingestion, Base64 screenshot gallery, and unified pipeline in web</t>
-        </is>
-      </c>
-      <c r="E14" s="35" t="inlineStr">
-        <is>
-          <t>🔥 HITO: TEMIS Media Studio Desktop</t>
-        </is>
-      </c>
-      <c r="F14" s="35" t="inlineStr">
-        <is>
-          <t>Sprint 07 - Sep 2026</t>
-        </is>
-      </c>
-      <c r="G14" s="36" t="inlineStr">
-        <is>
-          <t>Suite de escritorio offline para extracción multimedia, transcripción local Whisper y captura de fotogramas clave HD.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
       <c r="A15" s="35" t="inlineStr">
         <is>
-          <t>9b64dc3a</t>
+          <t>5061bb4a</t>
         </is>
       </c>
       <c r="B15" s="35" t="inlineStr">
         <is>
-          <t>2026-09-24 18:08:03 -0600</t>
+          <t>2026-09-24 20:35:14 -0600</t>
         </is>
       </c>
       <c r="C15" s="36" t="inlineStr">
@@ -5531,7 +5768,7 @@
       </c>
       <c r="D15" s="36" t="inlineStr">
         <is>
-          <t>feat(studio): switch TEMIS Media Studio to 100% local faster-whisper engine and zero-token local process builder</t>
+          <t>feat(zip-ingest): add TEMIS Media Studio ZIP package ingestion, Base64 screenshot gallery, and unified pipeline in web</t>
         </is>
       </c>
       <c r="E15" s="35" t="inlineStr">
@@ -5553,1330 +5790,1367 @@
     <row r="16" ht="20" customHeight="1">
       <c r="A16" s="35" t="inlineStr">
         <is>
+          <t>9b64dc3a</t>
+        </is>
+      </c>
+      <c r="B16" s="35" t="inlineStr">
+        <is>
+          <t>2026-09-24 18:08:03 -0600</t>
+        </is>
+      </c>
+      <c r="C16" s="36" t="inlineStr">
+        <is>
+          <t>Jose Antonio Hurtado Palestina</t>
+        </is>
+      </c>
+      <c r="D16" s="36" t="inlineStr">
+        <is>
+          <t>feat(studio): switch TEMIS Media Studio to 100% local faster-whisper engine and zero-token local process builder</t>
+        </is>
+      </c>
+      <c r="E16" s="35" t="inlineStr">
+        <is>
+          <t>🔥 HITO: TEMIS Media Studio Desktop</t>
+        </is>
+      </c>
+      <c r="F16" s="35" t="inlineStr">
+        <is>
+          <t>Sprint 07 - Sep 2026</t>
+        </is>
+      </c>
+      <c r="G16" s="36" t="inlineStr">
+        <is>
+          <t>Suite de escritorio offline para extracción multimedia, transcripción local Whisper y captura de fotogramas clave HD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="35" t="inlineStr">
+        <is>
           <t>2e80a295</t>
         </is>
       </c>
-      <c r="B16" s="35" t="inlineStr">
+      <c r="B17" s="35" t="inlineStr">
         <is>
           <t>2026-09-24 17:32:50 -0600</t>
         </is>
       </c>
-      <c r="C16" s="36" t="inlineStr">
+      <c r="C17" s="36" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D16" s="36" t="inlineStr">
+      <c r="D17" s="36" t="inlineStr">
         <is>
           <t>feat(studio): add TEMIS Media Studio desktop suite for offline whisper transcription, smart screenshot capture and TEMIS package export</t>
         </is>
       </c>
-      <c r="E16" s="35" t="inlineStr">
+      <c r="E17" s="35" t="inlineStr">
         <is>
           <t>🔥 HITO: TEMIS Media Studio Desktop</t>
         </is>
       </c>
-      <c r="F16" s="35" t="inlineStr">
+      <c r="F17" s="35" t="inlineStr">
         <is>
           <t>Sprint 07 - Sep 2026</t>
         </is>
       </c>
-      <c r="G16" s="36" t="inlineStr">
+      <c r="G17" s="36" t="inlineStr">
         <is>
           <t>Suite de escritorio offline para extracción multimedia, transcripción local Whisper y captura de fotogramas clave HD.</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="37" t="inlineStr">
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="37" t="inlineStr">
         <is>
           <t>6d2dc26b</t>
         </is>
       </c>
-      <c r="B17" s="40" t="inlineStr">
+      <c r="B18" s="40" t="inlineStr">
         <is>
           <t>2026-09-24 16:04:46 -0600</t>
         </is>
       </c>
-      <c r="C17" s="39" t="inlineStr">
+      <c r="C18" s="39" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D17" s="39" t="inlineStr">
+      <c r="D18" s="39" t="inlineStr">
         <is>
           <t>fix(upload): remove on_drop overwrite to let reflex default upload_file populate rx.selected_files</t>
         </is>
       </c>
-      <c r="E17" s="37" t="inlineStr">
+      <c r="E18" s="37" t="inlineStr">
         <is>
           <t>Ingesta ZIP / Galería Evidencias</t>
         </is>
       </c>
-      <c r="F17" s="40" t="inlineStr">
+      <c r="F18" s="40" t="inlineStr">
         <is>
           <t>Sprint 07 - Sep 2026</t>
         </is>
       </c>
-      <c r="G17" s="39" t="inlineStr">
+      <c r="G18" s="39" t="inlineStr">
         <is>
           <t>Parser de paquetes .zip de Media Studio, visor reactivo de capturas Base64 y drag-and-drop en web.</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="41" t="inlineStr">
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="41" t="inlineStr">
         <is>
           <t>92be41e7</t>
         </is>
       </c>
-      <c r="B18" s="44" t="inlineStr">
+      <c r="B19" s="44" t="inlineStr">
         <is>
           <t>2026-09-24 15:12:52 -0600</t>
         </is>
       </c>
-      <c r="C18" s="43" t="inlineStr">
+      <c r="C19" s="43" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D18" s="43" t="inlineStr">
+      <c r="D19" s="43" t="inlineStr">
         <is>
           <t>feat(media): integrate Gemini File API for large audio/video files up to 2GB</t>
         </is>
       </c>
-      <c r="E18" s="41" t="inlineStr">
+      <c r="E19" s="41" t="inlineStr">
         <is>
           <t>IA / Gemini 2.5 / Audio</t>
         </is>
       </c>
-      <c r="F18" s="44" t="inlineStr">
+      <c r="F19" s="44" t="inlineStr">
         <is>
           <t>Sprint 07 - Sep 2026</t>
         </is>
       </c>
-      <c r="G18" s="43" t="inlineStr">
+      <c r="G19" s="43" t="inlineStr">
         <is>
           <t>Ingesta de audios y videos masivos con Gemini File API y extracción incremental de narrativa.</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="37" t="inlineStr">
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="37" t="inlineStr">
         <is>
           <t>2d85d5ec</t>
         </is>
       </c>
-      <c r="B19" s="40" t="inlineStr">
+      <c r="B20" s="40" t="inlineStr">
         <is>
           <t>2026-09-24 15:06:46 -0600</t>
         </is>
       </c>
-      <c r="C19" s="39" t="inlineStr">
+      <c r="C20" s="39" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D19" s="39" t="inlineStr">
+      <c r="D20" s="39" t="inlineStr">
         <is>
           <t>feat(media): add upload spinner loading state and size tip note</t>
         </is>
       </c>
-      <c r="E19" s="37" t="inlineStr">
+      <c r="E20" s="37" t="inlineStr">
         <is>
           <t>Ingesta ZIP / Galería Evidencias</t>
         </is>
       </c>
-      <c r="F19" s="40" t="inlineStr">
+      <c r="F20" s="40" t="inlineStr">
         <is>
           <t>Sprint 07 - Sep 2026</t>
         </is>
       </c>
-      <c r="G19" s="39" t="inlineStr">
+      <c r="G20" s="39" t="inlineStr">
         <is>
           <t>Parser de paquetes .zip de Media Studio, visor reactivo de capturas Base64 y drag-and-drop en web.</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="41" t="inlineStr">
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="41" t="inlineStr">
         <is>
           <t>c7175a5e</t>
         </is>
       </c>
-      <c r="B20" s="44" t="inlineStr">
+      <c r="B21" s="44" t="inlineStr">
         <is>
           <t>2026-09-24 14:51:27 -0600</t>
         </is>
       </c>
-      <c r="C20" s="43" t="inlineStr">
+      <c r="C21" s="43" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D20" s="43" t="inlineStr">
+      <c r="D21" s="43" t="inlineStr">
         <is>
           <t>fix(upload): connect rx.upload_files to on_drop and add selected file process button</t>
         </is>
       </c>
-      <c r="E20" s="41" t="inlineStr">
+      <c r="E21" s="41" t="inlineStr">
         <is>
           <t>Ingesta ZIP / Galería Evidencias</t>
         </is>
       </c>
-      <c r="F20" s="44" t="inlineStr">
+      <c r="F21" s="44" t="inlineStr">
         <is>
           <t>Sprint 07 - Sep 2026</t>
         </is>
       </c>
-      <c r="G20" s="43" t="inlineStr">
+      <c r="G21" s="43" t="inlineStr">
         <is>
           <t>Parser de paquetes .zip de Media Studio, visor reactivo de capturas Base64 y drag-and-drop en web.</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="37" t="inlineStr">
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="37" t="inlineStr">
         <is>
           <t>5b3d027f</t>
         </is>
       </c>
-      <c r="B21" s="40" t="inlineStr">
+      <c r="B22" s="40" t="inlineStr">
         <is>
           <t>2026-09-24 14:41:38 -0600</t>
         </is>
       </c>
-      <c r="C21" s="39" t="inlineStr">
+      <c r="C22" s="39" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D21" s="39" t="inlineStr">
+      <c r="D22" s="39" t="inlineStr">
         <is>
           <t>fix(build): extract document_library_item to top-level typed component to resolve foreach UntypedVarError in Render</t>
         </is>
       </c>
-      <c r="E21" s="37" t="inlineStr">
+      <c r="E22" s="37" t="inlineStr">
         <is>
           <t>Frontend / UI</t>
         </is>
       </c>
-      <c r="F21" s="40" t="inlineStr">
+      <c r="F22" s="40" t="inlineStr">
         <is>
           <t>Sprint 07 - Sep 2026</t>
         </is>
       </c>
-      <c r="G21" s="39" t="inlineStr">
+      <c r="G22" s="39" t="inlineStr">
         <is>
           <t>fix(build): extract document_library_item to top-level typed component to resolve foreach UntypedVarError in Render</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="41" t="inlineStr">
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="41" t="inlineStr">
         <is>
           <t>957bfeba</t>
         </is>
       </c>
-      <c r="B22" s="44" t="inlineStr">
+      <c r="B23" s="44" t="inlineStr">
         <is>
           <t>2026-09-24 14:30:28 -0600</t>
         </is>
       </c>
-      <c r="C22" s="43" t="inlineStr">
+      <c r="C23" s="43" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D22" s="43" t="inlineStr">
+      <c r="D23" s="43" t="inlineStr">
         <is>
           <t>feat(media): implement universal audio/video ingestion with mutagen metadata and audit transcript export in docx/txt</t>
         </is>
       </c>
-      <c r="E22" s="41" t="inlineStr">
+      <c r="E23" s="41" t="inlineStr">
         <is>
           <t>Plantilla Maestra Word / Narrativa</t>
         </is>
       </c>
-      <c r="F22" s="44" t="inlineStr">
+      <c r="F23" s="44" t="inlineStr">
         <is>
           <t>Sprint 07 - Sep 2026</t>
         </is>
       </c>
-      <c r="G22" s="43" t="inlineStr">
+      <c r="G23" s="43" t="inlineStr">
         <is>
           <t>Integración del motor de población sobre Plantilla_Maestra_Oficial_Work_Instructions_TEMIS.docx y 4 tablas oficiales.</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="37" t="inlineStr">
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="37" t="inlineStr">
         <is>
           <t>3d0d6ded</t>
         </is>
       </c>
-      <c r="B23" s="40" t="inlineStr">
+      <c r="B24" s="40" t="inlineStr">
         <is>
           <t>2026-09-23 17:34:48 -0600</t>
         </is>
       </c>
-      <c r="C23" s="39" t="inlineStr">
+      <c r="C24" s="39" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D23" s="39" t="inlineStr">
+      <c r="D24" s="39" t="inlineStr">
         <is>
           <t>feat(narrative): implement multi-document incremental ingestion and enrichment pipeline</t>
         </is>
       </c>
-      <c r="E23" s="37" t="inlineStr">
+      <c r="E24" s="37" t="inlineStr">
         <is>
           <t>Plantilla Maestra Word / Narrativa</t>
         </is>
       </c>
-      <c r="F23" s="40" t="inlineStr">
+      <c r="F24" s="40" t="inlineStr">
         <is>
           <t>Sprint 07 - Sep 2026</t>
         </is>
       </c>
-      <c r="G23" s="39" t="inlineStr">
+      <c r="G24" s="39" t="inlineStr">
         <is>
           <t>Integración del motor de población sobre Plantilla_Maestra_Oficial_Work_Instructions_TEMIS.docx y 4 tablas oficiales.</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="41" t="inlineStr">
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="41" t="inlineStr">
         <is>
           <t>7229b48e</t>
         </is>
       </c>
-      <c r="B24" s="44" t="inlineStr">
+      <c r="B25" s="44" t="inlineStr">
         <is>
           <t>2026-09-23 15:58:38 -0600</t>
         </is>
       </c>
-      <c r="C24" s="43" t="inlineStr">
+      <c r="C25" s="43" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D24" s="43" t="inlineStr">
+      <c r="D25" s="43" t="inlineStr">
         <is>
           <t>feat(narrative): implement client narrative analysis, citations, dual SIPOC, 4-table Word manuals and dual BPMN generation</t>
         </is>
       </c>
-      <c r="E24" s="41" t="inlineStr">
+      <c r="E25" s="41" t="inlineStr">
         <is>
           <t>Plantilla Maestra Word / Narrativa</t>
         </is>
       </c>
-      <c r="F24" s="44" t="inlineStr">
+      <c r="F25" s="44" t="inlineStr">
         <is>
           <t>Sprint 07 - Sep 2026</t>
         </is>
       </c>
-      <c r="G24" s="43" t="inlineStr">
+      <c r="G25" s="43" t="inlineStr">
         <is>
           <t>Integración del motor de población sobre Plantilla_Maestra_Oficial_Work_Instructions_TEMIS.docx y 4 tablas oficiales.</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="20" customHeight="1">
-      <c r="A25" s="37" t="inlineStr">
+    <row r="26" ht="20" customHeight="1">
+      <c r="A26" s="37" t="inlineStr">
         <is>
           <t>74e28a73</t>
         </is>
       </c>
-      <c r="B25" s="40" t="inlineStr">
+      <c r="B26" s="40" t="inlineStr">
         <is>
           <t>2026-09-23 15:16:40 -0600</t>
         </is>
       </c>
-      <c r="C25" s="39" t="inlineStr">
+      <c r="C26" s="39" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D25" s="39" t="inlineStr">
+      <c r="D26" s="39" t="inlineStr">
         <is>
           <t>fix(deploy): initialize Reflex state and Starlette lifespan in prod_server for event processor</t>
         </is>
       </c>
-      <c r="E25" s="37" t="inlineStr">
+      <c r="E26" s="37" t="inlineStr">
         <is>
           <t>DevOps / Despliegue Cloud</t>
         </is>
       </c>
-      <c r="F25" s="40" t="inlineStr">
+      <c r="F26" s="40" t="inlineStr">
         <is>
           <t>Sprint 07 - Sep 2026</t>
         </is>
       </c>
-      <c r="G25" s="39" t="inlineStr">
+      <c r="G26" s="39" t="inlineStr">
         <is>
           <t>Optimización de servidor de producción ASGI, configuración de endpoints de upload y resolución de timeouts en Render.</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="20" customHeight="1">
-      <c r="A26" s="41" t="inlineStr">
+    <row r="27" ht="20" customHeight="1">
+      <c r="A27" s="41" t="inlineStr">
         <is>
           <t>158f0ff4</t>
         </is>
       </c>
-      <c r="B26" s="44" t="inlineStr">
+      <c r="B27" s="44" t="inlineStr">
         <is>
           <t>2026-09-23 14:51:23 -0600</t>
         </is>
       </c>
-      <c r="C26" s="43" t="inlineStr">
+      <c r="C27" s="43" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D26" s="43" t="inlineStr">
+      <c r="D27" s="43" t="inlineStr">
         <is>
           <t>feat(deploy): add lightweight ASGI prod_server.py to avoid runtime compile OOM in Render</t>
         </is>
       </c>
-      <c r="E26" s="41" t="inlineStr">
+      <c r="E27" s="41" t="inlineStr">
         <is>
           <t>DevOps / Despliegue Cloud</t>
         </is>
       </c>
-      <c r="F26" s="44" t="inlineStr">
+      <c r="F27" s="44" t="inlineStr">
         <is>
           <t>Sprint 07 - Sep 2026</t>
         </is>
       </c>
-      <c r="G26" s="43" t="inlineStr">
+      <c r="G27" s="43" t="inlineStr">
         <is>
           <t>Optimización de servidor de producción ASGI, configuración de endpoints de upload y resolución de timeouts en Render.</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="20" customHeight="1">
-      <c r="A27" s="37" t="inlineStr">
+    <row r="28" ht="20" customHeight="1">
+      <c r="A28" s="37" t="inlineStr">
         <is>
           <t>5af5f0a0</t>
         </is>
       </c>
-      <c r="B27" s="40" t="inlineStr">
+      <c r="B28" s="40" t="inlineStr">
         <is>
           <t>2026-09-23 13:07:44 -0600</t>
         </is>
       </c>
-      <c r="C27" s="39" t="inlineStr">
+      <c r="C28" s="39" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D27" s="39" t="inlineStr">
+      <c r="D28" s="39" t="inlineStr">
         <is>
           <t>fix(deploy): use --single-port with --backend-host 0.0.0.0 --backend-port \ in render.yaml</t>
         </is>
       </c>
-      <c r="E27" s="37" t="inlineStr">
+      <c r="E28" s="37" t="inlineStr">
         <is>
           <t>DevOps / Despliegue Cloud</t>
         </is>
       </c>
-      <c r="F27" s="40" t="inlineStr">
+      <c r="F28" s="40" t="inlineStr">
         <is>
           <t>Sprint 07 - Sep 2026</t>
         </is>
       </c>
-      <c r="G27" s="39" t="inlineStr">
+      <c r="G28" s="39" t="inlineStr">
         <is>
           <t>Optimización de servidor de producción ASGI, configuración de endpoints de upload y resolución de timeouts en Render.</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="20" customHeight="1">
-      <c r="A28" s="41" t="inlineStr">
+    <row r="29" ht="20" customHeight="1">
+      <c r="A29" s="41" t="inlineStr">
         <is>
           <t>ff604053</t>
         </is>
       </c>
-      <c r="B28" s="44" t="inlineStr">
+      <c r="B29" s="44" t="inlineStr">
         <is>
           <t>2026-09-23 12:44:30 -0600</t>
         </is>
       </c>
-      <c r="C28" s="43" t="inlineStr">
+      <c r="C29" s="43" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D28" s="43" t="inlineStr">
+      <c r="D29" s="43" t="inlineStr">
         <is>
           <t>fix(temis): resolve Radix HStack integer spacing and padding type constraints</t>
         </is>
       </c>
-      <c r="E28" s="41" t="inlineStr">
+      <c r="E29" s="41" t="inlineStr">
         <is>
           <t>Frontend / UI</t>
         </is>
       </c>
-      <c r="F28" s="44" t="inlineStr">
+      <c r="F29" s="44" t="inlineStr">
         <is>
           <t>Sprint 07 - Sep 2026</t>
         </is>
       </c>
-      <c r="G28" s="43" t="inlineStr">
+      <c r="G29" s="43" t="inlineStr">
         <is>
           <t>fix(temis): resolve Radix HStack integer spacing and padding type constraints</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="20" customHeight="1">
-      <c r="A29" s="37" t="inlineStr">
+    <row r="30" ht="20" customHeight="1">
+      <c r="A30" s="37" t="inlineStr">
         <is>
           <t>fa12f8df</t>
         </is>
       </c>
-      <c r="B29" s="40" t="inlineStr">
+      <c r="B30" s="40" t="inlineStr">
         <is>
           <t>2026-09-23 12:34:14 -0600</t>
         </is>
       </c>
-      <c r="C29" s="39" t="inlineStr">
+      <c r="C30" s="39" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D29" s="39" t="inlineStr">
+      <c r="D30" s="39" t="inlineStr">
         <is>
           <t>feat(temis): implement verification improvements H01 to H06</t>
         </is>
       </c>
-      <c r="E29" s="37" t="inlineStr">
+      <c r="E30" s="37" t="inlineStr">
         <is>
           <t>Frontend / UI</t>
         </is>
       </c>
-      <c r="F29" s="40" t="inlineStr">
+      <c r="F30" s="40" t="inlineStr">
         <is>
           <t>Sprint 07 - Sep 2026</t>
         </is>
       </c>
-      <c r="G29" s="39" t="inlineStr">
+      <c r="G30" s="39" t="inlineStr">
         <is>
           <t>feat(temis): implement verification improvements H01 to H06</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="20" customHeight="1">
-      <c r="A30" s="41" t="inlineStr">
+    <row r="31" ht="20" customHeight="1">
+      <c r="A31" s="41" t="inlineStr">
         <is>
           <t>1d3f1819</t>
         </is>
       </c>
-      <c r="B30" s="44" t="inlineStr">
+      <c r="B31" s="44" t="inlineStr">
         <is>
           <t>2026-09-23 11:52:59 -0600</t>
         </is>
       </c>
-      <c r="C30" s="43" t="inlineStr">
+      <c r="C31" s="43" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D30" s="43" t="inlineStr">
+      <c r="D31" s="43" t="inlineStr">
         <is>
           <t>feat(temis): implement formal verification audit findings (F01-F06) for phase gates, selection isolation, AI audit, and backlog modal</t>
         </is>
       </c>
-      <c r="E30" s="41" t="inlineStr">
+      <c r="E31" s="41" t="inlineStr">
         <is>
           <t>Frontend / UI</t>
         </is>
       </c>
-      <c r="F30" s="44" t="inlineStr">
+      <c r="F31" s="44" t="inlineStr">
         <is>
           <t>Sprint 07 - Sep 2026</t>
         </is>
       </c>
-      <c r="G30" s="43" t="inlineStr">
+      <c r="G31" s="43" t="inlineStr">
         <is>
           <t>feat(temis): implement formal verification audit findings (F01-F06) for phase gates, selection isolation, AI audit, and backlog modal</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="20" customHeight="1">
-      <c r="A31" s="37" t="inlineStr">
+    <row r="32" ht="20" customHeight="1">
+      <c r="A32" s="37" t="inlineStr">
         <is>
           <t>603d7945</t>
         </is>
       </c>
-      <c r="B31" s="40" t="inlineStr">
+      <c r="B32" s="40" t="inlineStr">
         <is>
           <t>2026-09-23 10:52:17 -0600</t>
         </is>
       </c>
-      <c r="C31" s="39" t="inlineStr">
+      <c r="C32" s="39" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D31" s="39" t="inlineStr">
+      <c r="D32" s="39" t="inlineStr">
         <is>
           <t>fix(render): pre-compile frontend during build phase with reflex export --no-zip to prevent port scan timeout on startup</t>
         </is>
       </c>
-      <c r="E31" s="37" t="inlineStr">
+      <c r="E32" s="37" t="inlineStr">
         <is>
           <t>Ingesta ZIP / Galería Evidencias</t>
         </is>
       </c>
-      <c r="F31" s="40" t="inlineStr">
+      <c r="F32" s="40" t="inlineStr">
         <is>
           <t>Sprint 07 - Sep 2026</t>
         </is>
       </c>
-      <c r="G31" s="39" t="inlineStr">
+      <c r="G32" s="39" t="inlineStr">
         <is>
           <t>Parser de paquetes .zip de Media Studio, visor reactivo de capturas Base64 y drag-and-drop en web.</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="20" customHeight="1">
-      <c r="A32" s="41" t="inlineStr">
+    <row r="33" ht="20" customHeight="1">
+      <c r="A33" s="41" t="inlineStr">
         <is>
           <t>7a70433a</t>
         </is>
       </c>
-      <c r="B32" s="44" t="inlineStr">
+      <c r="B33" s="44" t="inlineStr">
         <is>
           <t>2026-09-23 10:08:17 -0600</t>
         </is>
       </c>
-      <c r="C32" s="43" t="inlineStr">
+      <c r="C33" s="43" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D32" s="43" t="inlineStr">
+      <c r="D33" s="43" t="inlineStr">
         <is>
           <t>fix(temis): resolve BPMN multi-page selection desync P0, non-destructive SIPOC flow generation P0, accessible 44px nudge controls P1, AI proposal review modal P1, and Excel MIME export P2</t>
         </is>
       </c>
-      <c r="E32" s="41" t="inlineStr">
+      <c r="E33" s="41" t="inlineStr">
         <is>
           <t>SIPOC / Excel Oficial</t>
         </is>
       </c>
-      <c r="F32" s="44" t="inlineStr">
+      <c r="F33" s="44" t="inlineStr">
         <is>
           <t>Sprint 07 - Sep 2026</t>
         </is>
       </c>
-      <c r="G32" s="43" t="inlineStr">
+      <c r="G33" s="43" t="inlineStr">
         <is>
           <t>Estandarización del exportador Excel idéntico a Plantilla Matriz Sipoc.xlsx con 11 columnas y Century Gothic.</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="20" customHeight="1">
-      <c r="A33" s="37" t="inlineStr">
+    <row r="34" ht="20" customHeight="1">
+      <c r="A34" s="37" t="inlineStr">
         <is>
           <t>23a039ac</t>
         </is>
       </c>
-      <c r="B33" s="40" t="inlineStr">
+      <c r="B34" s="40" t="inlineStr">
         <is>
           <t>2026-09-23 09:50:35 -0600</t>
         </is>
       </c>
-      <c r="C33" s="39" t="inlineStr">
+      <c r="C34" s="39" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D33" s="39" t="inlineStr">
+      <c r="D34" s="39" t="inlineStr">
         <is>
           <t>feat(temis): resolve audit findings - P0 user recovery, canonical SP consistency, Executive Light Slate theme (WCAG 2.2 AA), and BPMN/SIPOC usability</t>
         </is>
       </c>
-      <c r="E33" s="37" t="inlineStr">
+      <c r="E34" s="37" t="inlineStr">
         <is>
           <t>Frontend / UI</t>
         </is>
       </c>
-      <c r="F33" s="40" t="inlineStr">
+      <c r="F34" s="40" t="inlineStr">
         <is>
           <t>Sprint 07 - Sep 2026</t>
         </is>
       </c>
-      <c r="G33" s="39" t="inlineStr">
+      <c r="G34" s="39" t="inlineStr">
         <is>
           <t>feat(temis): resolve audit findings - P0 user recovery, canonical SP consistency, Executive Light Slate theme (WCAG 2.2 AA), and BPMN/SIPOC usability</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="20" customHeight="1">
-      <c r="A34" s="41" t="inlineStr">
+    <row r="35" ht="20" customHeight="1">
+      <c r="A35" s="41" t="inlineStr">
         <is>
           <t>2dd8d83a</t>
         </is>
       </c>
-      <c r="B34" s="44" t="inlineStr">
+      <c r="B35" s="44" t="inlineStr">
         <is>
           <t>2026-09-22 22:42:55 -0600</t>
         </is>
       </c>
-      <c r="C34" s="43" t="inlineStr">
+      <c r="C35" s="43" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D34" s="43" t="inlineStr">
+      <c r="D35" s="43" t="inlineStr">
         <is>
           <t>fix(auth): fix login card z-index stacking and pointer-events layering issue</t>
         </is>
       </c>
-      <c r="E34" s="41" t="inlineStr">
+      <c r="E35" s="41" t="inlineStr">
         <is>
           <t>Frontend / UI</t>
         </is>
       </c>
-      <c r="F34" s="44" t="inlineStr">
+      <c r="F35" s="44" t="inlineStr">
         <is>
           <t>Sprint 07 - Sep 2026</t>
         </is>
       </c>
-      <c r="G34" s="43" t="inlineStr">
+      <c r="G35" s="43" t="inlineStr">
         <is>
           <t>fix(auth): fix login card z-index stacking and pointer-events layering issue</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="20" customHeight="1">
-      <c r="A35" s="37" t="inlineStr">
+    <row r="36" ht="20" customHeight="1">
+      <c r="A36" s="37" t="inlineStr">
         <is>
           <t>9e917f18</t>
         </is>
       </c>
-      <c r="B35" s="40" t="inlineStr">
+      <c r="B36" s="40" t="inlineStr">
         <is>
           <t>2026-09-22 22:29:27 -0600</t>
         </is>
       </c>
-      <c r="C35" s="39" t="inlineStr">
+      <c r="C36" s="39" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D35" s="39" t="inlineStr">
+      <c r="D36" s="39" t="inlineStr">
         <is>
           <t>feat(ui): complete executive dark mode overhaul across all views and canvas</t>
         </is>
       </c>
-      <c r="E35" s="37" t="inlineStr">
+      <c r="E36" s="37" t="inlineStr">
         <is>
           <t>Frontend / UI</t>
         </is>
       </c>
-      <c r="F35" s="40" t="inlineStr">
+      <c r="F36" s="40" t="inlineStr">
         <is>
           <t>Sprint 07 - Sep 2026</t>
         </is>
       </c>
-      <c r="G35" s="39" t="inlineStr">
+      <c r="G36" s="39" t="inlineStr">
         <is>
           <t>feat(ui): complete executive dark mode overhaul across all views and canvas</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="20" customHeight="1">
-      <c r="A36" s="41" t="inlineStr">
+    <row r="37" ht="20" customHeight="1">
+      <c r="A37" s="41" t="inlineStr">
         <is>
           <t>3b91534d</t>
         </is>
       </c>
-      <c r="B36" s="44" t="inlineStr">
+      <c r="B37" s="44" t="inlineStr">
         <is>
           <t>2026-09-22 21:58:44 -0600</t>
         </is>
       </c>
-      <c r="C36" s="43" t="inlineStr">
+      <c r="C37" s="43" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D36" s="43" t="inlineStr">
+      <c r="D37" s="43" t="inlineStr">
         <is>
           <t>fix(deploy): resolve FlowState export attribute error and normalize Lucide icon tags</t>
         </is>
       </c>
-      <c r="E36" s="41" t="inlineStr">
+      <c r="E37" s="41" t="inlineStr">
         <is>
           <t>SIPOC / Excel Oficial</t>
         </is>
       </c>
-      <c r="F36" s="44" t="inlineStr">
+      <c r="F37" s="44" t="inlineStr">
         <is>
           <t>Sprint 07 - Sep 2026</t>
         </is>
       </c>
-      <c r="G36" s="43" t="inlineStr">
+      <c r="G37" s="43" t="inlineStr">
         <is>
           <t>Estandarización del exportador Excel idéntico a Plantilla Matriz Sipoc.xlsx con 11 columnas y Century Gothic.</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="20" customHeight="1">
-      <c r="A37" s="37" t="inlineStr">
+    <row r="38" ht="20" customHeight="1">
+      <c r="A38" s="37" t="inlineStr">
         <is>
           <t>94572889</t>
         </is>
       </c>
-      <c r="B37" s="40" t="inlineStr">
+      <c r="B38" s="40" t="inlineStr">
         <is>
           <t>2026-09-22 21:48:22 -0600</t>
         </is>
       </c>
-      <c r="C37" s="39" t="inlineStr">
+      <c r="C38" s="39" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D37" s="39" t="inlineStr">
+      <c r="D38" s="39" t="inlineStr">
         <is>
           <t>feat(ui): complete executive visual redesign with slate contrast, 0% emojis, elevated cards and high-contrast typography</t>
         </is>
       </c>
-      <c r="E37" s="37" t="inlineStr">
+      <c r="E38" s="37" t="inlineStr">
         <is>
           <t>Frontend / UI</t>
         </is>
       </c>
-      <c r="F37" s="40" t="inlineStr">
+      <c r="F38" s="40" t="inlineStr">
         <is>
           <t>Sprint 07 - Sep 2026</t>
         </is>
       </c>
-      <c r="G37" s="39" t="inlineStr">
+      <c r="G38" s="39" t="inlineStr">
         <is>
           <t>feat(ui): complete executive visual redesign with slate contrast, 0% emojis, elevated cards and high-contrast typography</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="20" customHeight="1">
-      <c r="A38" s="41" t="inlineStr">
+    <row r="39" ht="20" customHeight="1">
+      <c r="A39" s="41" t="inlineStr">
         <is>
           <t>a90ae9cf</t>
         </is>
       </c>
-      <c r="B38" s="44" t="inlineStr">
+      <c r="B39" s="44" t="inlineStr">
         <is>
           <t>2026-09-22 21:30:33 -0600</t>
         </is>
       </c>
-      <c r="C38" s="43" t="inlineStr">
+      <c r="C39" s="43" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D38" s="43" t="inlineStr">
+      <c r="D39" s="43" t="inlineStr">
         <is>
           <t>feat(temis): add auto-save heartbeat, executive charter print/PDF export, floating toast alerts, and audit score delta</t>
         </is>
       </c>
-      <c r="E38" s="41" t="inlineStr">
+      <c r="E39" s="41" t="inlineStr">
         <is>
           <t>SIPOC / Excel Oficial</t>
         </is>
       </c>
-      <c r="F38" s="44" t="inlineStr">
+      <c r="F39" s="44" t="inlineStr">
         <is>
           <t>Sprint 07 - Sep 2026</t>
         </is>
       </c>
-      <c r="G38" s="43" t="inlineStr">
+      <c r="G39" s="43" t="inlineStr">
         <is>
           <t>Estandarización del exportador Excel idéntico a Plantilla Matriz Sipoc.xlsx con 11 columnas y Century Gothic.</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="20" customHeight="1">
-      <c r="A39" s="37" t="inlineStr">
+    <row r="40" ht="20" customHeight="1">
+      <c r="A40" s="37" t="inlineStr">
         <is>
           <t>a1a70ae0</t>
         </is>
       </c>
-      <c r="B39" s="40" t="inlineStr">
+      <c r="B40" s="40" t="inlineStr">
         <is>
           <t>2026-09-22 21:17:22 -0600</t>
         </is>
       </c>
-      <c r="C39" s="39" t="inlineStr">
+      <c r="C40" s="39" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D39" s="39" t="inlineStr">
+      <c r="D40" s="39" t="inlineStr">
         <is>
           <t>fix(temis): add responsive table containers and toolbar wrapping to SIPOC and Work Plan views</t>
         </is>
       </c>
-      <c r="E39" s="37" t="inlineStr">
+      <c r="E40" s="37" t="inlineStr">
         <is>
           <t>Frontend / UI</t>
         </is>
       </c>
-      <c r="F39" s="40" t="inlineStr">
+      <c r="F40" s="40" t="inlineStr">
         <is>
           <t>Sprint 07 - Sep 2026</t>
         </is>
       </c>
-      <c r="G39" s="39" t="inlineStr">
+      <c r="G40" s="39" t="inlineStr">
         <is>
           <t>fix(temis): add responsive table containers and toolbar wrapping to SIPOC and Work Plan views</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="20" customHeight="1">
-      <c r="A40" s="41" t="inlineStr">
+    <row r="41" ht="20" customHeight="1">
+      <c r="A41" s="41" t="inlineStr">
         <is>
           <t>c4b05b5c</t>
         </is>
       </c>
-      <c r="B40" s="44" t="inlineStr">
+      <c r="B41" s="44" t="inlineStr">
         <is>
           <t>2026-09-22 21:13:41 -0600</t>
         </is>
       </c>
-      <c r="C40" s="43" t="inlineStr">
+      <c r="C41" s="43" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D40" s="43" t="inlineStr">
+      <c r="D41" s="43" t="inlineStr">
         <is>
           <t>fix(temis): implement full UX/UI audit recommendations - responsive reflow, clean semantics, sprint sync, and zero emojis</t>
         </is>
       </c>
-      <c r="E40" s="41" t="inlineStr">
+      <c r="E41" s="41" t="inlineStr">
         <is>
           <t>Frontend / UI</t>
         </is>
       </c>
-      <c r="F40" s="44" t="inlineStr">
+      <c r="F41" s="44" t="inlineStr">
         <is>
           <t>Sprint 07 - Sep 2026</t>
         </is>
       </c>
-      <c r="G40" s="43" t="inlineStr">
+      <c r="G41" s="43" t="inlineStr">
         <is>
           <t>fix(temis): implement full UX/UI audit recommendations - responsive reflow, clean semantics, sprint sync, and zero emojis</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="20" customHeight="1">
-      <c r="A41" s="37" t="inlineStr">
+    <row r="42" ht="20" customHeight="1">
+      <c r="A42" s="37" t="inlineStr">
         <is>
           <t>5e1cc184</t>
         </is>
       </c>
-      <c r="B41" s="40" t="inlineStr">
+      <c r="B42" s="40" t="inlineStr">
         <is>
           <t>2026-09-22 20:38:56 -0600</t>
         </is>
       </c>
-      <c r="C41" s="39" t="inlineStr">
+      <c r="C42" s="39" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D41" s="39" t="inlineStr">
+      <c r="D42" s="39" t="inlineStr">
         <is>
           <t>fix(temis): resolve Reflex Var type in user table and standardize Lucide circle-check icon</t>
         </is>
       </c>
-      <c r="E41" s="37" t="inlineStr">
+      <c r="E42" s="37" t="inlineStr">
         <is>
           <t>Frontend / UI</t>
         </is>
       </c>
-      <c r="F41" s="40" t="inlineStr">
+      <c r="F42" s="40" t="inlineStr">
         <is>
           <t>Sprint 07 - Sep 2026</t>
         </is>
       </c>
-      <c r="G41" s="39" t="inlineStr">
+      <c r="G42" s="39" t="inlineStr">
         <is>
           <t>fix(temis): resolve Reflex Var type in user table and standardize Lucide circle-check icon</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="20" customHeight="1">
-      <c r="A42" s="41" t="inlineStr">
+    <row r="43" ht="20" customHeight="1">
+      <c r="A43" s="41" t="inlineStr">
         <is>
           <t>1f29dea3</t>
         </is>
       </c>
-      <c r="B42" s="44" t="inlineStr">
+      <c r="B43" s="44" t="inlineStr">
         <is>
           <t>2026-09-22 19:21:19 -0600</t>
         </is>
       </c>
-      <c r="C42" s="43" t="inlineStr">
+      <c r="C43" s="43" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D42" s="43" t="inlineStr">
+      <c r="D43" s="43" t="inlineStr">
         <is>
           <t>feat(temis): add project deletion with confirmation modal and project access assignment per user in user management</t>
         </is>
       </c>
-      <c r="E42" s="41" t="inlineStr">
+      <c r="E43" s="41" t="inlineStr">
         <is>
           <t>Frontend / UI</t>
         </is>
       </c>
-      <c r="F42" s="44" t="inlineStr">
+      <c r="F43" s="44" t="inlineStr">
         <is>
           <t>Sprint 07 - Sep 2026</t>
         </is>
       </c>
-      <c r="G42" s="43" t="inlineStr">
+      <c r="G43" s="43" t="inlineStr">
         <is>
           <t>feat(temis): add project deletion with confirmation modal and project access assignment per user in user management</t>
         </is>
       </c>
     </row>
-    <row r="43" ht="20" customHeight="1">
-      <c r="A43" s="37" t="inlineStr">
+    <row r="44" ht="20" customHeight="1">
+      <c r="A44" s="37" t="inlineStr">
         <is>
           <t>a5e507a4</t>
         </is>
       </c>
-      <c r="B43" s="40" t="inlineStr">
+      <c r="B44" s="40" t="inlineStr">
         <is>
           <t>2026-09-22 18:57:27 -0600</t>
         </is>
       </c>
-      <c r="C43" s="39" t="inlineStr">
+      <c r="C44" s="39" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D43" s="39" t="inlineStr">
+      <c r="D44" s="39" t="inlineStr">
         <is>
           <t>style(temis): complete 100% emoji-free UI and standard typographic strings across all views</t>
         </is>
       </c>
-      <c r="E43" s="37" t="inlineStr">
+      <c r="E44" s="37" t="inlineStr">
         <is>
           <t>Frontend / UI</t>
         </is>
       </c>
-      <c r="F43" s="40" t="inlineStr">
+      <c r="F44" s="40" t="inlineStr">
         <is>
           <t>Sprint 07 - Sep 2026</t>
         </is>
       </c>
-      <c r="G43" s="39" t="inlineStr">
+      <c r="G44" s="39" t="inlineStr">
         <is>
           <t>style(temis): complete 100% emoji-free UI and standard typographic strings across all views</t>
         </is>
       </c>
     </row>
-    <row r="44" ht="20" customHeight="1">
-      <c r="A44" s="41" t="inlineStr">
+    <row r="45" ht="20" customHeight="1">
+      <c r="A45" s="41" t="inlineStr">
         <is>
           <t>35787df4</t>
         </is>
       </c>
-      <c r="B44" s="44" t="inlineStr">
+      <c r="B45" s="44" t="inlineStr">
         <is>
           <t>2026-09-22 18:52:10 -0600</t>
         </is>
       </c>
-      <c r="C44" s="43" t="inlineStr">
+      <c r="C45" s="43" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D44" s="43" t="inlineStr">
+      <c r="D45" s="43" t="inlineStr">
         <is>
           <t>feat(temis): add executive attention banner in hub and 4-step onboarding roadmap in project charter</t>
         </is>
       </c>
-      <c r="E44" s="41" t="inlineStr">
+      <c r="E45" s="41" t="inlineStr">
         <is>
           <t>Frontend / UI</t>
         </is>
       </c>
-      <c r="F44" s="44" t="inlineStr">
+      <c r="F45" s="44" t="inlineStr">
         <is>
           <t>Sprint 07 - Sep 2026</t>
         </is>
       </c>
-      <c r="G44" s="43" t="inlineStr">
+      <c r="G45" s="43" t="inlineStr">
         <is>
           <t>feat(temis): add executive attention banner in hub and 4-step onboarding roadmap in project charter</t>
         </is>
       </c>
     </row>
-    <row r="45" ht="20" customHeight="1">
-      <c r="A45" s="37" t="inlineStr">
+    <row r="46" ht="20" customHeight="1">
+      <c r="A46" s="37" t="inlineStr">
         <is>
           <t>119cb5a5</t>
         </is>
       </c>
-      <c r="B45" s="40" t="inlineStr">
+      <c r="B46" s="40" t="inlineStr">
         <is>
           <t>2026-09-22 18:46:47 -0600</t>
         </is>
       </c>
-      <c r="C45" s="39" t="inlineStr">
+      <c r="C46" s="39" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D45" s="39" t="inlineStr">
+      <c r="D46" s="39" t="inlineStr">
         <is>
           <t>feat(temis): implement enterprise visual design system, 3-step project wizard, workspace lateral sidebar, and remove all emojis in favor of Lucide vector icons</t>
         </is>
       </c>
-      <c r="E45" s="37" t="inlineStr">
+      <c r="E46" s="37" t="inlineStr">
         <is>
           <t>Frontend / UI</t>
         </is>
       </c>
-      <c r="F45" s="40" t="inlineStr">
+      <c r="F46" s="40" t="inlineStr">
         <is>
           <t>Sprint 07 - Sep 2026</t>
         </is>
       </c>
-      <c r="G45" s="39" t="inlineStr">
+      <c r="G46" s="39" t="inlineStr">
         <is>
           <t>feat(temis): implement enterprise visual design system, 3-step project wizard, workspace lateral sidebar, and remove all emojis in favor of Lucide vector icons</t>
         </is>
       </c>
     </row>
-    <row r="46" ht="20" customHeight="1">
-      <c r="A46" s="41" t="inlineStr">
+    <row r="47" ht="20" customHeight="1">
+      <c r="A47" s="41" t="inlineStr">
         <is>
           <t>14d7dac8</t>
         </is>
       </c>
-      <c r="B46" s="44" t="inlineStr">
+      <c r="B47" s="44" t="inlineStr">
         <is>
           <t>2026-09-22 18:31:41 -0600</t>
         </is>
       </c>
-      <c r="C46" s="43" t="inlineStr">
+      <c r="C47" s="43" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D46" s="43" t="inlineStr">
+      <c r="D47" s="43" t="inlineStr">
         <is>
           <t>feat(temis): complete T15 and T16 audit tickets (onboarding tab routing, save states, and operational governance gates)</t>
         </is>
       </c>
-      <c r="E46" s="41" t="inlineStr">
+      <c r="E47" s="41" t="inlineStr">
         <is>
           <t>Frontend / UI</t>
         </is>
       </c>
-      <c r="F46" s="44" t="inlineStr">
+      <c r="F47" s="44" t="inlineStr">
         <is>
           <t>Sprint 07 - Sep 2026</t>
         </is>
       </c>
-      <c r="G46" s="43" t="inlineStr">
+      <c r="G47" s="43" t="inlineStr">
         <is>
           <t>feat(temis): complete T15 and T16 audit tickets (onboarding tab routing, save states, and operational governance gates)</t>
         </is>
       </c>
     </row>
-    <row r="47" ht="20" customHeight="1">
-      <c r="A47" s="37" t="inlineStr">
+    <row r="48" ht="20" customHeight="1">
+      <c r="A48" s="37" t="inlineStr">
         <is>
           <t>35b6a849</t>
         </is>
       </c>
-      <c r="B47" s="40" t="inlineStr">
+      <c r="B48" s="40" t="inlineStr">
         <is>
           <t>2026-09-22 18:26:30 -0600</t>
         </is>
       </c>
-      <c r="C47" s="39" t="inlineStr">
+      <c r="C48" s="39" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D47" s="39" t="inlineStr">
+      <c r="D48" s="39" t="inlineStr">
         <is>
           <t>fix(temis): resolve QA audit findings T01-T14 (security, data isolation, dates, idempotency, UX improvements)</t>
         </is>
       </c>
-      <c r="E47" s="37" t="inlineStr">
+      <c r="E48" s="37" t="inlineStr">
         <is>
           <t>Frontend / UI</t>
         </is>
       </c>
-      <c r="F47" s="40" t="inlineStr">
+      <c r="F48" s="40" t="inlineStr">
         <is>
           <t>Sprint 07 - Sep 2026</t>
         </is>
       </c>
-      <c r="G47" s="39" t="inlineStr">
+      <c r="G48" s="39" t="inlineStr">
         <is>
           <t>fix(temis): resolve QA audit findings T01-T14 (security, data isolation, dates, idempotency, UX improvements)</t>
         </is>
       </c>
     </row>
-    <row r="48" ht="20" customHeight="1">
-      <c r="A48" s="41" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="41" t="inlineStr">
         <is>
           <t>19f3e4e6</t>
         </is>
       </c>
-      <c r="B48" s="44" t="inlineStr">
+      <c r="B49" s="44" t="inlineStr">
         <is>
           <t>2026-09-22 13:38:38 -0600</t>
         </is>
       </c>
-      <c r="C48" s="43" t="inlineStr">
+      <c r="C49" s="43" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D48" s="43" t="inlineStr">
+      <c r="D49" s="43" t="inlineStr">
         <is>
           <t>feat(backend): robustecer schemas con aliases, unificar reply_text en CSAT y homologar cierre de AgenteComunicador</t>
         </is>
       </c>
-      <c r="E48" s="41" t="inlineStr">
+      <c r="E49" s="41" t="inlineStr">
         <is>
           <t>Frontend / UI</t>
         </is>
       </c>
-      <c r="F48" s="44" t="inlineStr">
+      <c r="F49" s="44" t="inlineStr">
         <is>
           <t>Sprint 07 - Sep 2026</t>
         </is>
       </c>
-      <c r="G48" s="43" t="inlineStr">
+      <c r="G49" s="43" t="inlineStr">
         <is>
           <t>feat(backend): robustecer schemas con aliases, unificar reply_text en CSAT y homologar cierre de AgenteComunicador</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="37" t="inlineStr">
+    <row r="50">
+      <c r="A50" s="37" t="inlineStr">
         <is>
           <t>8b2a6e55</t>
         </is>
       </c>
-      <c r="B49" s="40" t="inlineStr">
+      <c r="B50" s="40" t="inlineStr">
         <is>
           <t>2026-09-22 13:26:06 -0600</t>
         </is>
       </c>
-      <c r="C49" s="39" t="inlineStr">
+      <c r="C50" s="39" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D49" s="39" t="inlineStr">
+      <c r="D50" s="39" t="inlineStr">
         <is>
           <t>docs(cascada): homologar prompts de los 15 agentes, estandarizar payloads HTTP y orden de cierre</t>
         </is>
       </c>
-      <c r="E49" s="37" t="inlineStr">
+      <c r="E50" s="37" t="inlineStr">
         <is>
           <t>Frontend / UI</t>
         </is>
       </c>
-      <c r="F49" s="40" t="inlineStr">
+      <c r="F50" s="40" t="inlineStr">
         <is>
           <t>Sprint 07 - Sep 2026</t>
         </is>
       </c>
-      <c r="G49" s="39" t="inlineStr">
+      <c r="G50" s="39" t="inlineStr">
         <is>
           <t>docs(cascada): homologar prompts de los 15 agentes, estandarizar payloads HTTP y orden de cierre</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="41" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="41" t="inlineStr">
         <is>
           <t>23ba5a70</t>
         </is>
       </c>
-      <c r="B50" s="44" t="inlineStr">
+      <c r="B51" s="44" t="inlineStr">
         <is>
           <t>2026-09-22 13:13:46 -0600</t>
         </is>
       </c>
-      <c r="C50" s="43" t="inlineStr">
+      <c r="C51" s="43" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D50" s="43" t="inlineStr">
+      <c r="D51" s="43" t="inlineStr">
         <is>
           <t>fix(bsa-fraudes): implementar persistencia de estado post-cierre y emision de SC.037</t>
         </is>
       </c>
-      <c r="E50" s="41" t="inlineStr">
+      <c r="E51" s="41" t="inlineStr">
         <is>
           <t>Frontend / UI</t>
         </is>
       </c>
-      <c r="F50" s="44" t="inlineStr">
+      <c r="F51" s="44" t="inlineStr">
         <is>
           <t>Sprint 07 - Sep 2026</t>
         </is>
       </c>
-      <c r="G50" s="43" t="inlineStr">
+      <c r="G51" s="43" t="inlineStr">
         <is>
           <t>fix(bsa-fraudes): implementar persistencia de estado post-cierre y emision de SC.037</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="37" t="inlineStr">
+    <row r="52">
+      <c r="A52" s="37" t="inlineStr">
         <is>
           <t>8a76d8ef</t>
         </is>
       </c>
-      <c r="B51" s="40" t="inlineStr">
+      <c r="B52" s="40" t="inlineStr">
         <is>
           <t>2026-09-22 12:44:54 -0600</t>
         </is>
       </c>
-      <c r="C51" s="39" t="inlineStr">
+      <c r="C52" s="39" t="inlineStr">
         <is>
           <t>Jose Antonio Hurtado Palestina</t>
         </is>
       </c>
-      <c r="D51" s="39" t="inlineStr">
+      <c r="D52" s="39" t="inlineStr">
         <is>
           <t>fix(db): ignore deleted postgres host and fallback safely to SQLite for Google Drive persistence</t>
         </is>
       </c>
-      <c r="E51" s="37" t="inlineStr">
+      <c r="E52" s="37" t="inlineStr">
         <is>
           <t>Google Drive / Persistencia</t>
         </is>
       </c>
-      <c r="F51" s="40" t="inlineStr">
+      <c r="F52" s="40" t="inlineStr">
         <is>
           <t>Sprint 07 - Sep 2026</t>
         </is>
       </c>
-      <c r="G51" s="39" t="inlineStr">
+      <c r="G52" s="39" t="inlineStr">
         <is>
           <t>Respaldo automático en Google Workspace Shared Drive con Service Account institucional.</t>
         </is>

</xml_diff>